<commit_message>
Updated the sensor box deployment tracker excel file with more column names
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62C8F422-65E6-C44D-98E1-E36B19132724}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0C4792-C4AE-D54B-9119-044A3B7FAB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6920" yWindow="1840" windowWidth="27640" windowHeight="16940" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="118">
   <si>
     <t>Box Number</t>
   </si>
@@ -384,6 +384,12 @@
   </si>
   <si>
     <t>e00fce6859cf08424ab70193</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deployment code version </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Location </t>
   </si>
 </sst>
 </file>
@@ -772,16 +778,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:H56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.33203125" customWidth="1"/>
     <col min="3" max="3" width="19.5" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="6" max="6" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -797,8 +804,17 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="F1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>60</v>
       </c>
@@ -815,7 +831,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>61</v>
       </c>
@@ -832,7 +848,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>62</v>
       </c>
@@ -849,7 +865,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>63</v>
       </c>
@@ -866,7 +882,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
@@ -883,7 +899,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>65</v>
       </c>
@@ -900,7 +916,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>66</v>
       </c>
@@ -917,7 +933,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>67</v>
       </c>
@@ -934,7 +950,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -951,7 +967,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
@@ -968,7 +984,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
@@ -985,7 +1001,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
@@ -1002,7 +1018,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
@@ -1019,7 +1035,7 @@
         <v>45826</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
@@ -1036,7 +1052,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>74</v>
       </c>

</xml_diff>

<commit_message>
Added some more columns to the deployment inventory excel file
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF0C4792-C4AE-D54B-9119-044A3B7FAB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBBD470E-7169-714F-9E42-1970886B5407}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="34560" windowHeight="21600" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20460" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
+    <sheet name="BOX Health Checklist" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="120">
   <si>
     <t>Box Number</t>
   </si>
@@ -390,6 +391,12 @@
   </si>
   <si>
     <t xml:space="preserve">Location </t>
+  </si>
+  <si>
+    <t>Coordinates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: </t>
   </si>
 </sst>
 </file>
@@ -778,7 +785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -788,7 +795,7 @@
     <col min="6" max="6" width="22.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -813,8 +820,11 @@
       <c r="H1" s="1" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I1" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>60</v>
       </c>
@@ -831,7 +841,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>61</v>
       </c>
@@ -847,8 +857,11 @@
       <c r="E3" s="2">
         <v>45793</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="N3" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>62</v>
       </c>
@@ -865,7 +878,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>63</v>
       </c>
@@ -882,7 +895,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>64</v>
       </c>
@@ -899,7 +912,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>65</v>
       </c>
@@ -916,7 +929,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>66</v>
       </c>
@@ -933,7 +946,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>67</v>
       </c>
@@ -950,7 +963,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>68</v>
       </c>
@@ -967,7 +980,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>69</v>
       </c>
@@ -984,7 +997,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>70</v>
       </c>
@@ -1001,7 +1014,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>71</v>
       </c>
@@ -1018,7 +1031,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
@@ -1035,7 +1048,7 @@
         <v>45826</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>73</v>
       </c>
@@ -1052,7 +1065,7 @@
         <v>45793</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>74</v>
       </c>
@@ -1753,4 +1766,13 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CBFCE6-FDA2-9B4E-A8C1-1998B7362B23}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated file names as test deployment pictures and deployment tracker file
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1693A5E-53C5-4046-BD6A-9D98F194BD4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A4E6F5-C1B9-BB41-98AC-7445C9747C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="140" yWindow="920" windowWidth="34260" windowHeight="20220" activeTab="1" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -628,7 +628,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -654,6 +654,12 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -695,7 +701,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -705,6 +711,7 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3810,6 +3817,18 @@
       <c r="D1" s="2">
         <v>45754</v>
       </c>
+      <c r="E1" s="2">
+        <v>45784</v>
+      </c>
+      <c r="F1" s="2">
+        <v>45815</v>
+      </c>
+      <c r="G1" s="2">
+        <v>45845</v>
+      </c>
+      <c r="H1" s="2">
+        <v>45876</v>
+      </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
@@ -3818,6 +3837,10 @@
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -3826,6 +3849,10 @@
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
       <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
@@ -3834,6 +3861,10 @@
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
       <c r="L4" t="s">
         <v>162</v>
       </c>
@@ -3845,6 +3876,10 @@
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" t="s">
         <v>163</v>
@@ -3857,6 +3892,10 @@
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
       <c r="L6" s="7"/>
       <c r="M6" t="s">
         <v>164</v>
@@ -3869,6 +3908,10 @@
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
@@ -3877,6 +3920,10 @@
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
       <c r="D8" s="8"/>
+      <c r="E8" s="8"/>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
@@ -3885,6 +3932,10 @@
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
       <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
@@ -3893,6 +3944,10 @@
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
       <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
@@ -3901,6 +3956,10 @@
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
       <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
@@ -3909,6 +3968,10 @@
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
       <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
@@ -3917,6 +3980,10 @@
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
       <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
@@ -3925,114 +3992,166 @@
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
       <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>71</v>
       </c>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>75</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="8"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="8"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>77</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="8"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>78</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="8"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>79</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="8"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>80</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="8"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>82</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="8"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>88</v>
       </c>

</xml_diff>

<commit_message>
Updated the deployment track file with box 24s latest deployment
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64A4E6F5-C1B9-BB41-98AC-7445C9747C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F601326F-743C-1145-8F9B-C40C6D1AA872}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="920" windowWidth="34260" windowHeight="20220" activeTab="1" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="140" yWindow="920" windowWidth="34260" windowHeight="20220" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="775" uniqueCount="200">
   <si>
     <t>Box Number</t>
   </si>
@@ -622,13 +622,28 @@
   </si>
   <si>
     <t>Date the arduino was programmed</t>
+  </si>
+  <si>
+    <t>RTC Sync Date</t>
+  </si>
+  <si>
+    <t>The day the RTC was last synced to UTC time</t>
+  </si>
+  <si>
+    <t>07/15/2025</t>
+  </si>
+  <si>
+    <t>Samuel W. Mason Elementary</t>
+  </si>
+  <si>
+    <t>42.3261204,- 71.0706918</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -661,6 +676,12 @@
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -701,7 +722,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -712,6 +733,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1046,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:Z56"/>
+  <dimension ref="A1:AA56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -1055,22 +1077,23 @@
     <col min="4" max="4" width="7.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="11.1640625" customWidth="1"/>
-    <col min="9" max="9" width="26.33203125" customWidth="1"/>
-    <col min="10" max="10" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="25.6640625" customWidth="1"/>
-    <col min="12" max="12" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.5" customWidth="1"/>
-    <col min="17" max="17" width="28" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="22" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="51.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.33203125" customWidth="1"/>
+    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="25.6640625" customWidth="1"/>
+    <col min="13" max="13" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.5" customWidth="1"/>
+    <col min="18" max="18" width="28" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="51.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1096,40 +1119,43 @@
         <v>190</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="K1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="T1" s="1"/>
       <c r="U1" s="1"/>
-      <c r="W1" s="1"/>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>58</v>
       </c>
@@ -1154,40 +1180,41 @@
       <c r="H2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="4"/>
+      <c r="J2" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="4" t="s">
+      <c r="K2" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="K2" t="s">
-        <v>175</v>
-      </c>
-      <c r="L2" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="L2" t="s">
+        <v>175</v>
+      </c>
+      <c r="M2" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N2" t="s">
         <v>171</v>
       </c>
-      <c r="N2" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O2" t="s">
+      <c r="O2" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P2" t="s">
         <v>117</v>
       </c>
-      <c r="P2" s="5">
+      <c r="Q2" s="5">
         <v>0.55347222222222225</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>118</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>119</v>
       </c>
-      <c r="T2" s="2"/>
       <c r="U2" s="2"/>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V2" s="2"/>
+    </row>
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
@@ -1212,40 +1239,41 @@
       <c r="H3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="4"/>
+      <c r="J3" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="K3" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="K3" t="s">
-        <v>175</v>
-      </c>
-      <c r="L3" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="L3" t="s">
+        <v>175</v>
+      </c>
+      <c r="M3" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N3" t="s">
         <v>171</v>
       </c>
-      <c r="N3" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O3" t="s">
+      <c r="O3" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P3" t="s">
         <v>153</v>
       </c>
-      <c r="P3" s="5">
+      <c r="Q3" s="5">
         <v>0.47499999999999998</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>159</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>158</v>
       </c>
-      <c r="T3" s="2"/>
       <c r="U3" s="2"/>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V3" s="2"/>
+    </row>
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>60</v>
       </c>
@@ -1270,46 +1298,47 @@
       <c r="H4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="4"/>
+      <c r="J4" t="s">
         <v>6</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="K4" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="K4" t="s">
-        <v>175</v>
-      </c>
-      <c r="L4" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M4" t="s">
+      <c r="L4" t="s">
+        <v>175</v>
+      </c>
+      <c r="M4" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N4" t="s">
         <v>171</v>
       </c>
-      <c r="N4" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O4" t="s">
+      <c r="O4" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P4" t="s">
         <v>120</v>
       </c>
-      <c r="P4" s="5">
+      <c r="Q4" s="5">
         <v>0.65416666666666667</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>124</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>123</v>
       </c>
-      <c r="T4" s="2"/>
       <c r="U4" s="2"/>
-      <c r="Y4" s="1" t="s">
+      <c r="V4" s="2"/>
+      <c r="Z4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="Z4" t="s">
+      <c r="AA4" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
@@ -1334,46 +1363,47 @@
       <c r="H5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="4"/>
+      <c r="J5" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="K5" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="K5" t="s">
-        <v>175</v>
-      </c>
-      <c r="L5" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M5" t="s">
+      <c r="L5" t="s">
+        <v>175</v>
+      </c>
+      <c r="M5" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N5" t="s">
         <v>171</v>
       </c>
-      <c r="N5" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O5" t="s">
+      <c r="O5" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P5" t="s">
         <v>120</v>
       </c>
-      <c r="P5" s="5">
+      <c r="Q5" s="5">
         <v>0.6166666666666667</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>127</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>128</v>
       </c>
-      <c r="T5" s="2"/>
       <c r="U5" s="2"/>
-      <c r="Y5" s="1" t="s">
+      <c r="V5" s="2"/>
+      <c r="Z5" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="Z5" t="s">
+      <c r="AA5" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
@@ -1398,46 +1428,47 @@
       <c r="H6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="4"/>
+      <c r="J6" t="s">
         <v>8</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="K6" t="s">
-        <v>175</v>
-      </c>
-      <c r="L6" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M6" t="s">
+      <c r="L6" t="s">
+        <v>175</v>
+      </c>
+      <c r="M6" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N6" t="s">
         <v>171</v>
       </c>
-      <c r="N6" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O6" t="s">
+      <c r="O6" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P6" t="s">
         <v>120</v>
       </c>
-      <c r="P6" s="5">
+      <c r="Q6" s="5">
         <v>0.63541666666666663</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="R6" t="s">
         <v>121</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>122</v>
       </c>
-      <c r="T6" s="2"/>
       <c r="U6" s="2"/>
-      <c r="Y6" s="1" t="s">
+      <c r="V6" s="2"/>
+      <c r="Z6" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="Z6" t="s">
+      <c r="AA6" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>63</v>
       </c>
@@ -1462,46 +1493,47 @@
       <c r="H7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="4"/>
+      <c r="J7" t="s">
         <v>9</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="K7" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="K7" t="s">
-        <v>175</v>
-      </c>
-      <c r="L7" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M7" t="s">
+      <c r="L7" t="s">
+        <v>175</v>
+      </c>
+      <c r="M7" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N7" t="s">
         <v>171</v>
       </c>
-      <c r="N7" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O7" t="s">
+      <c r="O7" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P7" t="s">
         <v>120</v>
       </c>
-      <c r="P7" s="5">
+      <c r="Q7" s="5">
         <v>0.67777777777777781</v>
       </c>
-      <c r="Q7" t="s">
+      <c r="R7" t="s">
         <v>125</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>126</v>
       </c>
-      <c r="T7" s="2"/>
       <c r="U7" s="2"/>
-      <c r="Y7" s="1" t="s">
+      <c r="V7" s="2"/>
+      <c r="Z7" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="Z7" t="s">
+      <c r="AA7" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>64</v>
       </c>
@@ -1526,46 +1558,47 @@
       <c r="H8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="4"/>
+      <c r="J8" t="s">
         <v>10</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="K8" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="K8" t="s">
-        <v>175</v>
-      </c>
-      <c r="L8" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M8" t="s">
+      <c r="L8" t="s">
+        <v>175</v>
+      </c>
+      <c r="M8" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N8" t="s">
         <v>171</v>
       </c>
-      <c r="N8" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O8" t="s">
+      <c r="O8" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P8" t="s">
         <v>129</v>
       </c>
-      <c r="P8" s="5">
+      <c r="Q8" s="5">
         <v>0.44166666666666665</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="R8" t="s">
         <v>130</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>131</v>
       </c>
-      <c r="T8" s="2"/>
       <c r="U8" s="2"/>
-      <c r="Y8" s="1" t="s">
+      <c r="V8" s="2"/>
+      <c r="Z8" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="Z8" t="s">
+      <c r="AA8" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>65</v>
       </c>
@@ -1590,46 +1623,47 @@
       <c r="H9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="4"/>
+      <c r="J9" t="s">
         <v>11</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="K9" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="K9" t="s">
-        <v>175</v>
-      </c>
-      <c r="L9" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M9" t="s">
+      <c r="L9" t="s">
+        <v>175</v>
+      </c>
+      <c r="M9" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N9" t="s">
         <v>171</v>
       </c>
-      <c r="N9" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O9" t="s">
+      <c r="O9" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P9" t="s">
         <v>129</v>
       </c>
-      <c r="P9" s="5">
+      <c r="Q9" s="5">
         <v>0.45416666666666666</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="R9" t="s">
         <v>132</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>133</v>
       </c>
-      <c r="T9" s="2"/>
       <c r="U9" s="2"/>
-      <c r="Y9" s="1" t="s">
+      <c r="V9" s="2"/>
+      <c r="Z9" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="Z9" t="s">
+      <c r="AA9" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -1654,46 +1688,47 @@
       <c r="H10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="4"/>
+      <c r="J10" t="s">
         <v>12</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="K10" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="K10" t="s">
-        <v>175</v>
-      </c>
-      <c r="L10" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M10" t="s">
+      <c r="L10" t="s">
+        <v>175</v>
+      </c>
+      <c r="M10" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N10" t="s">
         <v>171</v>
       </c>
-      <c r="N10" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O10" t="s">
+      <c r="O10" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P10" t="s">
         <v>153</v>
       </c>
-      <c r="P10" s="5">
+      <c r="Q10" s="5">
         <v>0.44444444444444442</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="R10" t="s">
         <v>151</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>152</v>
       </c>
-      <c r="T10" s="2"/>
       <c r="U10" s="2"/>
-      <c r="Y10" s="1" t="s">
+      <c r="V10" s="2"/>
+      <c r="Z10" s="1" t="s">
         <v>187</v>
       </c>
-      <c r="Z10" t="s">
+      <c r="AA10" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>67</v>
       </c>
@@ -1718,43 +1753,44 @@
       <c r="H11" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="4"/>
+      <c r="J11" t="s">
         <v>13</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="K11" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="K11" t="s">
-        <v>175</v>
-      </c>
-      <c r="L11" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M11" t="s">
+      <c r="L11" t="s">
+        <v>175</v>
+      </c>
+      <c r="M11" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N11" t="s">
         <v>171</v>
       </c>
-      <c r="N11" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O11" t="s">
+      <c r="O11" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P11" t="s">
         <v>129</v>
       </c>
-      <c r="Q11" t="s">
+      <c r="R11" t="s">
         <v>135</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>136</v>
       </c>
-      <c r="T11" s="2"/>
       <c r="U11" s="2"/>
-      <c r="Y11" s="1" t="s">
+      <c r="V11" s="2"/>
+      <c r="Z11" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="Z11" t="s">
+      <c r="AA11" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>68</v>
       </c>
@@ -1779,46 +1815,47 @@
       <c r="H12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="4"/>
+      <c r="J12" t="s">
         <v>14</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="K12" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="K12" t="s">
-        <v>175</v>
-      </c>
-      <c r="L12" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M12" t="s">
+      <c r="L12" t="s">
+        <v>175</v>
+      </c>
+      <c r="M12" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N12" t="s">
         <v>171</v>
       </c>
-      <c r="N12" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O12" t="s">
+      <c r="O12" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P12" t="s">
         <v>129</v>
       </c>
-      <c r="P12" s="5">
+      <c r="Q12" s="5">
         <v>0.55347222222222225</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="R12" t="s">
         <v>143</v>
       </c>
-      <c r="R12" t="s">
+      <c r="S12" t="s">
         <v>144</v>
       </c>
-      <c r="T12" s="2"/>
       <c r="U12" s="2"/>
-      <c r="Y12" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V12" s="2"/>
+      <c r="Z12" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="AA12" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>69</v>
       </c>
@@ -1843,46 +1880,47 @@
       <c r="H13" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="4"/>
+      <c r="J13" t="s">
         <v>15</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="K13" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="K13" t="s">
-        <v>175</v>
-      </c>
-      <c r="L13" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M13" t="s">
+      <c r="L13" t="s">
+        <v>175</v>
+      </c>
+      <c r="M13" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N13" t="s">
         <v>171</v>
       </c>
-      <c r="N13" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O13" t="s">
+      <c r="O13" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P13" t="s">
         <v>129</v>
       </c>
-      <c r="P13" s="5">
+      <c r="Q13" s="5">
         <v>0.4861111111111111</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="R13" t="s">
         <v>137</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>138</v>
       </c>
-      <c r="T13" s="2"/>
       <c r="U13" s="2"/>
-      <c r="Y13" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V13" s="2"/>
+      <c r="Z13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>70</v>
       </c>
@@ -1907,46 +1945,47 @@
       <c r="H14" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="4"/>
+      <c r="J14" t="s">
         <v>113</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="K14" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="K14" t="s">
-        <v>175</v>
-      </c>
-      <c r="L14" s="2">
+      <c r="L14" t="s">
+        <v>175</v>
+      </c>
+      <c r="M14" s="2">
         <v>45826</v>
       </c>
-      <c r="M14" t="s">
+      <c r="N14" t="s">
         <v>171</v>
       </c>
-      <c r="N14" s="2">
+      <c r="O14" s="2">
         <v>45826</v>
       </c>
-      <c r="O14" t="s">
+      <c r="P14" t="s">
         <v>129</v>
       </c>
-      <c r="P14" s="5">
+      <c r="Q14" s="5">
         <v>0.50347222222222221</v>
       </c>
-      <c r="Q14" t="s">
+      <c r="R14" t="s">
         <v>140</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>139</v>
       </c>
-      <c r="T14" s="2"/>
       <c r="U14" s="2"/>
-      <c r="Y14" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V14" s="2"/>
+      <c r="Z14" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="AA14" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>71</v>
       </c>
@@ -1971,34 +2010,35 @@
       <c r="H15" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="4"/>
+      <c r="J15" t="s">
         <v>16</v>
       </c>
-      <c r="J15" s="4" t="s">
+      <c r="K15" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="K15" t="s">
-        <v>175</v>
-      </c>
-      <c r="L15" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M15" t="s">
+      <c r="L15" t="s">
+        <v>175</v>
+      </c>
+      <c r="M15" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N15" t="s">
         <v>171</v>
       </c>
-      <c r="N15" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T15" s="2"/>
+      <c r="O15" s="2">
+        <v>45793</v>
+      </c>
       <c r="U15" s="2"/>
-      <c r="Y15" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="Z15" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V15" s="2"/>
+      <c r="Z15" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="AA15" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>72</v>
       </c>
@@ -2023,34 +2063,35 @@
       <c r="H16" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="4"/>
+      <c r="J16" t="s">
         <v>17</v>
       </c>
-      <c r="J16" s="4" t="s">
+      <c r="K16" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="K16" t="s">
-        <v>175</v>
-      </c>
-      <c r="L16" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M16" t="s">
+      <c r="L16" t="s">
+        <v>175</v>
+      </c>
+      <c r="M16" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N16" t="s">
         <v>171</v>
       </c>
-      <c r="N16" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T16" s="2"/>
+      <c r="O16" s="2">
+        <v>45793</v>
+      </c>
       <c r="U16" s="2"/>
-      <c r="Y16" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V16" s="2"/>
+      <c r="Z16" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="AA16" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>73</v>
       </c>
@@ -2075,34 +2116,35 @@
       <c r="H17" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="4"/>
+      <c r="J17" t="s">
         <v>18</v>
       </c>
-      <c r="J17" s="4" t="s">
+      <c r="K17" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="K17" t="s">
-        <v>175</v>
-      </c>
-      <c r="L17" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M17" t="s">
+      <c r="L17" t="s">
+        <v>175</v>
+      </c>
+      <c r="M17" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N17" t="s">
         <v>171</v>
       </c>
-      <c r="N17" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T17" s="2"/>
+      <c r="O17" s="2">
+        <v>45793</v>
+      </c>
       <c r="U17" s="2"/>
-      <c r="Y17" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="Z17" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V17" s="2"/>
+      <c r="Z17" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="AA17" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>74</v>
       </c>
@@ -2127,34 +2169,35 @@
       <c r="H18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="4"/>
+      <c r="J18" t="s">
         <v>19</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="K18" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="K18" t="s">
-        <v>175</v>
-      </c>
-      <c r="L18" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M18" t="s">
+      <c r="L18" t="s">
+        <v>175</v>
+      </c>
+      <c r="M18" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N18" t="s">
         <v>171</v>
       </c>
-      <c r="N18" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T18" s="2"/>
+      <c r="O18" s="2">
+        <v>45793</v>
+      </c>
       <c r="U18" s="2"/>
-      <c r="Y18" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="Z18" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V18" s="2"/>
+      <c r="Z18" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>75</v>
       </c>
@@ -2179,46 +2222,47 @@
       <c r="H19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="4"/>
+      <c r="J19" t="s">
         <v>20</v>
       </c>
-      <c r="J19" s="4" t="s">
+      <c r="K19" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="K19" t="s">
-        <v>175</v>
-      </c>
-      <c r="L19" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M19" t="s">
+      <c r="L19" t="s">
+        <v>175</v>
+      </c>
+      <c r="M19" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N19" t="s">
         <v>171</v>
       </c>
-      <c r="N19" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O19" t="s">
+      <c r="O19" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P19" t="s">
         <v>153</v>
       </c>
-      <c r="P19" s="5">
+      <c r="Q19" s="5">
         <v>0.40625</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="R19" t="s">
         <v>160</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>161</v>
       </c>
-      <c r="T19" s="2"/>
       <c r="U19" s="2"/>
-      <c r="Y19" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V19" s="2"/>
+      <c r="Z19" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="AA19" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -2243,46 +2287,47 @@
       <c r="H20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="4"/>
+      <c r="J20" t="s">
         <v>21</v>
       </c>
-      <c r="J20" s="4" t="s">
+      <c r="K20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="K20" t="s">
-        <v>175</v>
-      </c>
-      <c r="L20" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M20" t="s">
+      <c r="L20" t="s">
+        <v>175</v>
+      </c>
+      <c r="M20" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N20" t="s">
         <v>171</v>
       </c>
-      <c r="N20" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O20" t="s">
+      <c r="O20" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P20" t="s">
         <v>129</v>
       </c>
-      <c r="P20" s="5">
+      <c r="Q20" s="5">
         <v>0.51597222222222228</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="R20" t="s">
         <v>141</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>142</v>
       </c>
-      <c r="T20" s="2"/>
       <c r="U20" s="2"/>
-      <c r="Y20" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="Z20" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V20" s="2"/>
+      <c r="Z20" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>77</v>
       </c>
@@ -2307,46 +2352,47 @@
       <c r="H21" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="4"/>
+      <c r="J21" t="s">
         <v>22</v>
       </c>
-      <c r="J21" s="4" t="s">
+      <c r="K21" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="K21" t="s">
-        <v>175</v>
-      </c>
-      <c r="L21" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M21" t="s">
+      <c r="L21" t="s">
+        <v>175</v>
+      </c>
+      <c r="M21" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N21" t="s">
         <v>171</v>
       </c>
-      <c r="N21" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O21" t="s">
+      <c r="O21" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P21" t="s">
         <v>129</v>
       </c>
-      <c r="P21" s="5">
+      <c r="Q21" s="5">
         <v>0.60972222222222228</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="R21" t="s">
         <v>149</v>
       </c>
-      <c r="R21" t="s">
+      <c r="S21" t="s">
         <v>150</v>
       </c>
-      <c r="T21" s="2"/>
       <c r="U21" s="2"/>
-      <c r="Y21" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="Z21" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V21" s="2"/>
+      <c r="Z21" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>78</v>
       </c>
@@ -2371,28 +2417,35 @@
       <c r="H22" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="4"/>
+      <c r="J22" t="s">
         <v>23</v>
       </c>
-      <c r="J22" s="4" t="s">
+      <c r="K22" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="K22" t="s">
-        <v>175</v>
-      </c>
-      <c r="L22" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M22" t="s">
+      <c r="L22" t="s">
+        <v>175</v>
+      </c>
+      <c r="M22" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N22" t="s">
         <v>171</v>
       </c>
-      <c r="N22" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T22" s="2"/>
+      <c r="O22" s="2">
+        <v>45793</v>
+      </c>
       <c r="U22" s="2"/>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V22" s="2"/>
+      <c r="Z22" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>79</v>
       </c>
@@ -2417,40 +2470,41 @@
       <c r="H23" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="4"/>
+      <c r="J23" t="s">
         <v>24</v>
       </c>
-      <c r="J23" s="4" t="s">
+      <c r="K23" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="K23" t="s">
-        <v>175</v>
-      </c>
-      <c r="L23" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M23" t="s">
+      <c r="L23" t="s">
+        <v>175</v>
+      </c>
+      <c r="M23" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N23" t="s">
         <v>171</v>
       </c>
-      <c r="N23" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O23" t="s">
+      <c r="O23" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P23" t="s">
         <v>153</v>
       </c>
-      <c r="P23" s="5">
+      <c r="Q23" s="5">
         <v>0.45763888888888887</v>
       </c>
-      <c r="Q23" t="s">
+      <c r="R23" t="s">
         <v>156</v>
       </c>
-      <c r="R23" t="s">
+      <c r="S23" t="s">
         <v>157</v>
       </c>
-      <c r="T23" s="2"/>
       <c r="U23" s="2"/>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V23" s="2"/>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>80</v>
       </c>
@@ -2475,40 +2529,41 @@
       <c r="H24" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="4"/>
+      <c r="J24" t="s">
         <v>25</v>
       </c>
-      <c r="J24" s="4" t="s">
+      <c r="K24" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="K24" t="s">
-        <v>175</v>
-      </c>
-      <c r="L24" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M24" t="s">
+      <c r="L24" t="s">
+        <v>175</v>
+      </c>
+      <c r="M24" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N24" t="s">
         <v>171</v>
       </c>
-      <c r="N24" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O24" t="s">
+      <c r="O24" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P24" t="s">
         <v>129</v>
       </c>
-      <c r="P24" s="5">
+      <c r="Q24" s="5">
         <v>0.56458333333333333</v>
       </c>
-      <c r="Q24" t="s">
+      <c r="R24" t="s">
         <v>145</v>
       </c>
-      <c r="R24" t="s">
+      <c r="S24" t="s">
         <v>146</v>
       </c>
-      <c r="T24" s="2"/>
       <c r="U24" s="2"/>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V24" s="2"/>
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>81</v>
       </c>
@@ -2533,28 +2588,41 @@
       <c r="H25" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="4"/>
+      <c r="J25" t="s">
         <v>26</v>
       </c>
-      <c r="J25" s="4" t="s">
+      <c r="K25" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="K25" t="s">
-        <v>175</v>
-      </c>
-      <c r="L25" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M25" t="s">
+      <c r="L25" t="s">
+        <v>175</v>
+      </c>
+      <c r="M25" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N25" t="s">
         <v>171</v>
       </c>
-      <c r="N25" s="2">
-        <v>45793</v>
-      </c>
-      <c r="T25" s="2"/>
+      <c r="O25" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P25" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q25" s="5">
+        <v>0.66736111111111107</v>
+      </c>
+      <c r="R25" t="s">
+        <v>198</v>
+      </c>
+      <c r="S25" t="s">
+        <v>199</v>
+      </c>
       <c r="U25" s="2"/>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V25" s="2"/>
+    </row>
+    <row r="26" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>82</v>
       </c>
@@ -2579,40 +2647,41 @@
       <c r="H26" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="4"/>
+      <c r="J26" t="s">
         <v>27</v>
       </c>
-      <c r="J26" s="4" t="s">
+      <c r="K26" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="K26" t="s">
-        <v>175</v>
-      </c>
-      <c r="L26" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M26" t="s">
+      <c r="L26" t="s">
+        <v>175</v>
+      </c>
+      <c r="M26" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N26" t="s">
         <v>171</v>
       </c>
-      <c r="N26" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O26" t="s">
+      <c r="O26" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P26" t="s">
         <v>129</v>
       </c>
-      <c r="P26" s="5">
+      <c r="Q26" s="5">
         <v>0.58750000000000002</v>
       </c>
-      <c r="Q26" t="s">
+      <c r="R26" t="s">
         <v>148</v>
       </c>
-      <c r="R26" t="s">
+      <c r="S26" t="s">
         <v>147</v>
       </c>
-      <c r="T26" s="2"/>
       <c r="U26" s="2"/>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V26" s="2"/>
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>83</v>
       </c>
@@ -2637,40 +2706,41 @@
       <c r="H27" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="4"/>
+      <c r="J27" t="s">
         <v>28</v>
       </c>
-      <c r="J27" s="4" t="s">
+      <c r="K27" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="K27" t="s">
-        <v>175</v>
-      </c>
-      <c r="L27" s="2">
-        <v>45793</v>
-      </c>
-      <c r="M27" t="s">
+      <c r="L27" t="s">
+        <v>175</v>
+      </c>
+      <c r="M27" s="2">
+        <v>45793</v>
+      </c>
+      <c r="N27" t="s">
         <v>171</v>
       </c>
-      <c r="N27" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O27" t="s">
+      <c r="O27" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P27" t="s">
         <v>153</v>
       </c>
-      <c r="P27" s="5">
+      <c r="Q27" s="5">
         <v>0.42499999999999999</v>
       </c>
-      <c r="Q27" t="s">
+      <c r="R27" t="s">
         <v>154</v>
       </c>
-      <c r="R27" t="s">
+      <c r="S27" t="s">
         <v>155</v>
       </c>
-      <c r="T27" s="2"/>
       <c r="U27" s="2"/>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V27" s="2"/>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>84</v>
       </c>
@@ -2695,23 +2765,24 @@
       <c r="H28" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="I28" t="s">
+      <c r="I28" s="4"/>
+      <c r="J28" t="s">
         <v>29</v>
       </c>
-      <c r="J28" s="4" t="s">
+      <c r="K28" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="K28" t="s">
-        <v>175</v>
-      </c>
-      <c r="L28" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N28" s="2"/>
-      <c r="T28" s="2"/>
+      <c r="L28" t="s">
+        <v>175</v>
+      </c>
+      <c r="M28" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O28" s="2"/>
       <c r="U28" s="2"/>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V28" s="2"/>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>85</v>
       </c>
@@ -2736,23 +2807,24 @@
       <c r="H29" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="I29" t="s">
+      <c r="I29" s="4"/>
+      <c r="J29" t="s">
         <v>30</v>
       </c>
-      <c r="J29" s="4" t="s">
+      <c r="K29" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="K29" t="s">
-        <v>175</v>
-      </c>
-      <c r="L29" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N29" s="2"/>
-      <c r="T29" s="2"/>
+      <c r="L29" t="s">
+        <v>175</v>
+      </c>
+      <c r="M29" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O29" s="2"/>
       <c r="U29" s="2"/>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V29" s="2"/>
+    </row>
+    <row r="30" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>86</v>
       </c>
@@ -2777,23 +2849,24 @@
       <c r="H30" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="4"/>
+      <c r="J30" t="s">
         <v>31</v>
       </c>
-      <c r="J30" s="4" t="s">
+      <c r="K30" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="K30" t="s">
-        <v>175</v>
-      </c>
-      <c r="L30" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N30" s="2"/>
-      <c r="T30" s="2"/>
+      <c r="L30" t="s">
+        <v>175</v>
+      </c>
+      <c r="M30" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O30" s="2"/>
       <c r="U30" s="2"/>
-    </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V30" s="2"/>
+    </row>
+    <row r="31" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>87</v>
       </c>
@@ -2818,23 +2891,24 @@
       <c r="H31" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" s="4"/>
+      <c r="J31" t="s">
         <v>32</v>
       </c>
-      <c r="J31" s="4" t="s">
+      <c r="K31" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="K31" t="s">
-        <v>175</v>
-      </c>
-      <c r="L31" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N31" s="2"/>
-      <c r="T31" s="2"/>
+      <c r="L31" t="s">
+        <v>175</v>
+      </c>
+      <c r="M31" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O31" s="2"/>
       <c r="U31" s="2"/>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="V31" s="2"/>
+    </row>
+    <row r="32" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>88</v>
       </c>
@@ -2859,23 +2933,24 @@
       <c r="H32" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" s="4"/>
+      <c r="J32" t="s">
         <v>33</v>
       </c>
-      <c r="J32" s="4" t="s">
+      <c r="K32" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="K32" t="s">
-        <v>175</v>
-      </c>
-      <c r="L32" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N32" s="2"/>
-      <c r="T32" s="2"/>
+      <c r="L32" t="s">
+        <v>175</v>
+      </c>
+      <c r="M32" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O32" s="2"/>
       <c r="U32" s="2"/>
-    </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V32" s="2"/>
+    </row>
+    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>89</v>
       </c>
@@ -2900,23 +2975,24 @@
       <c r="H33" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="4"/>
+      <c r="J33" t="s">
         <v>34</v>
       </c>
-      <c r="J33" s="4" t="s">
+      <c r="K33" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="K33" t="s">
-        <v>175</v>
-      </c>
-      <c r="L33" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N33" s="2"/>
-      <c r="T33" s="2"/>
+      <c r="L33" t="s">
+        <v>175</v>
+      </c>
+      <c r="M33" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O33" s="2"/>
       <c r="U33" s="2"/>
-    </row>
-    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V33" s="2"/>
+    </row>
+    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>90</v>
       </c>
@@ -2941,23 +3017,24 @@
       <c r="H34" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I34" s="4"/>
+      <c r="J34" t="s">
         <v>35</v>
       </c>
-      <c r="J34" s="4" t="s">
+      <c r="K34" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="K34" t="s">
-        <v>175</v>
-      </c>
-      <c r="L34" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N34" s="2"/>
-      <c r="T34" s="2"/>
+      <c r="L34" t="s">
+        <v>175</v>
+      </c>
+      <c r="M34" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O34" s="2"/>
       <c r="U34" s="2"/>
-    </row>
-    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V34" s="2"/>
+    </row>
+    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>91</v>
       </c>
@@ -2982,23 +3059,24 @@
       <c r="H35" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" s="4"/>
+      <c r="J35" t="s">
         <v>36</v>
       </c>
-      <c r="J35" s="4" t="s">
+      <c r="K35" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="K35" t="s">
-        <v>175</v>
-      </c>
-      <c r="L35" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N35" s="2"/>
-      <c r="T35" s="2"/>
+      <c r="L35" t="s">
+        <v>175</v>
+      </c>
+      <c r="M35" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O35" s="2"/>
       <c r="U35" s="2"/>
-    </row>
-    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V35" s="2"/>
+    </row>
+    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>92</v>
       </c>
@@ -3023,23 +3101,24 @@
       <c r="H36" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" s="4"/>
+      <c r="J36" t="s">
         <v>37</v>
       </c>
-      <c r="J36" s="4" t="s">
+      <c r="K36" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="K36" t="s">
-        <v>175</v>
-      </c>
-      <c r="L36" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N36" s="2"/>
-      <c r="T36" s="2"/>
+      <c r="L36" t="s">
+        <v>175</v>
+      </c>
+      <c r="M36" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O36" s="2"/>
       <c r="U36" s="2"/>
-    </row>
-    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V36" s="2"/>
+    </row>
+    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>93</v>
       </c>
@@ -3064,23 +3143,24 @@
       <c r="H37" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" s="4"/>
+      <c r="J37" t="s">
         <v>38</v>
       </c>
-      <c r="J37" s="4" t="s">
+      <c r="K37" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="K37" t="s">
-        <v>175</v>
-      </c>
-      <c r="L37" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N37" s="2"/>
-      <c r="T37" s="2"/>
+      <c r="L37" t="s">
+        <v>175</v>
+      </c>
+      <c r="M37" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O37" s="2"/>
       <c r="U37" s="2"/>
-    </row>
-    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V37" s="2"/>
+    </row>
+    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>94</v>
       </c>
@@ -3105,23 +3185,24 @@
       <c r="H38" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="I38" t="s">
+      <c r="I38" s="4"/>
+      <c r="J38" t="s">
         <v>39</v>
       </c>
-      <c r="J38" s="4" t="s">
+      <c r="K38" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="K38" t="s">
-        <v>175</v>
-      </c>
-      <c r="L38" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N38" s="2"/>
-      <c r="T38" s="2"/>
+      <c r="L38" t="s">
+        <v>175</v>
+      </c>
+      <c r="M38" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O38" s="2"/>
       <c r="U38" s="2"/>
-    </row>
-    <row r="39" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V38" s="2"/>
+    </row>
+    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>95</v>
       </c>
@@ -3146,23 +3227,24 @@
       <c r="H39" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="I39" t="s">
+      <c r="I39" s="4"/>
+      <c r="J39" t="s">
         <v>40</v>
       </c>
-      <c r="J39" s="4" t="s">
+      <c r="K39" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="K39" t="s">
-        <v>175</v>
-      </c>
-      <c r="L39" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N39" s="2"/>
-      <c r="T39" s="2"/>
+      <c r="L39" t="s">
+        <v>175</v>
+      </c>
+      <c r="M39" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O39" s="2"/>
       <c r="U39" s="2"/>
-    </row>
-    <row r="40" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V39" s="2"/>
+    </row>
+    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>96</v>
       </c>
@@ -3187,23 +3269,24 @@
       <c r="H40" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="I40" t="s">
+      <c r="I40" s="4"/>
+      <c r="J40" t="s">
         <v>41</v>
       </c>
-      <c r="J40" s="4" t="s">
+      <c r="K40" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="K40" t="s">
-        <v>175</v>
-      </c>
-      <c r="L40" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N40" s="2"/>
-      <c r="T40" s="2"/>
+      <c r="L40" t="s">
+        <v>175</v>
+      </c>
+      <c r="M40" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O40" s="2"/>
       <c r="U40" s="2"/>
-    </row>
-    <row r="41" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V40" s="2"/>
+    </row>
+    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>97</v>
       </c>
@@ -3228,23 +3311,24 @@
       <c r="H41" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="I41" t="s">
+      <c r="I41" s="4"/>
+      <c r="J41" t="s">
         <v>42</v>
       </c>
-      <c r="J41" s="4" t="s">
+      <c r="K41" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="K41" t="s">
-        <v>175</v>
-      </c>
-      <c r="L41" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N41" s="2"/>
-      <c r="T41" s="2"/>
+      <c r="L41" t="s">
+        <v>175</v>
+      </c>
+      <c r="M41" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O41" s="2"/>
       <c r="U41" s="2"/>
-    </row>
-    <row r="42" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V41" s="2"/>
+    </row>
+    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>98</v>
       </c>
@@ -3269,23 +3353,24 @@
       <c r="H42" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="I42" t="s">
+      <c r="I42" s="4"/>
+      <c r="J42" t="s">
         <v>43</v>
       </c>
-      <c r="J42" s="4" t="s">
+      <c r="K42" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K42" t="s">
-        <v>175</v>
-      </c>
-      <c r="L42" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N42" s="2"/>
-      <c r="T42" s="2"/>
+      <c r="L42" t="s">
+        <v>175</v>
+      </c>
+      <c r="M42" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O42" s="2"/>
       <c r="U42" s="2"/>
-    </row>
-    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V42" s="2"/>
+    </row>
+    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>99</v>
       </c>
@@ -3310,23 +3395,24 @@
       <c r="H43" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="I43" t="s">
+      <c r="I43" s="4"/>
+      <c r="J43" t="s">
         <v>44</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="K43" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="K43" t="s">
-        <v>175</v>
-      </c>
-      <c r="L43" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N43" s="2"/>
-      <c r="T43" s="2"/>
+      <c r="L43" t="s">
+        <v>175</v>
+      </c>
+      <c r="M43" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O43" s="2"/>
       <c r="U43" s="2"/>
-    </row>
-    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V43" s="2"/>
+    </row>
+    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>100</v>
       </c>
@@ -3351,23 +3437,24 @@
       <c r="H44" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I44" t="s">
+      <c r="I44" s="4"/>
+      <c r="J44" t="s">
         <v>45</v>
       </c>
-      <c r="J44" s="4" t="s">
+      <c r="K44" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="K44" t="s">
-        <v>175</v>
-      </c>
-      <c r="L44" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N44" s="2"/>
-      <c r="T44" s="2"/>
+      <c r="L44" t="s">
+        <v>175</v>
+      </c>
+      <c r="M44" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O44" s="2"/>
       <c r="U44" s="2"/>
-    </row>
-    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V44" s="2"/>
+    </row>
+    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>101</v>
       </c>
@@ -3392,23 +3479,24 @@
       <c r="H45" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="I45" t="s">
+      <c r="I45" s="4"/>
+      <c r="J45" t="s">
         <v>46</v>
       </c>
-      <c r="J45" s="4" t="s">
+      <c r="K45" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="K45" t="s">
-        <v>175</v>
-      </c>
-      <c r="L45" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N45" s="2"/>
-      <c r="T45" s="2"/>
+      <c r="L45" t="s">
+        <v>175</v>
+      </c>
+      <c r="M45" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O45" s="2"/>
       <c r="U45" s="2"/>
-    </row>
-    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V45" s="2"/>
+    </row>
+    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>102</v>
       </c>
@@ -3433,23 +3521,24 @@
       <c r="H46" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="I46" t="s">
+      <c r="I46" s="4"/>
+      <c r="J46" t="s">
         <v>47</v>
       </c>
-      <c r="J46" s="4" t="s">
+      <c r="K46" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="K46" t="s">
-        <v>175</v>
-      </c>
-      <c r="L46" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N46" s="2"/>
-      <c r="T46" s="2"/>
+      <c r="L46" t="s">
+        <v>175</v>
+      </c>
+      <c r="M46" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O46" s="2"/>
       <c r="U46" s="2"/>
-    </row>
-    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V46" s="2"/>
+    </row>
+    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>103</v>
       </c>
@@ -3474,23 +3563,24 @@
       <c r="H47" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I47" s="4"/>
+      <c r="J47" t="s">
         <v>48</v>
       </c>
-      <c r="J47" s="4" t="s">
+      <c r="K47" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="K47" t="s">
-        <v>175</v>
-      </c>
-      <c r="L47" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N47" s="2"/>
-      <c r="T47" s="2"/>
+      <c r="L47" t="s">
+        <v>175</v>
+      </c>
+      <c r="M47" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O47" s="2"/>
       <c r="U47" s="2"/>
-    </row>
-    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V47" s="2"/>
+    </row>
+    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>104</v>
       </c>
@@ -3515,23 +3605,24 @@
       <c r="H48" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="I48" t="s">
+      <c r="I48" s="4"/>
+      <c r="J48" t="s">
         <v>49</v>
       </c>
-      <c r="J48" s="4" t="s">
+      <c r="K48" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="K48" t="s">
-        <v>175</v>
-      </c>
-      <c r="L48" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N48" s="2"/>
-      <c r="T48" s="2"/>
+      <c r="L48" t="s">
+        <v>175</v>
+      </c>
+      <c r="M48" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O48" s="2"/>
       <c r="U48" s="2"/>
-    </row>
-    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V48" s="2"/>
+    </row>
+    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>105</v>
       </c>
@@ -3556,23 +3647,24 @@
       <c r="H49" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="I49" t="s">
+      <c r="I49" s="4"/>
+      <c r="J49" t="s">
         <v>50</v>
       </c>
-      <c r="J49" s="4" t="s">
+      <c r="K49" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="K49" t="s">
-        <v>175</v>
-      </c>
-      <c r="L49" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N49" s="2"/>
-      <c r="T49" s="2"/>
+      <c r="L49" t="s">
+        <v>175</v>
+      </c>
+      <c r="M49" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O49" s="2"/>
       <c r="U49" s="2"/>
-    </row>
-    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V49" s="2"/>
+    </row>
+    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>106</v>
       </c>
@@ -3597,23 +3689,24 @@
       <c r="H50" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="I50" t="s">
+      <c r="I50" s="4"/>
+      <c r="J50" t="s">
         <v>51</v>
       </c>
-      <c r="J50" s="4" t="s">
+      <c r="K50" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="K50" t="s">
-        <v>175</v>
-      </c>
-      <c r="L50" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N50" s="2"/>
-      <c r="T50" s="2"/>
+      <c r="L50" t="s">
+        <v>175</v>
+      </c>
+      <c r="M50" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O50" s="2"/>
       <c r="U50" s="2"/>
-    </row>
-    <row r="51" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V50" s="2"/>
+    </row>
+    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>107</v>
       </c>
@@ -3638,23 +3731,24 @@
       <c r="H51" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="I51" t="s">
+      <c r="I51" s="4"/>
+      <c r="J51" t="s">
         <v>52</v>
       </c>
-      <c r="J51" s="4" t="s">
+      <c r="K51" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="K51" t="s">
-        <v>175</v>
-      </c>
-      <c r="L51" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N51" s="2"/>
-      <c r="T51" s="2"/>
+      <c r="L51" t="s">
+        <v>175</v>
+      </c>
+      <c r="M51" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O51" s="2"/>
       <c r="U51" s="2"/>
-    </row>
-    <row r="52" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V51" s="2"/>
+    </row>
+    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>108</v>
       </c>
@@ -3665,23 +3759,24 @@
       <c r="F52" s="4"/>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
-      <c r="I52" t="s">
+      <c r="I52" s="4"/>
+      <c r="J52" t="s">
         <v>53</v>
       </c>
-      <c r="J52" s="4" t="s">
+      <c r="K52" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="K52" t="s">
-        <v>175</v>
-      </c>
-      <c r="L52" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N52" s="2"/>
-      <c r="T52" s="2"/>
+      <c r="L52" t="s">
+        <v>175</v>
+      </c>
+      <c r="M52" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O52" s="2"/>
       <c r="U52" s="2"/>
-    </row>
-    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V52" s="2"/>
+    </row>
+    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>109</v>
       </c>
@@ -3692,23 +3787,24 @@
       <c r="F53" s="4"/>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
-      <c r="I53" t="s">
+      <c r="I53" s="4"/>
+      <c r="J53" t="s">
         <v>54</v>
       </c>
-      <c r="J53" s="4" t="s">
+      <c r="K53" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="K53" t="s">
-        <v>175</v>
-      </c>
-      <c r="L53" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N53" s="2"/>
-      <c r="T53" s="2"/>
+      <c r="L53" t="s">
+        <v>175</v>
+      </c>
+      <c r="M53" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O53" s="2"/>
       <c r="U53" s="2"/>
-    </row>
-    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V53" s="2"/>
+    </row>
+    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>110</v>
       </c>
@@ -3719,23 +3815,24 @@
       <c r="F54" s="4"/>
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
-      <c r="I54" t="s">
+      <c r="I54" s="4"/>
+      <c r="J54" t="s">
         <v>55</v>
       </c>
-      <c r="J54" s="4" t="s">
+      <c r="K54" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="K54" t="s">
-        <v>175</v>
-      </c>
-      <c r="L54" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N54" s="2"/>
-      <c r="T54" s="2"/>
+      <c r="L54" t="s">
+        <v>175</v>
+      </c>
+      <c r="M54" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O54" s="2"/>
       <c r="U54" s="2"/>
-    </row>
-    <row r="55" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V54" s="2"/>
+    </row>
+    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>111</v>
       </c>
@@ -3746,23 +3843,24 @@
       <c r="F55" s="4"/>
       <c r="G55" s="4"/>
       <c r="H55" s="4"/>
-      <c r="I55" t="s">
+      <c r="I55" s="4"/>
+      <c r="J55" t="s">
         <v>56</v>
       </c>
-      <c r="J55" s="4" t="s">
+      <c r="K55" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="K55" t="s">
-        <v>175</v>
-      </c>
-      <c r="L55" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N55" s="2"/>
-      <c r="T55" s="2"/>
+      <c r="L55" t="s">
+        <v>175</v>
+      </c>
+      <c r="M55" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O55" s="2"/>
       <c r="U55" s="2"/>
-    </row>
-    <row r="56" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="V55" s="2"/>
+    </row>
+    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>112</v>
       </c>
@@ -3773,21 +3871,22 @@
       <c r="F56" s="4"/>
       <c r="G56" s="4"/>
       <c r="H56" s="4"/>
-      <c r="I56" t="s">
+      <c r="I56" s="4"/>
+      <c r="J56" t="s">
         <v>57</v>
       </c>
-      <c r="J56" s="4" t="s">
+      <c r="K56" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="K56" t="s">
-        <v>175</v>
-      </c>
-      <c r="L56" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N56" s="2"/>
-      <c r="T56" s="2"/>
+      <c r="L56" t="s">
+        <v>175</v>
+      </c>
+      <c r="M56" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O56" s="2"/>
       <c r="U56" s="2"/>
+      <c r="V56" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -3798,13 +3897,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CBFCE6-FDA2-9B4E-A8C1-1998B7362B23}">
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3829,8 +3928,20 @@
       <c r="H1" s="2">
         <v>45876</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I1" s="10">
+        <v>45907</v>
+      </c>
+      <c r="J1" s="10">
+        <v>45937</v>
+      </c>
+      <c r="K1" s="10">
+        <v>45968</v>
+      </c>
+      <c r="L1" s="10">
+        <v>45998</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>58</v>
       </c>
@@ -3841,8 +3952,12 @@
       <c r="F2" s="6"/>
       <c r="G2" s="6"/>
       <c r="H2" s="6"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>59</v>
       </c>
@@ -3853,8 +3968,12 @@
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
       <c r="H3" s="6"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I3" s="6"/>
+      <c r="J3" s="6"/>
+      <c r="K3" s="6"/>
+      <c r="L3" s="6"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>60</v>
       </c>
@@ -3865,11 +3984,12 @@
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
-      <c r="L4" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+      <c r="L4" s="6"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>61</v>
       </c>
@@ -3880,12 +4000,12 @@
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="K5" s="6"/>
       <c r="L5" s="6"/>
-      <c r="M5" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>62</v>
       </c>
@@ -3896,12 +4016,12 @@
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
-      <c r="L6" s="7"/>
-      <c r="M6" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="K6" s="6"/>
+      <c r="L6" s="6"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>63</v>
       </c>
@@ -3912,8 +4032,12 @@
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
       <c r="H7" s="8"/>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>64</v>
       </c>
@@ -3924,8 +4048,12 @@
       <c r="F8" s="8"/>
       <c r="G8" s="8"/>
       <c r="H8" s="8"/>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>65</v>
       </c>
@@ -3936,8 +4064,12 @@
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -3948,8 +4080,12 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="8"/>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="7"/>
+      <c r="L10" s="7"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>67</v>
       </c>
@@ -3960,8 +4096,12 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="8"/>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>68</v>
       </c>
@@ -3972,8 +4112,12 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="8"/>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>69</v>
       </c>
@@ -3984,8 +4128,12 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="8"/>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>70</v>
       </c>
@@ -3996,8 +4144,12 @@
       <c r="F14" s="8"/>
       <c r="G14" s="8"/>
       <c r="H14" s="8"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>71</v>
       </c>
@@ -4006,7 +4158,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>72</v>
       </c>
@@ -4015,7 +4167,7 @@
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>73</v>
       </c>
@@ -4024,7 +4176,7 @@
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>74</v>
       </c>
@@ -4033,7 +4185,7 @@
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>75</v>
       </c>
@@ -4044,8 +4196,12 @@
       <c r="F19" s="8"/>
       <c r="G19" s="8"/>
       <c r="H19" s="8"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>76</v>
       </c>
@@ -4056,8 +4212,12 @@
       <c r="F20" s="8"/>
       <c r="G20" s="8"/>
       <c r="H20" s="8"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>77</v>
       </c>
@@ -4068,8 +4228,12 @@
       <c r="F21" s="8"/>
       <c r="G21" s="8"/>
       <c r="H21" s="8"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>78</v>
       </c>
@@ -4080,8 +4244,12 @@
       <c r="F22" s="8"/>
       <c r="G22" s="8"/>
       <c r="H22" s="8"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>79</v>
       </c>
@@ -4092,8 +4260,12 @@
       <c r="F23" s="8"/>
       <c r="G23" s="8"/>
       <c r="H23" s="8"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>80</v>
       </c>
@@ -4104,8 +4276,12 @@
       <c r="F24" s="8"/>
       <c r="G24" s="8"/>
       <c r="H24" s="8"/>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>81</v>
       </c>
@@ -4114,7 +4290,7 @@
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>82</v>
       </c>
@@ -4125,113 +4301,128 @@
       <c r="F26" s="6"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="F32" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="F33" s="6"/>
+      <c r="G33" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="F34" s="7"/>
+      <c r="G34" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>104</v>
       </c>

</xml_diff>

<commit_message>
Updated the sensor box deployment tracker sheet
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC9A56CA-1E23-3945-AFDA-25BCB6E546C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FE0411B-775D-0548-A22B-46E517E131A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="8600" yWindow="1020" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="226">
   <si>
     <t>Box Number</t>
   </si>
@@ -712,6 +712,9 @@
   </si>
   <si>
     <t>Changed the RTC battery on 8/01/2025</t>
+  </si>
+  <si>
+    <t>Notes on any component alterations that were made</t>
   </si>
 </sst>
 </file>
@@ -2588,6 +2591,12 @@
       </c>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
+      <c r="Z23" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">

</xml_diff>

<commit_message>
Updated box 9's temperature sensor change on the deployment tracker file and made sure to specified locations of the stickers in the metadata
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EC1B68A-D7C3-5443-93F0-23851AF685C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34C4749-3434-3645-8677-F2DB0E84B086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="802" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="225">
   <si>
     <t>Box Number</t>
   </si>
@@ -579,36 +579,15 @@
     <t>Arduino ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Sticker number on the sound sensor </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sticker number on the T &amp; RH sensor </t>
-  </si>
-  <si>
     <t>T &amp; RH sensor ID</t>
   </si>
   <si>
-    <t>Sticker number on the ADC</t>
-  </si>
-  <si>
-    <t>Sticker number on the SD Module</t>
-  </si>
-  <si>
     <t>PCB ID</t>
   </si>
   <si>
-    <t>Sticker number on PCB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Written number on the  Arduino </t>
-  </si>
-  <si>
     <t>RTC ID</t>
   </si>
   <si>
-    <t>Sticker number on RTC</t>
-  </si>
-  <si>
     <t>Name assigned to each module on the particle website</t>
   </si>
   <si>
@@ -709,6 +688,30 @@
   </si>
   <si>
     <t>Changed the RTC battery on 8/01/2025</t>
+  </si>
+  <si>
+    <t>Changed temperature sensor on 07/22/2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sticker number on the yellow cable infor sticker of the T &amp; RH sensor </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sticker number on the ADC located under the electronics side </t>
+  </si>
+  <si>
+    <t>Sticker number on the sound sensor located behind the electronics side</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sticker number on the SD Module located under the elctronics side </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Written number under the electronics side of  the  Arduino </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sticker number on PCB loacted on the electronics side </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sticker number on RTC located on the electronics side </t>
   </si>
 </sst>
 </file>
@@ -1186,13 +1189,13 @@
         <v>179</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1225,7 +1228,7 @@
         <v>113</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
@@ -1476,7 +1479,7 @@
         <v>175</v>
       </c>
       <c r="AA5" t="s">
-        <v>180</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
@@ -1538,10 +1541,10 @@
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="Z6" s="1" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="AA6" t="s">
-        <v>181</v>
+        <v>218</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.2">
@@ -1606,7 +1609,7 @@
         <v>176</v>
       </c>
       <c r="AA7" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.2">
@@ -1671,7 +1674,7 @@
         <v>177</v>
       </c>
       <c r="AA8" t="s">
-        <v>184</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.2">
@@ -1736,7 +1739,7 @@
         <v>179</v>
       </c>
       <c r="AA9" t="s">
-        <v>187</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.2">
@@ -1747,7 +1750,7 @@
         <v>64</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>64</v>
+        <v>106</v>
       </c>
       <c r="D10" s="4" t="s">
         <v>64</v>
@@ -1795,13 +1798,16 @@
       <c r="S10" t="s">
         <v>150</v>
       </c>
+      <c r="T10" t="s">
+        <v>217</v>
+      </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
       <c r="Z10" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="AA10" t="s">
-        <v>186</v>
+        <v>223</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.2">
@@ -1860,10 +1866,10 @@
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
       <c r="Z11" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="AA11" t="s">
-        <v>189</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.2">
@@ -1925,10 +1931,10 @@
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
       <c r="Z12" s="1" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="AA12" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.2">
@@ -2058,7 +2064,7 @@
         <v>1</v>
       </c>
       <c r="AA14" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
@@ -2106,7 +2112,7 @@
         <v>45793</v>
       </c>
       <c r="T15" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
@@ -2167,7 +2173,7 @@
         <v>171</v>
       </c>
       <c r="AA16" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.2">
@@ -2268,7 +2274,7 @@
         <v>45793</v>
       </c>
       <c r="T18" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
@@ -2276,7 +2282,7 @@
         <v>172</v>
       </c>
       <c r="AA18" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.2">
@@ -2690,16 +2696,16 @@
         <v>45793</v>
       </c>
       <c r="P25" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="Q25" s="5">
         <v>0.66736111111111107</v>
       </c>
       <c r="R25" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="S25" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
@@ -2789,7 +2795,7 @@
         <v>81</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="J27" t="s">
         <v>28</v>
@@ -2850,7 +2856,7 @@
         <v>82</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="J28" t="s">
         <v>55</v>
@@ -2866,7 +2872,7 @@
       </c>
       <c r="O28" s="2"/>
       <c r="T28" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
@@ -2897,7 +2903,7 @@
         <v>83</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="J29" t="s">
         <v>29</v>
@@ -2941,7 +2947,7 @@
         <v>84</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J30" t="s">
         <v>30</v>
@@ -2985,7 +2991,7 @@
         <v>85</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J31" t="s">
         <v>31</v>
@@ -3029,7 +3035,7 @@
         <v>86</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J32" t="s">
         <v>32</v>
@@ -3073,7 +3079,7 @@
         <v>87</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J33" t="s">
         <v>33</v>
@@ -3117,7 +3123,7 @@
         <v>88</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="J34" t="s">
         <v>54</v>
@@ -4020,61 +4026,61 @@
         <v>45998</v>
       </c>
       <c r="M1" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>195</v>
+      </c>
+      <c r="O1" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="P1" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="Q1" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="R1" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="S1" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="T1" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="U1" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="V1" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="W1" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="X1" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="Y1" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="AA1" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="AB1" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="AC1" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>211</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="AE1" s="11" t="s">
         <v>212</v>
-      </c>
-      <c r="Y1" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="Z1" s="11" t="s">
-        <v>214</v>
-      </c>
-      <c r="AA1" s="11" t="s">
-        <v>215</v>
-      </c>
-      <c r="AB1" s="11" t="s">
-        <v>216</v>
-      </c>
-      <c r="AC1" s="11" t="s">
-        <v>217</v>
-      </c>
-      <c r="AD1" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="AE1" s="11" t="s">
-        <v>219</v>
       </c>
       <c r="AF1" s="10">
         <v>45870</v>
@@ -4887,7 +4893,7 @@
         <v>161</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
@@ -4899,7 +4905,7 @@
         <v>162</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Swapped LTE34 with 53 and changed battery for RTC37
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D34C4749-3434-3645-8677-F2DB0E84B086}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A6E956-0856-6A41-A0C2-45A2399E9F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="224">
   <si>
     <t>Box Number</t>
   </si>
@@ -139,9 +139,6 @@
   </si>
   <si>
     <t>e00fce689495e369536fcad7</t>
-  </si>
-  <si>
-    <t>e00fce689901fcf4cd677c9a</t>
   </si>
   <si>
     <t>e00fce687151b0efcb830758</t>
@@ -1174,28 +1171,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>179</v>
-      </c>
       <c r="G1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>182</v>
-      </c>
       <c r="I1" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
@@ -1207,28 +1204,28 @@
         <v>2</v>
       </c>
       <c r="M1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>172</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="R1" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="S1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="T1" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="U1" s="1"/>
       <c r="V1" s="1"/>
@@ -1236,177 +1233,177 @@
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="I2" s="4"/>
       <c r="J2" t="s">
         <v>4</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L2" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M2" s="2">
         <v>45793</v>
       </c>
       <c r="N2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O2" s="2">
         <v>45793</v>
       </c>
       <c r="P2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="Q2" s="5">
         <v>0.55347222222222225</v>
       </c>
       <c r="R2" t="s">
+        <v>115</v>
+      </c>
+      <c r="S2" t="s">
         <v>116</v>
-      </c>
-      <c r="S2" t="s">
-        <v>117</v>
       </c>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I3" s="4"/>
       <c r="J3" t="s">
         <v>5</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L3" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M3" s="2">
         <v>45793</v>
       </c>
       <c r="N3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O3" s="2">
         <v>45793</v>
       </c>
       <c r="P3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q3" s="5">
         <v>0.47499999999999998</v>
       </c>
       <c r="R3" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="S3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="U3" s="2"/>
       <c r="V3" s="2"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I4" s="4"/>
       <c r="J4" t="s">
         <v>6</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M4" s="2">
         <v>45793</v>
       </c>
       <c r="N4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O4" s="2">
         <v>45793</v>
       </c>
       <c r="P4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q4" s="5">
         <v>0.65416666666666667</v>
       </c>
       <c r="R4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="S4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="U4" s="2"/>
       <c r="V4" s="2"/>
@@ -1414,584 +1411,584 @@
         <v>0</v>
       </c>
       <c r="AA4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" t="s">
         <v>7</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L5" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M5" s="2">
         <v>45793</v>
       </c>
       <c r="N5" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O5" s="2">
         <v>45793</v>
       </c>
       <c r="P5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q5" s="5">
         <v>0.6166666666666667</v>
       </c>
       <c r="R5" t="s">
+        <v>124</v>
+      </c>
+      <c r="S5" t="s">
         <v>125</v>
-      </c>
-      <c r="S5" t="s">
-        <v>126</v>
       </c>
       <c r="U5" s="2"/>
       <c r="V5" s="2"/>
       <c r="Z5" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AA5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I6" s="4"/>
       <c r="J6" t="s">
         <v>8</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M6" s="2">
         <v>45793</v>
       </c>
       <c r="N6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O6" s="2">
         <v>45793</v>
       </c>
       <c r="P6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q6" s="5">
         <v>0.63541666666666663</v>
       </c>
       <c r="R6" t="s">
+        <v>118</v>
+      </c>
+      <c r="S6" t="s">
         <v>119</v>
-      </c>
-      <c r="S6" t="s">
-        <v>120</v>
       </c>
       <c r="U6" s="2"/>
       <c r="V6" s="2"/>
       <c r="Z6" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AA6" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" t="s">
         <v>9</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M7" s="2">
         <v>45793</v>
       </c>
       <c r="N7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O7" s="2">
         <v>45793</v>
       </c>
       <c r="P7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q7" s="5">
         <v>0.67777777777777781</v>
       </c>
       <c r="R7" t="s">
+        <v>122</v>
+      </c>
+      <c r="S7" t="s">
         <v>123</v>
-      </c>
-      <c r="S7" t="s">
-        <v>124</v>
       </c>
       <c r="U7" s="2"/>
       <c r="V7" s="2"/>
       <c r="Z7" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AA7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" s="4"/>
       <c r="J8" t="s">
         <v>10</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L8" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M8" s="2">
         <v>45793</v>
       </c>
       <c r="N8" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O8" s="2">
         <v>45793</v>
       </c>
       <c r="P8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q8" s="5">
         <v>0.44166666666666665</v>
       </c>
       <c r="R8" t="s">
+        <v>127</v>
+      </c>
+      <c r="S8" t="s">
         <v>128</v>
-      </c>
-      <c r="S8" t="s">
-        <v>129</v>
       </c>
       <c r="U8" s="2"/>
       <c r="V8" s="2"/>
       <c r="Z8" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AA8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I9" s="4"/>
       <c r="J9" t="s">
         <v>11</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L9" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M9" s="2">
         <v>45793</v>
       </c>
       <c r="N9" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O9" s="2">
         <v>45793</v>
       </c>
       <c r="P9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q9" s="5">
         <v>0.45416666666666666</v>
       </c>
       <c r="R9" t="s">
+        <v>129</v>
+      </c>
+      <c r="S9" t="s">
         <v>130</v>
-      </c>
-      <c r="S9" t="s">
-        <v>131</v>
       </c>
       <c r="U9" s="2"/>
       <c r="V9" s="2"/>
       <c r="Z9" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AA9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I10" s="4"/>
       <c r="J10" t="s">
         <v>12</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L10" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M10" s="2">
         <v>45793</v>
       </c>
       <c r="N10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O10" s="2">
         <v>45793</v>
       </c>
       <c r="P10" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q10" s="5">
         <v>0.44444444444444442</v>
       </c>
       <c r="R10" t="s">
+        <v>148</v>
+      </c>
+      <c r="S10" t="s">
         <v>149</v>
       </c>
-      <c r="S10" t="s">
-        <v>150</v>
-      </c>
       <c r="T10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
       <c r="Z10" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AA10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I11" s="4"/>
       <c r="J11" t="s">
         <v>13</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M11" s="2">
         <v>45793</v>
       </c>
       <c r="N11" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O11" s="2">
         <v>45793</v>
       </c>
       <c r="P11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="R11" t="s">
+        <v>132</v>
+      </c>
+      <c r="S11" t="s">
         <v>133</v>
-      </c>
-      <c r="S11" t="s">
-        <v>134</v>
       </c>
       <c r="U11" s="2"/>
       <c r="V11" s="2"/>
       <c r="Z11" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AA11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I12" s="4"/>
       <c r="J12" t="s">
         <v>14</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M12" s="2">
         <v>45793</v>
       </c>
       <c r="N12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O12" s="2">
         <v>45793</v>
       </c>
       <c r="P12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q12" s="5">
         <v>0.55347222222222225</v>
       </c>
       <c r="R12" t="s">
+        <v>140</v>
+      </c>
+      <c r="S12" t="s">
         <v>141</v>
-      </c>
-      <c r="S12" t="s">
-        <v>142</v>
       </c>
       <c r="U12" s="2"/>
       <c r="V12" s="2"/>
       <c r="Z12" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="AA12" t="s">
         <v>186</v>
-      </c>
-      <c r="AA12" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" t="s">
         <v>15</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M13" s="2">
         <v>45793</v>
       </c>
       <c r="N13" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O13" s="2">
         <v>45793</v>
       </c>
       <c r="P13" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q13" s="5">
         <v>0.4861111111111111</v>
       </c>
       <c r="R13" t="s">
+        <v>134</v>
+      </c>
+      <c r="S13" t="s">
         <v>135</v>
-      </c>
-      <c r="S13" t="s">
-        <v>136</v>
       </c>
       <c r="U13" s="2"/>
       <c r="V13" s="2"/>
@@ -1999,64 +1996,64 @@
         <v>3</v>
       </c>
       <c r="AA13" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I14" s="4"/>
       <c r="J14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M14" s="2">
         <v>45826</v>
       </c>
       <c r="N14" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O14" s="2">
         <v>45826</v>
       </c>
       <c r="P14" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q14" s="5">
         <v>0.50347222222222221</v>
       </c>
       <c r="R14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="S14" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
@@ -2064,55 +2061,55 @@
         <v>1</v>
       </c>
       <c r="AA14" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I15" s="4"/>
       <c r="J15" t="s">
         <v>16</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L15" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M15" s="2">
         <v>45793</v>
       </c>
       <c r="N15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O15" s="2">
         <v>45793</v>
       </c>
       <c r="T15" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
@@ -2120,49 +2117,49 @@
         <v>2</v>
       </c>
       <c r="AA15" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I16" s="4"/>
       <c r="J16" t="s">
         <v>17</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M16" s="2">
         <v>45793</v>
       </c>
       <c r="N16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O16" s="2">
         <v>45793</v>
@@ -2170,52 +2167,52 @@
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="Z16" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AA16" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" t="s">
         <v>18</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M17" s="2">
         <v>45793</v>
       </c>
       <c r="N17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O17" s="2">
         <v>45793</v>
@@ -2223,303 +2220,303 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="Z17" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AA17" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I18" s="4"/>
       <c r="J18" t="s">
         <v>19</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="L18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M18" s="2">
         <v>45793</v>
       </c>
       <c r="N18" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O18" s="2">
         <v>45793</v>
       </c>
       <c r="T18" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="U18" s="2"/>
       <c r="V18" s="2"/>
       <c r="Z18" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AA18" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I19" s="4"/>
       <c r="J19" t="s">
         <v>20</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M19" s="2">
         <v>45793</v>
       </c>
       <c r="N19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O19" s="2">
         <v>45793</v>
       </c>
       <c r="P19" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q19" s="5">
         <v>0.40625</v>
       </c>
       <c r="R19" t="s">
+        <v>157</v>
+      </c>
+      <c r="S19" t="s">
         <v>158</v>
-      </c>
-      <c r="S19" t="s">
-        <v>159</v>
       </c>
       <c r="U19" s="2"/>
       <c r="V19" s="2"/>
       <c r="Z19" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="AA19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I20" s="4"/>
       <c r="J20" t="s">
         <v>21</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L20" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M20" s="2">
         <v>45793</v>
       </c>
       <c r="N20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O20" s="2">
         <v>45793</v>
       </c>
       <c r="P20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q20" s="5">
         <v>0.51597222222222228</v>
       </c>
       <c r="R20" t="s">
+        <v>138</v>
+      </c>
+      <c r="S20" t="s">
         <v>139</v>
-      </c>
-      <c r="S20" t="s">
-        <v>140</v>
       </c>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
       <c r="Z20" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="AA20" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I21" s="4"/>
       <c r="J21" t="s">
         <v>22</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M21" s="2">
         <v>45793</v>
       </c>
       <c r="N21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O21" s="2">
         <v>45793</v>
       </c>
       <c r="P21" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q21" s="5">
         <v>0.60972222222222228</v>
       </c>
       <c r="R21" t="s">
+        <v>146</v>
+      </c>
+      <c r="S21" t="s">
         <v>147</v>
-      </c>
-      <c r="S21" t="s">
-        <v>148</v>
       </c>
       <c r="U21" s="2"/>
       <c r="V21" s="2"/>
       <c r="Z21" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="AA21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I22" s="4"/>
       <c r="J22" t="s">
         <v>23</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L22" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M22" s="2">
         <v>45793</v>
       </c>
       <c r="N22" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O22" s="2">
         <v>45793</v>
@@ -2527,392 +2524,392 @@
       <c r="U22" s="2"/>
       <c r="V22" s="2"/>
       <c r="Z22" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="AA22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="I23" s="4"/>
       <c r="J23" t="s">
         <v>24</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M23" s="2">
         <v>45793</v>
       </c>
       <c r="N23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O23" s="2">
         <v>45793</v>
       </c>
       <c r="P23" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q23" s="5">
         <v>0.45763888888888887</v>
       </c>
       <c r="R23" t="s">
+        <v>153</v>
+      </c>
+      <c r="S23" t="s">
         <v>154</v>
-      </c>
-      <c r="S23" t="s">
-        <v>155</v>
       </c>
       <c r="U23" s="2"/>
       <c r="V23" s="2"/>
     </row>
     <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="I24" s="4"/>
       <c r="J24" t="s">
         <v>25</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M24" s="2">
         <v>45793</v>
       </c>
       <c r="N24" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O24" s="2">
         <v>45793</v>
       </c>
       <c r="P24" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q24" s="5">
         <v>0.56458333333333333</v>
       </c>
       <c r="R24" t="s">
+        <v>142</v>
+      </c>
+      <c r="S24" t="s">
         <v>143</v>
-      </c>
-      <c r="S24" t="s">
-        <v>144</v>
       </c>
       <c r="U24" s="2"/>
       <c r="V24" s="2"/>
     </row>
     <row r="25" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I25" s="4"/>
       <c r="J25" t="s">
         <v>26</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="L25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M25" s="2">
         <v>45793</v>
       </c>
       <c r="N25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O25" s="2">
         <v>45793</v>
       </c>
       <c r="P25" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="Q25" s="5">
         <v>0.66736111111111107</v>
       </c>
       <c r="R25" t="s">
+        <v>188</v>
+      </c>
+      <c r="S25" t="s">
         <v>189</v>
-      </c>
-      <c r="S25" t="s">
-        <v>190</v>
       </c>
       <c r="U25" s="2"/>
       <c r="V25" s="2"/>
     </row>
     <row r="26" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I26" s="4"/>
       <c r="J26" t="s">
         <v>27</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="L26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M26" s="2">
         <v>45793</v>
       </c>
       <c r="N26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O26" s="2">
         <v>45793</v>
       </c>
       <c r="P26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="Q26" s="5">
         <v>0.58750000000000002</v>
       </c>
       <c r="R26" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="S26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="U26" s="2"/>
       <c r="V26" s="2"/>
     </row>
     <row r="27" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J27" t="s">
         <v>28</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="L27" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M27" s="2">
         <v>45793</v>
       </c>
       <c r="N27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="O27" s="2">
         <v>45793</v>
       </c>
       <c r="P27" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="Q27" s="5">
         <v>0.42499999999999999</v>
       </c>
       <c r="R27" t="s">
+        <v>151</v>
+      </c>
+      <c r="S27" t="s">
         <v>152</v>
-      </c>
-      <c r="S27" t="s">
-        <v>153</v>
       </c>
       <c r="U27" s="2"/>
       <c r="V27" s="2"/>
     </row>
     <row r="28" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="L28" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M28" s="2">
         <v>45793</v>
       </c>
       <c r="O28" s="2"/>
       <c r="T28" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
     </row>
     <row r="29" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="J29" t="s">
         <v>29</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="L29" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M29" s="2">
         <v>45793</v>
@@ -2923,40 +2920,40 @@
     </row>
     <row r="30" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J30" t="s">
         <v>30</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="L30" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M30" s="2">
         <v>45793</v>
@@ -2967,40 +2964,40 @@
     </row>
     <row r="31" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J31" t="s">
         <v>31</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L31" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M31" s="2">
         <v>45793</v>
@@ -3011,40 +3008,40 @@
     </row>
     <row r="32" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J32" t="s">
         <v>32</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="L32" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M32" s="2">
         <v>45793</v>
@@ -3055,40 +3052,40 @@
     </row>
     <row r="33" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="H33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J33" t="s">
         <v>33</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="L33" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M33" s="2">
         <v>45793</v>
@@ -3099,40 +3096,40 @@
     </row>
     <row r="34" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J34" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="L34" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M34" s="2">
         <v>45793</v>
@@ -3143,38 +3140,40 @@
     </row>
     <row r="35" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H35" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="I35" s="4"/>
+        <v>88</v>
+      </c>
+      <c r="I35" s="4" t="s">
+        <v>214</v>
+      </c>
       <c r="J35" t="s">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L35" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M35" s="2">
         <v>45793</v>
@@ -3185,38 +3184,40 @@
     </row>
     <row r="36" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H36" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="I36" s="4"/>
+        <v>89</v>
+      </c>
+      <c r="I36" s="4" t="s">
+        <v>214</v>
+      </c>
       <c r="J36" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="L36" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M36" s="2">
         <v>45793</v>
@@ -3227,38 +3228,40 @@
     </row>
     <row r="37" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="I37" s="4"/>
+        <v>90</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>214</v>
+      </c>
       <c r="J37" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M37" s="2">
         <v>45793</v>
@@ -3269,80 +3272,85 @@
     </row>
     <row r="38" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="I38" s="4"/>
+        <v>91</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>214</v>
+      </c>
       <c r="J38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="L38" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M38" s="2">
         <v>45793</v>
       </c>
       <c r="O38" s="2"/>
+      <c r="T38" t="s">
+        <v>215</v>
+      </c>
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
     </row>
     <row r="39" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I39" s="4"/>
       <c r="J39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M39" s="2">
         <v>45793</v>
@@ -3353,38 +3361,38 @@
     </row>
     <row r="40" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I40" s="4"/>
       <c r="J40" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L40" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M40" s="2">
         <v>45793</v>
@@ -3395,38 +3403,38 @@
     </row>
     <row r="41" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I41" s="4"/>
       <c r="J41" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L41" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M41" s="2">
         <v>45793</v>
@@ -3437,38 +3445,38 @@
     </row>
     <row r="42" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L42" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M42" s="2">
         <v>45793</v>
@@ -3479,38 +3487,38 @@
     </row>
     <row r="43" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I43" s="4"/>
       <c r="J43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="L43" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M43" s="2">
         <v>45793</v>
@@ -3521,38 +3529,38 @@
     </row>
     <row r="44" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I44" s="4"/>
       <c r="J44" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="L44" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M44" s="2">
         <v>45793</v>
@@ -3563,38 +3571,38 @@
     </row>
     <row r="45" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I45" s="4"/>
       <c r="J45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L45" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M45" s="2">
         <v>45793</v>
@@ -3605,38 +3613,38 @@
     </row>
     <row r="46" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I46" s="4"/>
       <c r="J46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="L46" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M46" s="2">
         <v>45793</v>
@@ -3647,38 +3655,38 @@
     </row>
     <row r="47" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I47" s="4"/>
       <c r="J47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="L47" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M47" s="2">
         <v>45793</v>
@@ -3689,38 +3697,38 @@
     </row>
     <row r="48" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="I48" s="4"/>
       <c r="J48" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="L48" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M48" s="2">
         <v>45793</v>
@@ -3731,38 +3739,38 @@
     </row>
     <row r="49" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="I49" s="4"/>
       <c r="J49" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="L49" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M49" s="2">
         <v>45793</v>
@@ -3773,38 +3781,38 @@
     </row>
     <row r="50" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="I50" s="4"/>
       <c r="J50" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="L50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M50" s="2">
         <v>45793</v>
@@ -3815,38 +3823,38 @@
     </row>
     <row r="51" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I51" s="4"/>
       <c r="J51" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L51" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M51" s="2">
         <v>45793</v>
@@ -3857,7 +3865,7 @@
     </row>
     <row r="52" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B52" s="4"/>
       <c r="C52" s="4"/>
@@ -3868,13 +3876,13 @@
       <c r="H52" s="4"/>
       <c r="I52" s="4"/>
       <c r="J52" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K52" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L52" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M52" s="2">
         <v>45793</v>
@@ -3885,7 +3893,7 @@
     </row>
     <row r="53" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B53" s="4"/>
       <c r="C53" s="4"/>
@@ -3896,13 +3904,13 @@
       <c r="H53" s="4"/>
       <c r="I53" s="4"/>
       <c r="J53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K53" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="L53" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="M53" s="2">
         <v>45793</v>
@@ -3913,7 +3921,7 @@
     </row>
     <row r="54" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B54" s="4"/>
       <c r="C54" s="4"/>
@@ -3923,25 +3931,14 @@
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4"/>
-      <c r="J54" t="s">
-        <v>53</v>
-      </c>
-      <c r="K54" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="L54" t="s">
-        <v>173</v>
-      </c>
-      <c r="M54" s="2">
-        <v>45793</v>
-      </c>
+      <c r="M54" s="2"/>
       <c r="O54" s="2"/>
       <c r="U54" s="2"/>
       <c r="V54" s="2"/>
     </row>
     <row r="55" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -3958,7 +3955,7 @@
     </row>
     <row r="56" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -4026,61 +4023,61 @@
         <v>45998</v>
       </c>
       <c r="M1" s="11" t="s">
+        <v>193</v>
+      </c>
+      <c r="N1" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="O1" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="P1" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="Q1" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="R1" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="S1" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="T1" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="U1" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="V1" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="W1" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="X1" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="Y1" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="AA1" s="11" t="s">
         <v>207</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="AB1" s="11" t="s">
         <v>208</v>
       </c>
-      <c r="AB1" s="11" t="s">
+      <c r="AC1" s="11" t="s">
         <v>209</v>
       </c>
-      <c r="AC1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="AD1" s="11" t="s">
+      <c r="AE1" s="11" t="s">
         <v>211</v>
-      </c>
-      <c r="AE1" s="11" t="s">
-        <v>212</v>
       </c>
       <c r="AF1" s="10">
         <v>45870</v>
@@ -4088,7 +4085,7 @@
     </row>
     <row r="2" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -4124,7 +4121,7 @@
     </row>
     <row r="3" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B3" s="6"/>
       <c r="C3" s="6"/>
@@ -4160,7 +4157,7 @@
     </row>
     <row r="4" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B4" s="6"/>
       <c r="C4" s="6"/>
@@ -4196,7 +4193,7 @@
     </row>
     <row r="5" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -4232,7 +4229,7 @@
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
@@ -4268,7 +4265,7 @@
     </row>
     <row r="7" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -4304,7 +4301,7 @@
     </row>
     <row r="8" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="6"/>
@@ -4340,7 +4337,7 @@
     </row>
     <row r="9" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="6"/>
@@ -4376,7 +4373,7 @@
     </row>
     <row r="10" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -4412,7 +4409,7 @@
     </row>
     <row r="11" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>
@@ -4448,7 +4445,7 @@
     </row>
     <row r="12" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B12" s="6"/>
       <c r="C12" s="6"/>
@@ -4484,7 +4481,7 @@
     </row>
     <row r="13" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B13" s="6"/>
       <c r="C13" s="6"/>
@@ -4520,7 +4517,7 @@
     </row>
     <row r="14" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4556,7 +4553,7 @@
     </row>
     <row r="15" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E15" s="9"/>
       <c r="F15" s="9"/>
@@ -4565,7 +4562,7 @@
     </row>
     <row r="16" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E16" s="9"/>
       <c r="F16" s="9"/>
@@ -4574,7 +4571,7 @@
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E17" s="9"/>
       <c r="F17" s="9"/>
@@ -4583,7 +4580,7 @@
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
@@ -4592,7 +4589,7 @@
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B19" s="6"/>
       <c r="C19" s="6"/>
@@ -4628,7 +4625,7 @@
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -4664,7 +4661,7 @@
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
@@ -4700,7 +4697,7 @@
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
@@ -4736,7 +4733,7 @@
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -4772,7 +4769,7 @@
     </row>
     <row r="24" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
@@ -4808,7 +4805,7 @@
     </row>
     <row r="25" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E25" s="9"/>
       <c r="F25" s="9"/>
@@ -4817,7 +4814,7 @@
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
@@ -4853,169 +4850,169 @@
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F32" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F34" s="7"/>
       <c r="G34" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated sensor deployment tracker sheet as well as the box health sheet
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8A6E956-0856-6A41-A0C2-45A2399E9F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6037CA19-65B4-9A4B-BBFC-0CEE82B4F6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="900" yWindow="1260" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="805" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="230">
   <si>
     <t>Box Number</t>
   </si>
@@ -678,9 +678,6 @@
     <t>Notes:</t>
   </si>
   <si>
-    <t>BOX 09 was brought back to the lab from te field on Tuesday 07/15/2025 at 15:30 it was taken down. We have put this box on hold until the issue is diagnosed.,</t>
-  </si>
-  <si>
     <t>08/01/2025</t>
   </si>
   <si>
@@ -709,6 +706,27 @@
   </si>
   <si>
     <t xml:space="preserve">Sticker number on RTC located on the electronics side </t>
+  </si>
+  <si>
+    <t>BOX 09 was brought back to the lab from te field on Tuesday 07/15/2025 at 15:30 it was taken down. We have put this box on hold until the issue is diagnosed.</t>
+  </si>
+  <si>
+    <t>Sargent st</t>
+  </si>
+  <si>
+    <t>42.3152962,-71.0738930</t>
+  </si>
+  <si>
+    <t>Moreland st @ learning together day care</t>
+  </si>
+  <si>
+    <t>42.3255823, -71.0817659</t>
+  </si>
+  <si>
+    <t>Warren @ Quincy</t>
+  </si>
+  <si>
+    <t>42.3164061, -71.0826839</t>
   </si>
 </sst>
 </file>
@@ -794,7 +812,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -807,6 +825,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1476,7 +1495,7 @@
         <v>174</v>
       </c>
       <c r="AA5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
@@ -1541,7 +1560,7 @@
         <v>179</v>
       </c>
       <c r="AA6" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.2">
@@ -1606,7 +1625,7 @@
         <v>175</v>
       </c>
       <c r="AA7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.2">
@@ -1671,7 +1690,7 @@
         <v>176</v>
       </c>
       <c r="AA8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.2">
@@ -1736,7 +1755,7 @@
         <v>178</v>
       </c>
       <c r="AA9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.2">
@@ -1796,7 +1815,7 @@
         <v>149</v>
       </c>
       <c r="T10" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="U10" s="2"/>
       <c r="V10" s="2"/>
@@ -1804,7 +1823,7 @@
         <v>180</v>
       </c>
       <c r="AA10" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.2">
@@ -1866,7 +1885,7 @@
         <v>181</v>
       </c>
       <c r="AA11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.2">
@@ -2164,6 +2183,18 @@
       <c r="O16" s="2">
         <v>45793</v>
       </c>
+      <c r="P16" s="2">
+        <v>45785</v>
+      </c>
+      <c r="Q16" s="5">
+        <v>0.48055555555555557</v>
+      </c>
+      <c r="R16" t="s">
+        <v>226</v>
+      </c>
+      <c r="S16" t="s">
+        <v>227</v>
+      </c>
       <c r="U16" s="2"/>
       <c r="V16" s="2"/>
       <c r="Z16" s="1" t="s">
@@ -2217,6 +2248,18 @@
       <c r="O17" s="2">
         <v>45793</v>
       </c>
+      <c r="P17" s="2">
+        <v>45785</v>
+      </c>
+      <c r="Q17" s="5">
+        <v>0.49722222222222223</v>
+      </c>
+      <c r="R17" t="s">
+        <v>228</v>
+      </c>
+      <c r="S17" t="s">
+        <v>229</v>
+      </c>
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="Z17" s="1" t="s">
@@ -2270,6 +2313,18 @@
       <c r="O18" s="2">
         <v>45793</v>
       </c>
+      <c r="P18" s="2">
+        <v>45785</v>
+      </c>
+      <c r="Q18" s="5">
+        <v>0.51736111111111116</v>
+      </c>
+      <c r="R18" t="s">
+        <v>224</v>
+      </c>
+      <c r="S18" t="s">
+        <v>225</v>
+      </c>
       <c r="T18" t="s">
         <v>192</v>
       </c>
@@ -2869,7 +2924,7 @@
       </c>
       <c r="O28" s="2"/>
       <c r="T28" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="U28" s="2"/>
       <c r="V28" s="2"/>
@@ -2944,7 +2999,7 @@
         <v>83</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J30" t="s">
         <v>30</v>
@@ -2988,7 +3043,7 @@
         <v>84</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J31" t="s">
         <v>31</v>
@@ -3032,7 +3087,7 @@
         <v>85</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J32" t="s">
         <v>32</v>
@@ -3076,7 +3131,7 @@
         <v>86</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J33" t="s">
         <v>33</v>
@@ -3120,7 +3175,7 @@
         <v>87</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J34" t="s">
         <v>53</v>
@@ -3164,7 +3219,7 @@
         <v>88</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J35" t="s">
         <v>52</v>
@@ -3208,7 +3263,7 @@
         <v>89</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J36" t="s">
         <v>34</v>
@@ -3252,7 +3307,7 @@
         <v>90</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J37" t="s">
         <v>35</v>
@@ -3296,7 +3351,7 @@
         <v>91</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J38" t="s">
         <v>36</v>
@@ -3312,7 +3367,7 @@
       </c>
       <c r="O38" s="2"/>
       <c r="T38" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="U38" s="2"/>
       <c r="V38" s="2"/>
@@ -3979,13 +4034,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CBFCE6-FDA2-9B4E-A8C1-1998B7362B23}">
-  <dimension ref="A1:AF56"/>
+  <dimension ref="A1:AL56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4082,8 +4137,26 @@
       <c r="AF1" s="10">
         <v>45870</v>
       </c>
-    </row>
-    <row r="2" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG1" s="10">
+        <v>45696</v>
+      </c>
+      <c r="AH1" s="10">
+        <v>45724</v>
+      </c>
+      <c r="AI1" s="10">
+        <v>45755</v>
+      </c>
+      <c r="AJ1" s="10">
+        <v>45785</v>
+      </c>
+      <c r="AK1" s="10">
+        <v>45816</v>
+      </c>
+      <c r="AL1" s="10">
+        <v>45846</v>
+      </c>
+    </row>
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -4118,8 +4191,14 @@
       <c r="AD2" s="6"/>
       <c r="AE2" s="6"/>
       <c r="AF2" s="6"/>
-    </row>
-    <row r="3" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG2" s="6"/>
+      <c r="AH2" s="6"/>
+      <c r="AI2" s="6"/>
+      <c r="AJ2" s="6"/>
+      <c r="AK2" s="6"/>
+      <c r="AL2" s="6"/>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
@@ -4154,8 +4233,14 @@
       <c r="AD3" s="6"/>
       <c r="AE3" s="6"/>
       <c r="AF3" s="6"/>
-    </row>
-    <row r="4" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG3" s="6"/>
+      <c r="AH3" s="6"/>
+      <c r="AI3" s="6"/>
+      <c r="AJ3" s="6"/>
+      <c r="AK3" s="6"/>
+      <c r="AL3" s="6"/>
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>57</v>
       </c>
@@ -4190,8 +4275,14 @@
       <c r="AD4" s="6"/>
       <c r="AE4" s="6"/>
       <c r="AF4" s="6"/>
-    </row>
-    <row r="5" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG4" s="6"/>
+      <c r="AH4" s="6"/>
+      <c r="AI4" s="6"/>
+      <c r="AJ4" s="6"/>
+      <c r="AK4" s="6"/>
+      <c r="AL4" s="6"/>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>58</v>
       </c>
@@ -4226,8 +4317,14 @@
       <c r="AD5" s="6"/>
       <c r="AE5" s="6"/>
       <c r="AF5" s="6"/>
-    </row>
-    <row r="6" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG5" s="6"/>
+      <c r="AH5" s="6"/>
+      <c r="AI5" s="6"/>
+      <c r="AJ5" s="6"/>
+      <c r="AK5" s="6"/>
+      <c r="AL5" s="6"/>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>59</v>
       </c>
@@ -4262,8 +4359,14 @@
       <c r="AD6" s="6"/>
       <c r="AE6" s="6"/>
       <c r="AF6" s="6"/>
-    </row>
-    <row r="7" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG6" s="6"/>
+      <c r="AH6" s="6"/>
+      <c r="AI6" s="6"/>
+      <c r="AJ6" s="6"/>
+      <c r="AK6" s="6"/>
+      <c r="AL6" s="6"/>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>60</v>
       </c>
@@ -4298,8 +4401,14 @@
       <c r="AD7" s="8"/>
       <c r="AE7" s="8"/>
       <c r="AF7" s="8"/>
-    </row>
-    <row r="8" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG7" s="8"/>
+      <c r="AH7" s="8"/>
+      <c r="AI7" s="8"/>
+      <c r="AJ7" s="8"/>
+      <c r="AK7" s="8"/>
+      <c r="AL7" s="8"/>
+    </row>
+    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>61</v>
       </c>
@@ -4334,8 +4443,14 @@
       <c r="AD8" s="8"/>
       <c r="AE8" s="8"/>
       <c r="AF8" s="8"/>
-    </row>
-    <row r="9" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG8" s="8"/>
+      <c r="AH8" s="8"/>
+      <c r="AI8" s="8"/>
+      <c r="AJ8" s="8"/>
+      <c r="AK8" s="8"/>
+      <c r="AL8" s="8"/>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>62</v>
       </c>
@@ -4370,8 +4485,14 @@
       <c r="AD9" s="8"/>
       <c r="AE9" s="8"/>
       <c r="AF9" s="8"/>
-    </row>
-    <row r="10" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG9" s="8"/>
+      <c r="AH9" s="8"/>
+      <c r="AI9" s="8"/>
+      <c r="AJ9" s="8"/>
+      <c r="AK9" s="8"/>
+      <c r="AL9" s="8"/>
+    </row>
+    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>63</v>
       </c>
@@ -4385,29 +4506,35 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="7"/>
-      <c r="Q10" s="7"/>
-      <c r="R10" s="7"/>
-      <c r="S10" s="7"/>
-      <c r="T10" s="7"/>
-      <c r="U10" s="7"/>
-      <c r="V10" s="7"/>
-      <c r="W10" s="7"/>
-      <c r="X10" s="7"/>
-      <c r="Y10" s="7"/>
-      <c r="Z10" s="7"/>
-      <c r="AA10" s="7"/>
-      <c r="AB10" s="7"/>
-      <c r="AC10" s="7"/>
-      <c r="AD10" s="7"/>
-      <c r="AE10" s="7"/>
-      <c r="AF10" s="7"/>
-    </row>
-    <row r="11" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="L10" s="12"/>
+      <c r="M10" s="12"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="12"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="12"/>
+      <c r="V10" s="12"/>
+      <c r="W10" s="12"/>
+      <c r="X10" s="12"/>
+      <c r="Y10" s="12"/>
+      <c r="Z10" s="12"/>
+      <c r="AA10" s="12"/>
+      <c r="AB10" s="12"/>
+      <c r="AC10" s="12"/>
+      <c r="AD10" s="12"/>
+      <c r="AE10" s="12"/>
+      <c r="AF10" s="12"/>
+      <c r="AG10" s="12"/>
+      <c r="AH10" s="12"/>
+      <c r="AI10" s="12"/>
+      <c r="AJ10" s="12"/>
+      <c r="AK10" s="12"/>
+      <c r="AL10" s="12"/>
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>64</v>
       </c>
@@ -4442,8 +4569,14 @@
       <c r="AD11" s="8"/>
       <c r="AE11" s="8"/>
       <c r="AF11" s="8"/>
-    </row>
-    <row r="12" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG11" s="8"/>
+      <c r="AH11" s="8"/>
+      <c r="AI11" s="8"/>
+      <c r="AJ11" s="8"/>
+      <c r="AK11" s="8"/>
+      <c r="AL11" s="8"/>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>65</v>
       </c>
@@ -4478,8 +4611,14 @@
       <c r="AD12" s="8"/>
       <c r="AE12" s="8"/>
       <c r="AF12" s="8"/>
-    </row>
-    <row r="13" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG12" s="8"/>
+      <c r="AH12" s="8"/>
+      <c r="AI12" s="8"/>
+      <c r="AJ12" s="8"/>
+      <c r="AK12" s="8"/>
+      <c r="AL12" s="8"/>
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
@@ -4514,8 +4653,14 @@
       <c r="AD13" s="8"/>
       <c r="AE13" s="8"/>
       <c r="AF13" s="8"/>
-    </row>
-    <row r="14" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG13" s="8"/>
+      <c r="AH13" s="8"/>
+      <c r="AI13" s="8"/>
+      <c r="AJ13" s="8"/>
+      <c r="AK13" s="8"/>
+      <c r="AL13" s="8"/>
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>67</v>
       </c>
@@ -4550,8 +4695,14 @@
       <c r="AD14" s="8"/>
       <c r="AE14" s="8"/>
       <c r="AF14" s="8"/>
-    </row>
-    <row r="15" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG14" s="8"/>
+      <c r="AH14" s="8"/>
+      <c r="AI14" s="8"/>
+      <c r="AJ14" s="8"/>
+      <c r="AK14" s="8"/>
+      <c r="AL14" s="8"/>
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>68</v>
       </c>
@@ -4560,7 +4711,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="16" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
@@ -4568,8 +4719,11 @@
       <c r="F16" s="9"/>
       <c r="G16" s="9"/>
       <c r="H16" s="9"/>
-    </row>
-    <row r="17" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AJ16" s="8"/>
+      <c r="AK16" s="8"/>
+      <c r="AL16" s="8"/>
+    </row>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -4577,8 +4731,11 @@
       <c r="F17" s="9"/>
       <c r="G17" s="9"/>
       <c r="H17" s="9"/>
-    </row>
-    <row r="18" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AJ17" s="8"/>
+      <c r="AK17" s="8"/>
+      <c r="AL17" s="8"/>
+    </row>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>71</v>
       </c>
@@ -4586,8 +4743,11 @@
       <c r="F18" s="9"/>
       <c r="G18" s="9"/>
       <c r="H18" s="9"/>
-    </row>
-    <row r="19" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AJ18" s="8"/>
+      <c r="AK18" s="8"/>
+      <c r="AL18" s="8"/>
+    </row>
+    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>72</v>
       </c>
@@ -4622,8 +4782,14 @@
       <c r="AD19" s="8"/>
       <c r="AE19" s="8"/>
       <c r="AF19" s="8"/>
-    </row>
-    <row r="20" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG19" s="8"/>
+      <c r="AH19" s="8"/>
+      <c r="AI19" s="8"/>
+      <c r="AJ19" s="8"/>
+      <c r="AK19" s="8"/>
+      <c r="AL19" s="8"/>
+    </row>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>73</v>
       </c>
@@ -4658,8 +4824,14 @@
       <c r="AD20" s="8"/>
       <c r="AE20" s="8"/>
       <c r="AF20" s="8"/>
-    </row>
-    <row r="21" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG20" s="8"/>
+      <c r="AH20" s="8"/>
+      <c r="AI20" s="8"/>
+      <c r="AJ20" s="8"/>
+      <c r="AK20" s="8"/>
+      <c r="AL20" s="8"/>
+    </row>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>74</v>
       </c>
@@ -4694,8 +4866,14 @@
       <c r="AD21" s="8"/>
       <c r="AE21" s="8"/>
       <c r="AF21" s="8"/>
-    </row>
-    <row r="22" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG21" s="8"/>
+      <c r="AH21" s="8"/>
+      <c r="AI21" s="8"/>
+      <c r="AJ21" s="8"/>
+      <c r="AK21" s="8"/>
+      <c r="AL21" s="8"/>
+    </row>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>75</v>
       </c>
@@ -4730,8 +4908,14 @@
       <c r="AD22" s="8"/>
       <c r="AE22" s="8"/>
       <c r="AF22" s="8"/>
-    </row>
-    <row r="23" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG22" s="8"/>
+      <c r="AH22" s="8"/>
+      <c r="AI22" s="8"/>
+      <c r="AJ22" s="8"/>
+      <c r="AK22" s="8"/>
+      <c r="AL22" s="8"/>
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>76</v>
       </c>
@@ -4766,8 +4950,14 @@
       <c r="AD23" s="8"/>
       <c r="AE23" s="8"/>
       <c r="AF23" s="8"/>
-    </row>
-    <row r="24" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG23" s="8"/>
+      <c r="AH23" s="8"/>
+      <c r="AI23" s="8"/>
+      <c r="AJ23" s="8"/>
+      <c r="AK23" s="8"/>
+      <c r="AL23" s="8"/>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>77</v>
       </c>
@@ -4802,8 +4992,14 @@
       <c r="AD24" s="8"/>
       <c r="AE24" s="8"/>
       <c r="AF24" s="8"/>
-    </row>
-    <row r="25" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG24" s="8"/>
+      <c r="AH24" s="8"/>
+      <c r="AI24" s="8"/>
+      <c r="AJ24" s="8"/>
+      <c r="AK24" s="8"/>
+      <c r="AL24" s="8"/>
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>78</v>
       </c>
@@ -4811,8 +5007,32 @@
       <c r="F25" s="9"/>
       <c r="G25" s="9"/>
       <c r="H25" s="9"/>
-    </row>
-    <row r="26" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+      <c r="V25" s="8"/>
+      <c r="W25" s="8"/>
+      <c r="X25" s="8"/>
+      <c r="Y25" s="8"/>
+      <c r="Z25" s="8"/>
+      <c r="AA25" s="8"/>
+      <c r="AB25" s="8"/>
+      <c r="AC25" s="8"/>
+      <c r="AD25" s="8"/>
+      <c r="AE25" s="8"/>
+      <c r="AF25" s="8"/>
+      <c r="AG25" s="8"/>
+      <c r="AH25" s="8"/>
+      <c r="AI25" s="8"/>
+      <c r="AJ25" s="8"/>
+      <c r="AK25" s="8"/>
+      <c r="AL25" s="8"/>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>79</v>
       </c>
@@ -4847,33 +5067,39 @@
       <c r="AD26" s="8"/>
       <c r="AE26" s="8"/>
       <c r="AF26" s="8"/>
-    </row>
-    <row r="27" spans="1:32" x14ac:dyDescent="0.2">
+      <c r="AG26" s="8"/>
+      <c r="AH26" s="8"/>
+      <c r="AI26" s="8"/>
+      <c r="AJ26" s="8"/>
+      <c r="AK26" s="8"/>
+      <c r="AL26" s="8"/>
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="28" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="30" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:32" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>85</v>
       </c>
@@ -4902,7 +5128,7 @@
         <v>161</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated box component tracker and updated box deployment pictures
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6037CA19-65B4-9A4B-BBFC-0CEE82B4F6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8CAA77-83AC-A64F-B889-1EA13E0E2248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="900" yWindow="1260" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="4600" yWindow="2340" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="231">
   <si>
     <t>Box Number</t>
   </si>
@@ -727,6 +727,9 @@
   </si>
   <si>
     <t>42.3164061, -71.0826839</t>
+  </si>
+  <si>
+    <t>Collection Date</t>
   </si>
 </sst>
 </file>
@@ -812,7 +815,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -825,7 +828,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1160,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:AA56"/>
+  <dimension ref="A1:AC56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -1180,12 +1182,13 @@
     <col min="17" max="17" width="15.5" customWidth="1"/>
     <col min="18" max="18" width="28" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="22" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="51.5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="26" max="26" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="51.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1244,13 +1247,17 @@
         <v>112</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="U1" s="1"/>
       <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
       <c r="X1" s="1"/>
-    </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z1" s="1"/>
+    </row>
+    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -1306,10 +1313,10 @@
       <c r="S2" t="s">
         <v>116</v>
       </c>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-    </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W2" s="2"/>
+      <c r="X2" s="2"/>
+    </row>
+    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
@@ -1365,10 +1372,10 @@
       <c r="S3" t="s">
         <v>155</v>
       </c>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-    </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W3" s="2"/>
+      <c r="X3" s="2"/>
+    </row>
+    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>57</v>
       </c>
@@ -1424,16 +1431,16 @@
       <c r="S4" t="s">
         <v>120</v>
       </c>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="Z4" s="1" t="s">
+      <c r="W4" s="2"/>
+      <c r="X4" s="2"/>
+      <c r="AB4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="AA4" t="s">
+      <c r="AC4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>58</v>
       </c>
@@ -1489,16 +1496,16 @@
       <c r="S5" t="s">
         <v>125</v>
       </c>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="Z5" s="1" t="s">
+      <c r="W5" s="2"/>
+      <c r="X5" s="2"/>
+      <c r="AB5" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="AA5" t="s">
+      <c r="AC5" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>59</v>
       </c>
@@ -1554,16 +1561,16 @@
       <c r="S6" t="s">
         <v>119</v>
       </c>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="Z6" s="1" t="s">
+      <c r="W6" s="2"/>
+      <c r="X6" s="2"/>
+      <c r="AB6" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="AA6" t="s">
+      <c r="AC6" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>60</v>
       </c>
@@ -1619,16 +1626,16 @@
       <c r="S7" t="s">
         <v>123</v>
       </c>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="Z7" s="1" t="s">
+      <c r="W7" s="2"/>
+      <c r="X7" s="2"/>
+      <c r="AB7" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="AA7" t="s">
+      <c r="AC7" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>61</v>
       </c>
@@ -1684,16 +1691,16 @@
       <c r="S8" t="s">
         <v>128</v>
       </c>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="Z8" s="1" t="s">
+      <c r="W8" s="2"/>
+      <c r="X8" s="2"/>
+      <c r="AB8" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AC8" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>62</v>
       </c>
@@ -1749,16 +1756,16 @@
       <c r="S9" t="s">
         <v>130</v>
       </c>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="Z9" s="1" t="s">
+      <c r="W9" s="2"/>
+      <c r="X9" s="2"/>
+      <c r="AB9" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AC9" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>63</v>
       </c>
@@ -1814,19 +1821,19 @@
       <c r="S10" t="s">
         <v>149</v>
       </c>
-      <c r="T10" t="s">
+      <c r="U10" t="s">
         <v>215</v>
       </c>
-      <c r="U10" s="2"/>
-      <c r="V10" s="2"/>
-      <c r="Z10" s="1" t="s">
+      <c r="W10" s="2"/>
+      <c r="X10" s="2"/>
+      <c r="AB10" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AC10" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>64</v>
       </c>
@@ -1873,22 +1880,25 @@
       <c r="P11" t="s">
         <v>126</v>
       </c>
+      <c r="Q11" s="5">
+        <v>0.47569444444444442</v>
+      </c>
       <c r="R11" t="s">
         <v>132</v>
       </c>
       <c r="S11" t="s">
         <v>133</v>
       </c>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="Z11" s="1" t="s">
+      <c r="W11" s="2"/>
+      <c r="X11" s="2"/>
+      <c r="AB11" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AC11" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>65</v>
       </c>
@@ -1944,16 +1954,16 @@
       <c r="S12" t="s">
         <v>141</v>
       </c>
-      <c r="U12" s="2"/>
-      <c r="V12" s="2"/>
-      <c r="Z12" s="1" t="s">
+      <c r="W12" s="2"/>
+      <c r="X12" s="2"/>
+      <c r="AB12" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="AA12" t="s">
+      <c r="AC12" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
@@ -2009,16 +2019,16 @@
       <c r="S13" t="s">
         <v>135</v>
       </c>
-      <c r="U13" s="2"/>
-      <c r="V13" s="2"/>
-      <c r="Z13" s="1" t="s">
+      <c r="W13" s="2"/>
+      <c r="X13" s="2"/>
+      <c r="AB13" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AA13" t="s">
+      <c r="AC13" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>67</v>
       </c>
@@ -2074,16 +2084,16 @@
       <c r="S14" t="s">
         <v>136</v>
       </c>
-      <c r="U14" s="2"/>
-      <c r="V14" s="2"/>
-      <c r="Z14" s="3" t="s">
+      <c r="W14" s="2"/>
+      <c r="X14" s="2"/>
+      <c r="AB14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="AA14" t="s">
+      <c r="AC14" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>68</v>
       </c>
@@ -2127,19 +2137,19 @@
       <c r="O15" s="2">
         <v>45793</v>
       </c>
-      <c r="T15" t="s">
+      <c r="U15" t="s">
         <v>192</v>
       </c>
-      <c r="U15" s="2"/>
-      <c r="V15" s="2"/>
-      <c r="Z15" s="1" t="s">
+      <c r="W15" s="2"/>
+      <c r="X15" s="2"/>
+      <c r="AB15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AA15" t="s">
+      <c r="AC15" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
@@ -2195,16 +2205,16 @@
       <c r="S16" t="s">
         <v>227</v>
       </c>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-      <c r="Z16" s="1" t="s">
+      <c r="W16" s="2"/>
+      <c r="X16" s="2"/>
+      <c r="AB16" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="AA16" t="s">
+      <c r="AC16" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -2260,16 +2270,16 @@
       <c r="S17" t="s">
         <v>229</v>
       </c>
-      <c r="U17" s="2"/>
-      <c r="V17" s="2"/>
-      <c r="Z17" s="1" t="s">
+      <c r="W17" s="2"/>
+      <c r="X17" s="2"/>
+      <c r="AB17" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="AA17" t="s">
+      <c r="AC17" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>71</v>
       </c>
@@ -2325,19 +2335,19 @@
       <c r="S18" t="s">
         <v>225</v>
       </c>
-      <c r="T18" t="s">
+      <c r="U18" t="s">
         <v>192</v>
       </c>
-      <c r="U18" s="2"/>
-      <c r="V18" s="2"/>
-      <c r="Z18" s="1" t="s">
+      <c r="W18" s="2"/>
+      <c r="X18" s="2"/>
+      <c r="AB18" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="AA18" t="s">
+      <c r="AC18" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>72</v>
       </c>
@@ -2393,16 +2403,16 @@
       <c r="S19" t="s">
         <v>158</v>
       </c>
-      <c r="U19" s="2"/>
-      <c r="V19" s="2"/>
-      <c r="Z19" s="1" t="s">
+      <c r="W19" s="2"/>
+      <c r="X19" s="2"/>
+      <c r="AB19" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AA19" t="s">
+      <c r="AC19" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>73</v>
       </c>
@@ -2458,16 +2468,16 @@
       <c r="S20" t="s">
         <v>139</v>
       </c>
-      <c r="U20" s="2"/>
-      <c r="V20" s="2"/>
-      <c r="Z20" s="1" t="s">
+      <c r="W20" s="2"/>
+      <c r="X20" s="2"/>
+      <c r="AB20" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="AA20" t="s">
+      <c r="AC20" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>74</v>
       </c>
@@ -2523,16 +2533,16 @@
       <c r="S21" t="s">
         <v>147</v>
       </c>
-      <c r="U21" s="2"/>
-      <c r="V21" s="2"/>
-      <c r="Z21" s="1" t="s">
+      <c r="W21" s="2"/>
+      <c r="X21" s="2"/>
+      <c r="AB21" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="AA21" t="s">
+      <c r="AC21" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>75</v>
       </c>
@@ -2576,16 +2586,28 @@
       <c r="O22" s="2">
         <v>45793</v>
       </c>
-      <c r="U22" s="2"/>
-      <c r="V22" s="2"/>
-      <c r="Z22" s="1" t="s">
+      <c r="P22" t="s">
+        <v>150</v>
+      </c>
+      <c r="Q22" s="5">
+        <v>0.45763888888888887</v>
+      </c>
+      <c r="R22" t="s">
+        <v>153</v>
+      </c>
+      <c r="S22" t="s">
+        <v>154</v>
+      </c>
+      <c r="W22" s="2"/>
+      <c r="X22" s="2"/>
+      <c r="AB22" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="AA22" t="s">
+      <c r="AC22" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="23" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>76</v>
       </c>
@@ -2633,18 +2655,18 @@
         <v>150</v>
       </c>
       <c r="Q23" s="5">
-        <v>0.45763888888888887</v>
+        <v>0.42499999999999999</v>
       </c>
       <c r="R23" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="S23" t="s">
-        <v>154</v>
-      </c>
-      <c r="U23" s="2"/>
-      <c r="V23" s="2"/>
-    </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
+        <v>152</v>
+      </c>
+      <c r="W23" s="2"/>
+      <c r="X23" s="2"/>
+    </row>
+    <row r="24" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>77</v>
       </c>
@@ -2700,10 +2722,10 @@
       <c r="S24" t="s">
         <v>143</v>
       </c>
-      <c r="U24" s="2"/>
-      <c r="V24" s="2"/>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W24" s="2"/>
+      <c r="X24" s="2"/>
+    </row>
+    <row r="25" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>78</v>
       </c>
@@ -2759,10 +2781,10 @@
       <c r="S25" t="s">
         <v>189</v>
       </c>
-      <c r="U25" s="2"/>
-      <c r="V25" s="2"/>
-    </row>
-    <row r="26" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W25" s="2"/>
+      <c r="X25" s="2"/>
+    </row>
+    <row r="26" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>79</v>
       </c>
@@ -2818,10 +2840,10 @@
       <c r="S26" t="s">
         <v>144</v>
       </c>
-      <c r="U26" s="2"/>
-      <c r="V26" s="2"/>
-    </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W26" s="2"/>
+      <c r="X26" s="2"/>
+    </row>
+    <row r="27" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
@@ -2865,24 +2887,12 @@
         <v>168</v>
       </c>
       <c r="O27" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P27" t="s">
-        <v>150</v>
-      </c>
-      <c r="Q27" s="5">
-        <v>0.42499999999999999</v>
-      </c>
-      <c r="R27" t="s">
-        <v>151</v>
-      </c>
-      <c r="S27" t="s">
-        <v>152</v>
-      </c>
-      <c r="U27" s="2"/>
-      <c r="V27" s="2"/>
-    </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.2">
+        <v>45874</v>
+      </c>
+      <c r="W27" s="2"/>
+      <c r="X27" s="2"/>
+    </row>
+    <row r="28" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>81</v>
       </c>
@@ -2923,13 +2933,13 @@
         <v>45793</v>
       </c>
       <c r="O28" s="2"/>
-      <c r="T28" t="s">
+      <c r="U28" t="s">
         <v>214</v>
       </c>
-      <c r="U28" s="2"/>
-      <c r="V28" s="2"/>
-    </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W28" s="2"/>
+      <c r="X28" s="2"/>
+    </row>
+    <row r="29" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>82</v>
       </c>
@@ -2970,10 +2980,10 @@
         <v>45793</v>
       </c>
       <c r="O29" s="2"/>
-      <c r="U29" s="2"/>
-      <c r="V29" s="2"/>
-    </row>
-    <row r="30" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W29" s="2"/>
+      <c r="X29" s="2"/>
+    </row>
+    <row r="30" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>83</v>
       </c>
@@ -3014,10 +3024,10 @@
         <v>45793</v>
       </c>
       <c r="O30" s="2"/>
-      <c r="U30" s="2"/>
-      <c r="V30" s="2"/>
-    </row>
-    <row r="31" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W30" s="2"/>
+      <c r="X30" s="2"/>
+    </row>
+    <row r="31" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
@@ -3058,10 +3068,10 @@
         <v>45793</v>
       </c>
       <c r="O31" s="2"/>
-      <c r="U31" s="2"/>
-      <c r="V31" s="2"/>
-    </row>
-    <row r="32" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="W31" s="2"/>
+      <c r="X31" s="2"/>
+    </row>
+    <row r="32" spans="1:29" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>85</v>
       </c>
@@ -3102,10 +3112,10 @@
         <v>45793</v>
       </c>
       <c r="O32" s="2"/>
-      <c r="U32" s="2"/>
-      <c r="V32" s="2"/>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W32" s="2"/>
+      <c r="X32" s="2"/>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>86</v>
       </c>
@@ -3146,10 +3156,10 @@
         <v>45793</v>
       </c>
       <c r="O33" s="2"/>
-      <c r="U33" s="2"/>
-      <c r="V33" s="2"/>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W33" s="2"/>
+      <c r="X33" s="2"/>
+    </row>
+    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>87</v>
       </c>
@@ -3190,10 +3200,10 @@
         <v>45793</v>
       </c>
       <c r="O34" s="2"/>
-      <c r="U34" s="2"/>
-      <c r="V34" s="2"/>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W34" s="2"/>
+      <c r="X34" s="2"/>
+    </row>
+    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>88</v>
       </c>
@@ -3234,10 +3244,10 @@
         <v>45793</v>
       </c>
       <c r="O35" s="2"/>
-      <c r="U35" s="2"/>
-      <c r="V35" s="2"/>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W35" s="2"/>
+      <c r="X35" s="2"/>
+    </row>
+    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>89</v>
       </c>
@@ -3278,10 +3288,10 @@
         <v>45793</v>
       </c>
       <c r="O36" s="2"/>
-      <c r="U36" s="2"/>
-      <c r="V36" s="2"/>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W36" s="2"/>
+      <c r="X36" s="2"/>
+    </row>
+    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>90</v>
       </c>
@@ -3322,10 +3332,10 @@
         <v>45793</v>
       </c>
       <c r="O37" s="2"/>
-      <c r="U37" s="2"/>
-      <c r="V37" s="2"/>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W37" s="2"/>
+      <c r="X37" s="2"/>
+    </row>
+    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>91</v>
       </c>
@@ -3366,13 +3376,13 @@
         <v>45793</v>
       </c>
       <c r="O38" s="2"/>
-      <c r="T38" t="s">
+      <c r="U38" t="s">
         <v>214</v>
       </c>
-      <c r="U38" s="2"/>
-      <c r="V38" s="2"/>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W38" s="2"/>
+      <c r="X38" s="2"/>
+    </row>
+    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>92</v>
       </c>
@@ -3411,10 +3421,10 @@
         <v>45793</v>
       </c>
       <c r="O39" s="2"/>
-      <c r="U39" s="2"/>
-      <c r="V39" s="2"/>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W39" s="2"/>
+      <c r="X39" s="2"/>
+    </row>
+    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>93</v>
       </c>
@@ -3453,10 +3463,10 @@
         <v>45793</v>
       </c>
       <c r="O40" s="2"/>
-      <c r="U40" s="2"/>
-      <c r="V40" s="2"/>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W40" s="2"/>
+      <c r="X40" s="2"/>
+    </row>
+    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>94</v>
       </c>
@@ -3495,10 +3505,10 @@
         <v>45793</v>
       </c>
       <c r="O41" s="2"/>
-      <c r="U41" s="2"/>
-      <c r="V41" s="2"/>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W41" s="2"/>
+      <c r="X41" s="2"/>
+    </row>
+    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>95</v>
       </c>
@@ -3537,10 +3547,10 @@
         <v>45793</v>
       </c>
       <c r="O42" s="2"/>
-      <c r="U42" s="2"/>
-      <c r="V42" s="2"/>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W42" s="2"/>
+      <c r="X42" s="2"/>
+    </row>
+    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>96</v>
       </c>
@@ -3579,10 +3589,10 @@
         <v>45793</v>
       </c>
       <c r="O43" s="2"/>
-      <c r="U43" s="2"/>
-      <c r="V43" s="2"/>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W43" s="2"/>
+      <c r="X43" s="2"/>
+    </row>
+    <row r="44" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>97</v>
       </c>
@@ -3621,10 +3631,10 @@
         <v>45793</v>
       </c>
       <c r="O44" s="2"/>
-      <c r="U44" s="2"/>
-      <c r="V44" s="2"/>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W44" s="2"/>
+      <c r="X44" s="2"/>
+    </row>
+    <row r="45" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>98</v>
       </c>
@@ -3663,10 +3673,10 @@
         <v>45793</v>
       </c>
       <c r="O45" s="2"/>
-      <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W45" s="2"/>
+      <c r="X45" s="2"/>
+    </row>
+    <row r="46" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>99</v>
       </c>
@@ -3705,10 +3715,10 @@
         <v>45793</v>
       </c>
       <c r="O46" s="2"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="2"/>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W46" s="2"/>
+      <c r="X46" s="2"/>
+    </row>
+    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>100</v>
       </c>
@@ -3747,10 +3757,10 @@
         <v>45793</v>
       </c>
       <c r="O47" s="2"/>
-      <c r="U47" s="2"/>
-      <c r="V47" s="2"/>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W47" s="2"/>
+      <c r="X47" s="2"/>
+    </row>
+    <row r="48" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>101</v>
       </c>
@@ -3789,10 +3799,10 @@
         <v>45793</v>
       </c>
       <c r="O48" s="2"/>
-      <c r="U48" s="2"/>
-      <c r="V48" s="2"/>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W48" s="2"/>
+      <c r="X48" s="2"/>
+    </row>
+    <row r="49" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>102</v>
       </c>
@@ -3831,10 +3841,10 @@
         <v>45793</v>
       </c>
       <c r="O49" s="2"/>
-      <c r="U49" s="2"/>
-      <c r="V49" s="2"/>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W49" s="2"/>
+      <c r="X49" s="2"/>
+    </row>
+    <row r="50" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>103</v>
       </c>
@@ -3873,10 +3883,10 @@
         <v>45793</v>
       </c>
       <c r="O50" s="2"/>
-      <c r="U50" s="2"/>
-      <c r="V50" s="2"/>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W50" s="2"/>
+      <c r="X50" s="2"/>
+    </row>
+    <row r="51" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>104</v>
       </c>
@@ -3915,10 +3925,10 @@
         <v>45793</v>
       </c>
       <c r="O51" s="2"/>
-      <c r="U51" s="2"/>
-      <c r="V51" s="2"/>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W51" s="2"/>
+      <c r="X51" s="2"/>
+    </row>
+    <row r="52" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>105</v>
       </c>
@@ -3943,10 +3953,10 @@
         <v>45793</v>
       </c>
       <c r="O52" s="2"/>
-      <c r="U52" s="2"/>
-      <c r="V52" s="2"/>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W52" s="2"/>
+      <c r="X52" s="2"/>
+    </row>
+    <row r="53" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>106</v>
       </c>
@@ -3971,10 +3981,10 @@
         <v>45793</v>
       </c>
       <c r="O53" s="2"/>
-      <c r="U53" s="2"/>
-      <c r="V53" s="2"/>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W53" s="2"/>
+      <c r="X53" s="2"/>
+    </row>
+    <row r="54" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>107</v>
       </c>
@@ -3988,10 +3998,10 @@
       <c r="I54" s="4"/>
       <c r="M54" s="2"/>
       <c r="O54" s="2"/>
-      <c r="U54" s="2"/>
-      <c r="V54" s="2"/>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W54" s="2"/>
+      <c r="X54" s="2"/>
+    </row>
+    <row r="55" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
@@ -4005,10 +4015,10 @@
       <c r="I55" s="4"/>
       <c r="M55" s="2"/>
       <c r="O55" s="2"/>
-      <c r="U55" s="2"/>
-      <c r="V55" s="2"/>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="W55" s="2"/>
+      <c r="X55" s="2"/>
+    </row>
+    <row r="56" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>109</v>
       </c>
@@ -4022,8 +4032,8 @@
       <c r="I56" s="4"/>
       <c r="M56" s="2"/>
       <c r="O56" s="2"/>
-      <c r="U56" s="2"/>
-      <c r="V56" s="2"/>
+      <c r="W56" s="2"/>
+      <c r="X56" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -4506,33 +4516,6 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="7"/>
-      <c r="L10" s="12"/>
-      <c r="M10" s="12"/>
-      <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="12"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="12"/>
-      <c r="W10" s="12"/>
-      <c r="X10" s="12"/>
-      <c r="Y10" s="12"/>
-      <c r="Z10" s="12"/>
-      <c r="AA10" s="12"/>
-      <c r="AB10" s="12"/>
-      <c r="AC10" s="12"/>
-      <c r="AD10" s="12"/>
-      <c r="AE10" s="12"/>
-      <c r="AF10" s="12"/>
-      <c r="AG10" s="12"/>
-      <c r="AH10" s="12"/>
-      <c r="AI10" s="12"/>
-      <c r="AJ10" s="12"/>
-      <c r="AK10" s="12"/>
-      <c r="AL10" s="12"/>
     </row>
     <row r="11" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">

</xml_diff>

<commit_message>
Updated the deployment tracker sheet for components 51-55
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C8CAA77-83AC-A64F-B889-1EA13E0E2248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3377F4DA-9D41-F44A-98AB-32147E6F64EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4600" yWindow="2340" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="1040" yWindow="1240" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="812" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="232">
   <si>
     <t>Box Number</t>
   </si>
@@ -730,6 +730,9 @@
   </si>
   <si>
     <t>Collection Date</t>
+  </si>
+  <si>
+    <t>08/14/2025</t>
   </si>
 </sst>
 </file>
@@ -2889,6 +2892,18 @@
       <c r="O27" s="2">
         <v>45874</v>
       </c>
+      <c r="P27" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="Q27" s="5">
+        <v>0.4909722222222222</v>
+      </c>
+      <c r="R27" t="s">
+        <v>148</v>
+      </c>
+      <c r="S27" t="s">
+        <v>149</v>
+      </c>
       <c r="W27" s="2"/>
       <c r="X27" s="2"/>
     </row>
@@ -3932,13 +3947,27 @@
       <c r="A52" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="4"/>
-      <c r="C52" s="4"/>
-      <c r="D52" s="4"/>
-      <c r="E52" s="4"/>
-      <c r="F52" s="4"/>
-      <c r="G52" s="4"/>
-      <c r="H52" s="4"/>
+      <c r="B52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>105</v>
+      </c>
       <c r="I52" s="4"/>
       <c r="J52" t="s">
         <v>50</v>
@@ -3960,13 +3989,27 @@
       <c r="A53" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B53" s="4"/>
-      <c r="C53" s="4"/>
-      <c r="D53" s="4"/>
-      <c r="E53" s="4"/>
-      <c r="F53" s="4"/>
-      <c r="G53" s="4"/>
-      <c r="H53" s="4"/>
+      <c r="B53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="I53" s="4"/>
       <c r="J53" t="s">
         <v>51</v>
@@ -3988,13 +4031,27 @@
       <c r="A54" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
-      <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
-      <c r="F54" s="4"/>
-      <c r="G54" s="4"/>
-      <c r="H54" s="4"/>
+      <c r="B54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="I54" s="4"/>
       <c r="M54" s="2"/>
       <c r="O54" s="2"/>
@@ -4005,13 +4062,27 @@
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="4"/>
-      <c r="C55" s="4"/>
-      <c r="D55" s="4"/>
-      <c r="E55" s="4"/>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
-      <c r="H55" s="4"/>
+      <c r="B55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="H55" s="4" t="s">
+        <v>108</v>
+      </c>
       <c r="I55" s="4"/>
       <c r="M55" s="2"/>
       <c r="O55" s="2"/>
@@ -4022,13 +4093,27 @@
       <c r="A56" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="B56" s="4"/>
-      <c r="C56" s="4"/>
-      <c r="D56" s="4"/>
-      <c r="E56" s="4"/>
-      <c r="F56" s="4"/>
-      <c r="G56" s="4"/>
-      <c r="H56" s="4"/>
+      <c r="B56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H56" s="4" t="s">
+        <v>109</v>
+      </c>
       <c r="I56" s="4"/>
       <c r="M56" s="2"/>
       <c r="O56" s="2"/>

</xml_diff>

<commit_message>
Updated the sensor box deployment tracker sheet for the latest deployment of boxes
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0392F055-DF90-1140-9490-1223769BD0F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE140A8-C0BF-A44C-B3EF-4FA3AEE5ACD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1040" yWindow="1240" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="241">
   <si>
     <t>Box Number</t>
   </si>
@@ -733,6 +733,33 @@
   </si>
   <si>
     <t>08/14/2025</t>
+  </si>
+  <si>
+    <t>08/27/2025</t>
+  </si>
+  <si>
+    <t>Daureath St</t>
+  </si>
+  <si>
+    <t>42.3232051, -71.0805673</t>
+  </si>
+  <si>
+    <t>Other Dudley Commons</t>
+  </si>
+  <si>
+    <t>42.3267352, -71.0755563</t>
+  </si>
+  <si>
+    <t>Lauydon St Farm</t>
+  </si>
+  <si>
+    <t>42.3243402, -71.0723826</t>
+  </si>
+  <si>
+    <t>Moreland St, Howes Playground</t>
+  </si>
+  <si>
+    <t>42.3240841, -71.0793291</t>
   </si>
 </sst>
 </file>
@@ -818,7 +845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -831,6 +858,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2892,19 +2922,19 @@
       <c r="N27" t="s">
         <v>168</v>
       </c>
-      <c r="O27" s="2">
+      <c r="O27" s="12">
         <v>45874</v>
       </c>
-      <c r="P27" s="2" t="s">
+      <c r="P27" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="Q27" s="5">
+      <c r="Q27" s="13">
         <v>0.4909722222222222</v>
       </c>
-      <c r="R27" t="s">
+      <c r="R27" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="S27" t="s">
+      <c r="S27" s="9" t="s">
         <v>149</v>
       </c>
       <c r="W27" s="2"/>
@@ -2950,7 +2980,24 @@
       <c r="M28" s="2">
         <v>45793</v>
       </c>
-      <c r="O28" s="2"/>
+      <c r="N28" t="s">
+        <v>168</v>
+      </c>
+      <c r="O28" s="12">
+        <v>45874</v>
+      </c>
+      <c r="P28" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q28" s="14">
+        <v>0.68472222222222223</v>
+      </c>
+      <c r="R28" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="S28" s="11" t="s">
+        <v>234</v>
+      </c>
       <c r="U28" t="s">
         <v>214</v>
       </c>
@@ -2997,7 +3044,24 @@
       <c r="M29" s="2">
         <v>45793</v>
       </c>
-      <c r="O29" s="2"/>
+      <c r="N29" t="s">
+        <v>168</v>
+      </c>
+      <c r="O29" s="12">
+        <v>45874</v>
+      </c>
+      <c r="P29" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q29" s="14">
+        <v>0.63749999999999996</v>
+      </c>
+      <c r="R29" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="S29" s="11" t="s">
+        <v>236</v>
+      </c>
       <c r="W29" s="2"/>
       <c r="X29" s="2"/>
     </row>
@@ -3041,7 +3105,24 @@
       <c r="M30" s="2">
         <v>45793</v>
       </c>
-      <c r="O30" s="2"/>
+      <c r="N30" t="s">
+        <v>168</v>
+      </c>
+      <c r="O30" s="12">
+        <v>45874</v>
+      </c>
+      <c r="P30" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q30" s="14">
+        <v>0.62222222222222223</v>
+      </c>
+      <c r="R30" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="S30" s="11" t="s">
+        <v>238</v>
+      </c>
       <c r="W30" s="2"/>
       <c r="X30" s="2"/>
     </row>
@@ -3085,7 +3166,16 @@
       <c r="M31" s="2">
         <v>45793</v>
       </c>
-      <c r="O31" s="2"/>
+      <c r="N31" t="s">
+        <v>168</v>
+      </c>
+      <c r="O31" s="12">
+        <v>45874</v>
+      </c>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
+      <c r="S31" s="9"/>
       <c r="W31" s="2"/>
       <c r="X31" s="2"/>
     </row>
@@ -3129,7 +3219,24 @@
       <c r="M32" s="2">
         <v>45793</v>
       </c>
-      <c r="O32" s="2"/>
+      <c r="N32" t="s">
+        <v>168</v>
+      </c>
+      <c r="O32" s="12">
+        <v>45874</v>
+      </c>
+      <c r="P32" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="Q32" s="14">
+        <v>0.66041666666666665</v>
+      </c>
+      <c r="R32" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="S32" s="11" t="s">
+        <v>240</v>
+      </c>
       <c r="W32" s="2"/>
       <c r="X32" s="2"/>
     </row>

</xml_diff>

<commit_message>
The changes made during the Box test
Change some batteries for RTC and changed one T sensor
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE140A8-C0BF-A44C-B3EF-4FA3AEE5ACD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91C4256-DD87-2249-87C4-6A8A58DF0289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1040" yWindow="1240" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="243">
   <si>
     <t>Box Number</t>
   </si>
@@ -760,6 +760,12 @@
   </si>
   <si>
     <t>42.3240841, -71.0793291</t>
+  </si>
+  <si>
+    <t>Changed the RTC battery on 8/27/2025</t>
+  </si>
+  <si>
+    <t>T sensor Power cable reversed and changed T sensor</t>
   </si>
 </sst>
 </file>
@@ -3630,6 +3636,9 @@
         <v>45793</v>
       </c>
       <c r="O41" s="2"/>
+      <c r="U41" t="s">
+        <v>241</v>
+      </c>
       <c r="W41" s="2"/>
       <c r="X41" s="2"/>
     </row>
@@ -3672,6 +3681,9 @@
         <v>45793</v>
       </c>
       <c r="O42" s="2"/>
+      <c r="U42" t="s">
+        <v>242</v>
+      </c>
       <c r="W42" s="2"/>
       <c r="X42" s="2"/>
     </row>
@@ -4050,6 +4062,9 @@
         <v>45793</v>
       </c>
       <c r="O51" s="2"/>
+      <c r="U51" t="s">
+        <v>241</v>
+      </c>
       <c r="W51" s="2"/>
       <c r="X51" s="2"/>
     </row>

</xml_diff>

<commit_message>
Added Cellular Module Serial Number
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A91C4256-DD87-2249-87C4-6A8A58DF0289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F544C5-F917-454A-B283-AEFBBDF29B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="1240" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="250">
   <si>
     <t>Box Number</t>
   </si>
@@ -766,6 +766,27 @@
   </si>
   <si>
     <t>T sensor Power cable reversed and changed T sensor</t>
+  </si>
+  <si>
+    <t>Cellular Module Serial No.</t>
+  </si>
+  <si>
+    <t>P044AD309WDG7M5</t>
+  </si>
+  <si>
+    <t>P044AD309APJYTL</t>
+  </si>
+  <si>
+    <t>P044AD309PCJ3VH</t>
+  </si>
+  <si>
+    <t>P044AD3096C3JSA</t>
+  </si>
+  <si>
+    <t>P044AD309WMGY4X</t>
+  </si>
+  <si>
+    <t>P044AD309JYD9NM</t>
   </si>
 </sst>
 </file>
@@ -1201,7 +1222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:AC56"/>
+  <dimension ref="A1:AD56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -1211,23 +1232,23 @@
     <col min="5" max="5" width="12.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="8" width="11.1640625" customWidth="1"/>
     <col min="9" max="9" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="26.33203125" customWidth="1"/>
-    <col min="11" max="11" width="19.5" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="25.6640625" customWidth="1"/>
-    <col min="13" max="13" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="23.83203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.5" customWidth="1"/>
-    <col min="18" max="18" width="28" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="22" customWidth="1"/>
-    <col min="26" max="26" width="22.5" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="51.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="11" width="26.33203125" customWidth="1"/>
+    <col min="12" max="12" width="19.5" style="4" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="25.6640625" customWidth="1"/>
+    <col min="14" max="14" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="23.83203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.5" customWidth="1"/>
+    <col min="19" max="19" width="28" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22" customWidth="1"/>
+    <col min="27" max="27" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="51.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1258,45 +1279,48 @@
       <c r="J1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>191</v>
       </c>
-      <c r="V1" s="1"/>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
-      <c r="Z1" s="1"/>
-    </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y1" s="1"/>
+      <c r="AA1" s="1"/>
+    </row>
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -1325,37 +1349,40 @@
       <c r="J2" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" t="s">
+        <v>244</v>
+      </c>
+      <c r="L2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>172</v>
       </c>
-      <c r="M2" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="N2" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O2" t="s">
         <v>168</v>
       </c>
-      <c r="O2" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P2" t="s">
+      <c r="P2" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q2" t="s">
         <v>114</v>
       </c>
-      <c r="Q2" s="5">
+      <c r="R2" s="5">
         <v>0.55347222222222225</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>115</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>116</v>
       </c>
-      <c r="W2" s="2"/>
       <c r="X2" s="2"/>
-    </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y2" s="2"/>
+    </row>
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
@@ -1384,37 +1411,40 @@
       <c r="J3" t="s">
         <v>5</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" t="s">
+        <v>245</v>
+      </c>
+      <c r="L3" s="4" t="s">
         <v>56</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>172</v>
       </c>
-      <c r="M3" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N3" t="s">
+      <c r="N3" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O3" t="s">
         <v>168</v>
       </c>
-      <c r="O3" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P3" t="s">
+      <c r="P3" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q3" t="s">
         <v>150</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="R3" s="5">
         <v>0.47499999999999998</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>156</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>155</v>
       </c>
-      <c r="W3" s="2"/>
       <c r="X3" s="2"/>
-    </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y3" s="2"/>
+    </row>
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>57</v>
       </c>
@@ -1443,43 +1473,46 @@
       <c r="J4" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" t="s">
+        <v>246</v>
+      </c>
+      <c r="L4" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>172</v>
       </c>
-      <c r="M4" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="N4" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O4" t="s">
         <v>168</v>
       </c>
-      <c r="O4" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P4" t="s">
+      <c r="P4" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q4" t="s">
         <v>117</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="R4" s="5">
         <v>0.65416666666666667</v>
       </c>
-      <c r="R4" t="s">
+      <c r="S4" t="s">
         <v>121</v>
       </c>
-      <c r="S4" t="s">
+      <c r="T4" t="s">
         <v>120</v>
       </c>
-      <c r="W4" s="2"/>
       <c r="X4" s="2"/>
-      <c r="AB4" s="1" t="s">
+      <c r="Y4" s="2"/>
+      <c r="AC4" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="AC4" t="s">
+      <c r="AD4" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>58</v>
       </c>
@@ -1508,43 +1541,46 @@
       <c r="J5" t="s">
         <v>7</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" t="s">
+        <v>247</v>
+      </c>
+      <c r="L5" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>172</v>
       </c>
-      <c r="M5" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N5" t="s">
+      <c r="N5" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O5" t="s">
         <v>168</v>
       </c>
-      <c r="O5" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P5" t="s">
+      <c r="P5" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q5" t="s">
         <v>117</v>
       </c>
-      <c r="Q5" s="5">
+      <c r="R5" s="5">
         <v>0.6166666666666667</v>
       </c>
-      <c r="R5" t="s">
+      <c r="S5" t="s">
         <v>124</v>
       </c>
-      <c r="S5" t="s">
+      <c r="T5" t="s">
         <v>125</v>
       </c>
-      <c r="W5" s="2"/>
       <c r="X5" s="2"/>
-      <c r="AB5" s="1" t="s">
+      <c r="Y5" s="2"/>
+      <c r="AC5" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="AC5" t="s">
+      <c r="AD5" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>59</v>
       </c>
@@ -1573,43 +1609,46 @@
       <c r="J6" t="s">
         <v>8</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" t="s">
+        <v>248</v>
+      </c>
+      <c r="L6" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>172</v>
       </c>
-      <c r="M6" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N6" t="s">
+      <c r="N6" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O6" t="s">
         <v>168</v>
       </c>
-      <c r="O6" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P6" t="s">
+      <c r="P6" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q6" t="s">
         <v>117</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="R6" s="5">
         <v>0.63541666666666663</v>
       </c>
-      <c r="R6" t="s">
+      <c r="S6" t="s">
         <v>118</v>
       </c>
-      <c r="S6" t="s">
+      <c r="T6" t="s">
         <v>119</v>
       </c>
-      <c r="W6" s="2"/>
       <c r="X6" s="2"/>
-      <c r="AB6" s="1" t="s">
+      <c r="Y6" s="2"/>
+      <c r="AC6" s="1" t="s">
         <v>179</v>
       </c>
-      <c r="AC6" t="s">
+      <c r="AD6" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>60</v>
       </c>
@@ -1638,43 +1677,46 @@
       <c r="J7" t="s">
         <v>9</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" t="s">
+        <v>249</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>172</v>
       </c>
-      <c r="M7" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N7" t="s">
+      <c r="N7" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O7" t="s">
         <v>168</v>
       </c>
-      <c r="O7" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P7" t="s">
+      <c r="P7" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q7" t="s">
         <v>117</v>
       </c>
-      <c r="Q7" s="5">
+      <c r="R7" s="5">
         <v>0.67777777777777781</v>
       </c>
-      <c r="R7" t="s">
+      <c r="S7" t="s">
         <v>122</v>
       </c>
-      <c r="S7" t="s">
+      <c r="T7" t="s">
         <v>123</v>
       </c>
-      <c r="W7" s="2"/>
       <c r="X7" s="2"/>
-      <c r="AB7" s="1" t="s">
+      <c r="Y7" s="2"/>
+      <c r="AC7" s="1" t="s">
         <v>175</v>
       </c>
-      <c r="AC7" t="s">
+      <c r="AD7" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>61</v>
       </c>
@@ -1703,43 +1745,43 @@
       <c r="J8" t="s">
         <v>10</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="L8" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>172</v>
       </c>
-      <c r="M8" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="N8" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O8" t="s">
         <v>168</v>
       </c>
-      <c r="O8" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P8" t="s">
+      <c r="P8" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q8" t="s">
         <v>126</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="R8" s="5">
         <v>0.44166666666666665</v>
       </c>
-      <c r="R8" t="s">
+      <c r="S8" t="s">
         <v>127</v>
       </c>
-      <c r="S8" t="s">
+      <c r="T8" t="s">
         <v>128</v>
       </c>
-      <c r="W8" s="2"/>
       <c r="X8" s="2"/>
-      <c r="AB8" s="1" t="s">
+      <c r="Y8" s="2"/>
+      <c r="AC8" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AD8" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>62</v>
       </c>
@@ -1768,43 +1810,43 @@
       <c r="J9" t="s">
         <v>11</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="L9" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>172</v>
       </c>
-      <c r="M9" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N9" t="s">
+      <c r="N9" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O9" t="s">
         <v>168</v>
       </c>
-      <c r="O9" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P9" t="s">
+      <c r="P9" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q9" t="s">
         <v>126</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="R9" s="5">
         <v>0.45416666666666666</v>
       </c>
-      <c r="R9" t="s">
+      <c r="S9" t="s">
         <v>129</v>
       </c>
-      <c r="S9" t="s">
+      <c r="T9" t="s">
         <v>130</v>
       </c>
-      <c r="W9" s="2"/>
       <c r="X9" s="2"/>
-      <c r="AB9" s="1" t="s">
+      <c r="Y9" s="2"/>
+      <c r="AC9" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AD9" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>63</v>
       </c>
@@ -1833,49 +1875,49 @@
       <c r="J10" t="s">
         <v>12</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="L10" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>172</v>
       </c>
-      <c r="M10" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N10" t="s">
+      <c r="N10" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O10" t="s">
         <v>168</v>
       </c>
-      <c r="O10" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P10" t="s">
+      <c r="P10" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q10" t="s">
         <v>150</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="R10" s="5">
         <v>0.44444444444444442</v>
       </c>
-      <c r="R10" t="s">
+      <c r="S10" t="s">
         <v>148</v>
       </c>
-      <c r="S10" t="s">
+      <c r="T10" t="s">
         <v>149</v>
       </c>
-      <c r="T10" s="10">
+      <c r="U10" s="10">
         <v>45968</v>
       </c>
-      <c r="U10" t="s">
+      <c r="V10" t="s">
         <v>215</v>
       </c>
-      <c r="W10" s="2"/>
       <c r="X10" s="2"/>
-      <c r="AB10" s="1" t="s">
+      <c r="Y10" s="2"/>
+      <c r="AC10" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AD10" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>64</v>
       </c>
@@ -1904,43 +1946,43 @@
       <c r="J11" t="s">
         <v>13</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="L11" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>172</v>
       </c>
-      <c r="M11" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N11" t="s">
+      <c r="N11" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O11" t="s">
         <v>168</v>
       </c>
-      <c r="O11" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P11" t="s">
+      <c r="P11" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q11" t="s">
         <v>126</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="R11" s="5">
         <v>0.47569444444444442</v>
       </c>
-      <c r="R11" t="s">
+      <c r="S11" t="s">
         <v>132</v>
       </c>
-      <c r="S11" t="s">
+      <c r="T11" t="s">
         <v>133</v>
       </c>
-      <c r="W11" s="2"/>
       <c r="X11" s="2"/>
-      <c r="AB11" s="1" t="s">
+      <c r="Y11" s="2"/>
+      <c r="AC11" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AD11" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>65</v>
       </c>
@@ -1969,43 +2011,43 @@
       <c r="J12" t="s">
         <v>14</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="L12" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>172</v>
       </c>
-      <c r="M12" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N12" t="s">
+      <c r="N12" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O12" t="s">
         <v>168</v>
       </c>
-      <c r="O12" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P12" t="s">
+      <c r="P12" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q12" t="s">
         <v>126</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="R12" s="5">
         <v>0.55347222222222225</v>
       </c>
-      <c r="R12" t="s">
+      <c r="S12" t="s">
         <v>140</v>
       </c>
-      <c r="S12" t="s">
+      <c r="T12" t="s">
         <v>141</v>
       </c>
-      <c r="W12" s="2"/>
       <c r="X12" s="2"/>
-      <c r="AB12" s="1" t="s">
+      <c r="Y12" s="2"/>
+      <c r="AC12" s="1" t="s">
         <v>185</v>
       </c>
-      <c r="AC12" t="s">
+      <c r="AD12" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
@@ -2034,43 +2076,43 @@
       <c r="J13" t="s">
         <v>15</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="L13" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>172</v>
       </c>
-      <c r="M13" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N13" t="s">
+      <c r="N13" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O13" t="s">
         <v>168</v>
       </c>
-      <c r="O13" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P13" t="s">
+      <c r="P13" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q13" t="s">
         <v>126</v>
       </c>
-      <c r="Q13" s="5">
+      <c r="R13" s="5">
         <v>0.4861111111111111</v>
       </c>
-      <c r="R13" t="s">
+      <c r="S13" t="s">
         <v>134</v>
       </c>
-      <c r="S13" t="s">
+      <c r="T13" t="s">
         <v>135</v>
       </c>
-      <c r="W13" s="2"/>
       <c r="X13" s="2"/>
-      <c r="AB13" s="1" t="s">
+      <c r="Y13" s="2"/>
+      <c r="AC13" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="AC13" t="s">
+      <c r="AD13" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>67</v>
       </c>
@@ -2099,43 +2141,43 @@
       <c r="J14" t="s">
         <v>110</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="L14" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>172</v>
       </c>
-      <c r="M14" s="2">
+      <c r="N14" s="2">
         <v>45826</v>
       </c>
-      <c r="N14" t="s">
+      <c r="O14" t="s">
         <v>168</v>
       </c>
-      <c r="O14" s="2">
+      <c r="P14" s="2">
         <v>45826</v>
       </c>
-      <c r="P14" t="s">
+      <c r="Q14" t="s">
         <v>126</v>
       </c>
-      <c r="Q14" s="5">
+      <c r="R14" s="5">
         <v>0.50347222222222221</v>
       </c>
-      <c r="R14" t="s">
+      <c r="S14" t="s">
         <v>137</v>
       </c>
-      <c r="S14" t="s">
+      <c r="T14" t="s">
         <v>136</v>
       </c>
-      <c r="W14" s="2"/>
       <c r="X14" s="2"/>
-      <c r="AB14" s="3" t="s">
+      <c r="Y14" s="2"/>
+      <c r="AC14" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="AC14" t="s">
+      <c r="AD14" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>68</v>
       </c>
@@ -2164,34 +2206,34 @@
       <c r="J15" t="s">
         <v>16</v>
       </c>
-      <c r="K15" s="4" t="s">
+      <c r="L15" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>172</v>
       </c>
-      <c r="M15" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N15" t="s">
+      <c r="N15" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O15" t="s">
         <v>168</v>
       </c>
-      <c r="O15" s="2">
-        <v>45793</v>
-      </c>
-      <c r="U15" t="s">
+      <c r="P15" s="2">
+        <v>45793</v>
+      </c>
+      <c r="V15" t="s">
         <v>192</v>
       </c>
-      <c r="W15" s="2"/>
       <c r="X15" s="2"/>
-      <c r="AB15" s="1" t="s">
+      <c r="Y15" s="2"/>
+      <c r="AC15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="AC15" t="s">
+      <c r="AD15" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
@@ -2220,43 +2262,43 @@
       <c r="J16" t="s">
         <v>17</v>
       </c>
-      <c r="K16" s="4" t="s">
+      <c r="L16" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>172</v>
       </c>
-      <c r="M16" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N16" t="s">
+      <c r="N16" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O16" t="s">
         <v>168</v>
       </c>
-      <c r="O16" s="2">
-        <v>45793</v>
-      </c>
       <c r="P16" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q16" s="2">
         <v>45785</v>
       </c>
-      <c r="Q16" s="5">
+      <c r="R16" s="5">
         <v>0.48055555555555557</v>
       </c>
-      <c r="R16" t="s">
+      <c r="S16" t="s">
         <v>226</v>
       </c>
-      <c r="S16" t="s">
+      <c r="T16" t="s">
         <v>227</v>
       </c>
-      <c r="W16" s="2"/>
       <c r="X16" s="2"/>
-      <c r="AB16" s="1" t="s">
+      <c r="Y16" s="2"/>
+      <c r="AC16" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="AC16" t="s">
+      <c r="AD16" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -2285,43 +2327,43 @@
       <c r="J17" t="s">
         <v>18</v>
       </c>
-      <c r="K17" s="4" t="s">
+      <c r="L17" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>172</v>
       </c>
-      <c r="M17" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N17" t="s">
+      <c r="N17" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O17" t="s">
         <v>168</v>
       </c>
-      <c r="O17" s="2">
-        <v>45793</v>
-      </c>
       <c r="P17" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q17" s="2">
         <v>45785</v>
       </c>
-      <c r="Q17" s="5">
+      <c r="R17" s="5">
         <v>0.49722222222222223</v>
       </c>
-      <c r="R17" t="s">
+      <c r="S17" t="s">
         <v>228</v>
       </c>
-      <c r="S17" t="s">
+      <c r="T17" t="s">
         <v>229</v>
       </c>
-      <c r="W17" s="2"/>
       <c r="X17" s="2"/>
-      <c r="AB17" s="1" t="s">
+      <c r="Y17" s="2"/>
+      <c r="AC17" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="AC17" t="s">
+      <c r="AD17" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>71</v>
       </c>
@@ -2350,46 +2392,46 @@
       <c r="J18" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="4" t="s">
+      <c r="L18" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>172</v>
       </c>
-      <c r="M18" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N18" t="s">
+      <c r="N18" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O18" t="s">
         <v>168</v>
       </c>
-      <c r="O18" s="2">
-        <v>45793</v>
-      </c>
       <c r="P18" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q18" s="2">
         <v>45785</v>
       </c>
-      <c r="Q18" s="5">
+      <c r="R18" s="5">
         <v>0.51736111111111116</v>
       </c>
-      <c r="R18" t="s">
+      <c r="S18" t="s">
         <v>224</v>
       </c>
-      <c r="S18" t="s">
+      <c r="T18" t="s">
         <v>225</v>
       </c>
-      <c r="U18" t="s">
+      <c r="V18" t="s">
         <v>192</v>
       </c>
-      <c r="W18" s="2"/>
       <c r="X18" s="2"/>
-      <c r="AB18" s="1" t="s">
+      <c r="Y18" s="2"/>
+      <c r="AC18" s="1" t="s">
         <v>171</v>
       </c>
-      <c r="AC18" t="s">
+      <c r="AD18" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>72</v>
       </c>
@@ -2418,43 +2460,43 @@
       <c r="J19" t="s">
         <v>20</v>
       </c>
-      <c r="K19" s="4" t="s">
+      <c r="L19" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>172</v>
       </c>
-      <c r="M19" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N19" t="s">
+      <c r="N19" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O19" t="s">
         <v>168</v>
       </c>
-      <c r="O19" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P19" t="s">
+      <c r="P19" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q19" t="s">
         <v>150</v>
       </c>
-      <c r="Q19" s="5">
+      <c r="R19" s="5">
         <v>0.40625</v>
       </c>
-      <c r="R19" t="s">
+      <c r="S19" t="s">
         <v>157</v>
       </c>
-      <c r="S19" t="s">
+      <c r="T19" t="s">
         <v>158</v>
       </c>
-      <c r="W19" s="2"/>
       <c r="X19" s="2"/>
-      <c r="AB19" s="1" t="s">
+      <c r="Y19" s="2"/>
+      <c r="AC19" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="AC19" t="s">
+      <c r="AD19" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>73</v>
       </c>
@@ -2483,43 +2525,43 @@
       <c r="J20" t="s">
         <v>21</v>
       </c>
-      <c r="K20" s="4" t="s">
+      <c r="L20" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>172</v>
       </c>
-      <c r="M20" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N20" t="s">
+      <c r="N20" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O20" t="s">
         <v>168</v>
       </c>
-      <c r="O20" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P20" t="s">
+      <c r="P20" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q20" t="s">
         <v>126</v>
       </c>
-      <c r="Q20" s="5">
+      <c r="R20" s="5">
         <v>0.51597222222222228</v>
       </c>
-      <c r="R20" t="s">
+      <c r="S20" t="s">
         <v>138</v>
       </c>
-      <c r="S20" t="s">
+      <c r="T20" t="s">
         <v>139</v>
       </c>
-      <c r="W20" s="2"/>
       <c r="X20" s="2"/>
-      <c r="AB20" s="1" t="s">
+      <c r="Y20" s="2"/>
+      <c r="AC20" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="AC20" t="s">
+      <c r="AD20" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>74</v>
       </c>
@@ -2548,43 +2590,43 @@
       <c r="J21" t="s">
         <v>22</v>
       </c>
-      <c r="K21" s="4" t="s">
+      <c r="L21" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>172</v>
       </c>
-      <c r="M21" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N21" t="s">
+      <c r="N21" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O21" t="s">
         <v>168</v>
       </c>
-      <c r="O21" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P21" t="s">
+      <c r="P21" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q21" t="s">
         <v>126</v>
       </c>
-      <c r="Q21" s="5">
+      <c r="R21" s="5">
         <v>0.60972222222222228</v>
       </c>
-      <c r="R21" t="s">
+      <c r="S21" t="s">
         <v>146</v>
       </c>
-      <c r="S21" t="s">
+      <c r="T21" t="s">
         <v>147</v>
       </c>
-      <c r="W21" s="2"/>
       <c r="X21" s="2"/>
-      <c r="AB21" s="1" t="s">
+      <c r="Y21" s="2"/>
+      <c r="AC21" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="AC21" t="s">
+      <c r="AD21" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>75</v>
       </c>
@@ -2613,43 +2655,43 @@
       <c r="J22" t="s">
         <v>23</v>
       </c>
-      <c r="K22" s="4" t="s">
+      <c r="L22" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="L22" t="s">
+      <c r="M22" t="s">
         <v>172</v>
       </c>
-      <c r="M22" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N22" t="s">
+      <c r="N22" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O22" t="s">
         <v>168</v>
       </c>
-      <c r="O22" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P22" t="s">
+      <c r="P22" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q22" t="s">
         <v>150</v>
       </c>
-      <c r="Q22" s="5">
+      <c r="R22" s="5">
         <v>0.45763888888888887</v>
       </c>
-      <c r="R22" t="s">
+      <c r="S22" t="s">
         <v>153</v>
       </c>
-      <c r="S22" t="s">
+      <c r="T22" t="s">
         <v>154</v>
       </c>
-      <c r="W22" s="2"/>
       <c r="X22" s="2"/>
-      <c r="AB22" s="1" t="s">
+      <c r="Y22" s="2"/>
+      <c r="AC22" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="AC22" t="s">
+      <c r="AD22" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="23" spans="1:29" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>76</v>
       </c>
@@ -2678,37 +2720,37 @@
       <c r="J23" t="s">
         <v>24</v>
       </c>
-      <c r="K23" s="4" t="s">
+      <c r="L23" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>172</v>
       </c>
-      <c r="M23" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N23" t="s">
+      <c r="N23" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O23" t="s">
         <v>168</v>
       </c>
-      <c r="O23" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P23" t="s">
+      <c r="P23" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q23" t="s">
         <v>150</v>
       </c>
-      <c r="Q23" s="5">
+      <c r="R23" s="5">
         <v>0.42499999999999999</v>
       </c>
-      <c r="R23" t="s">
+      <c r="S23" t="s">
         <v>151</v>
       </c>
-      <c r="S23" t="s">
+      <c r="T23" t="s">
         <v>152</v>
       </c>
-      <c r="W23" s="2"/>
       <c r="X23" s="2"/>
-    </row>
-    <row r="24" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y23" s="2"/>
+    </row>
+    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>77</v>
       </c>
@@ -2737,37 +2779,37 @@
       <c r="J24" t="s">
         <v>25</v>
       </c>
-      <c r="K24" s="4" t="s">
+      <c r="L24" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>172</v>
       </c>
-      <c r="M24" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N24" t="s">
+      <c r="N24" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O24" t="s">
         <v>168</v>
       </c>
-      <c r="O24" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P24" t="s">
+      <c r="P24" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q24" t="s">
         <v>126</v>
       </c>
-      <c r="Q24" s="5">
+      <c r="R24" s="5">
         <v>0.56458333333333333</v>
       </c>
-      <c r="R24" t="s">
+      <c r="S24" t="s">
         <v>142</v>
       </c>
-      <c r="S24" t="s">
+      <c r="T24" t="s">
         <v>143</v>
       </c>
-      <c r="W24" s="2"/>
       <c r="X24" s="2"/>
-    </row>
-    <row r="25" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y24" s="2"/>
+    </row>
+    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>78</v>
       </c>
@@ -2796,37 +2838,37 @@
       <c r="J25" t="s">
         <v>26</v>
       </c>
-      <c r="K25" s="4" t="s">
+      <c r="L25" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="L25" t="s">
+      <c r="M25" t="s">
         <v>172</v>
       </c>
-      <c r="M25" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N25" t="s">
+      <c r="N25" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O25" t="s">
         <v>168</v>
       </c>
-      <c r="O25" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P25" t="s">
+      <c r="P25" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q25" t="s">
         <v>187</v>
       </c>
-      <c r="Q25" s="5">
+      <c r="R25" s="5">
         <v>0.66736111111111107</v>
       </c>
-      <c r="R25" t="s">
+      <c r="S25" t="s">
         <v>188</v>
       </c>
-      <c r="S25" t="s">
+      <c r="T25" t="s">
         <v>189</v>
       </c>
-      <c r="W25" s="2"/>
       <c r="X25" s="2"/>
-    </row>
-    <row r="26" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y25" s="2"/>
+    </row>
+    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>79</v>
       </c>
@@ -2855,37 +2897,37 @@
       <c r="J26" t="s">
         <v>27</v>
       </c>
-      <c r="K26" s="4" t="s">
+      <c r="L26" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="L26" t="s">
+      <c r="M26" t="s">
         <v>172</v>
       </c>
-      <c r="M26" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N26" t="s">
+      <c r="N26" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O26" t="s">
         <v>168</v>
       </c>
-      <c r="O26" s="2">
-        <v>45793</v>
-      </c>
-      <c r="P26" t="s">
+      <c r="P26" s="2">
+        <v>45793</v>
+      </c>
+      <c r="Q26" t="s">
         <v>126</v>
       </c>
-      <c r="Q26" s="5">
+      <c r="R26" s="5">
         <v>0.58750000000000002</v>
       </c>
-      <c r="R26" t="s">
+      <c r="S26" t="s">
         <v>145</v>
       </c>
-      <c r="S26" t="s">
+      <c r="T26" t="s">
         <v>144</v>
       </c>
-      <c r="W26" s="2"/>
       <c r="X26" s="2"/>
-    </row>
-    <row r="27" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y26" s="2"/>
+    </row>
+    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
@@ -2916,37 +2958,37 @@
       <c r="J27" t="s">
         <v>28</v>
       </c>
-      <c r="K27" s="4" t="s">
+      <c r="L27" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="L27" t="s">
+      <c r="M27" t="s">
         <v>172</v>
       </c>
-      <c r="M27" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N27" t="s">
+      <c r="N27" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O27" t="s">
         <v>168</v>
       </c>
-      <c r="O27" s="12">
+      <c r="P27" s="12">
         <v>45874</v>
       </c>
-      <c r="P27" s="11" t="s">
+      <c r="Q27" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="Q27" s="13">
+      <c r="R27" s="13">
         <v>0.4909722222222222</v>
       </c>
-      <c r="R27" s="9" t="s">
+      <c r="S27" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="S27" s="9" t="s">
+      <c r="T27" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="W27" s="2"/>
       <c r="X27" s="2"/>
-    </row>
-    <row r="28" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y27" s="2"/>
+    </row>
+    <row r="28" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>81</v>
       </c>
@@ -2977,40 +3019,40 @@
       <c r="J28" t="s">
         <v>54</v>
       </c>
-      <c r="K28" s="4" t="s">
+      <c r="L28" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="L28" t="s">
+      <c r="M28" t="s">
         <v>172</v>
       </c>
-      <c r="M28" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N28" t="s">
+      <c r="N28" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O28" t="s">
         <v>168</v>
       </c>
-      <c r="O28" s="12">
+      <c r="P28" s="12">
         <v>45874</v>
       </c>
-      <c r="P28" s="11" t="s">
+      <c r="Q28" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="Q28" s="14">
+      <c r="R28" s="14">
         <v>0.68472222222222223</v>
       </c>
-      <c r="R28" s="11" t="s">
+      <c r="S28" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="S28" s="11" t="s">
+      <c r="T28" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="U28" t="s">
+      <c r="V28" t="s">
         <v>214</v>
       </c>
-      <c r="W28" s="2"/>
       <c r="X28" s="2"/>
-    </row>
-    <row r="29" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y28" s="2"/>
+    </row>
+    <row r="29" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>82</v>
       </c>
@@ -3041,37 +3083,37 @@
       <c r="J29" t="s">
         <v>29</v>
       </c>
-      <c r="K29" s="4" t="s">
+      <c r="L29" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>172</v>
       </c>
-      <c r="M29" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N29" t="s">
+      <c r="N29" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O29" t="s">
         <v>168</v>
       </c>
-      <c r="O29" s="12">
+      <c r="P29" s="12">
         <v>45874</v>
       </c>
-      <c r="P29" s="11" t="s">
+      <c r="Q29" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="Q29" s="14">
+      <c r="R29" s="14">
         <v>0.63749999999999996</v>
       </c>
-      <c r="R29" s="11" t="s">
+      <c r="S29" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="S29" s="11" t="s">
+      <c r="T29" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="W29" s="2"/>
       <c r="X29" s="2"/>
-    </row>
-    <row r="30" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y29" s="2"/>
+    </row>
+    <row r="30" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>83</v>
       </c>
@@ -3102,37 +3144,37 @@
       <c r="J30" t="s">
         <v>30</v>
       </c>
-      <c r="K30" s="4" t="s">
+      <c r="L30" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>172</v>
       </c>
-      <c r="M30" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N30" t="s">
+      <c r="N30" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O30" t="s">
         <v>168</v>
       </c>
-      <c r="O30" s="12">
+      <c r="P30" s="12">
         <v>45874</v>
       </c>
-      <c r="P30" s="11" t="s">
+      <c r="Q30" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="Q30" s="14">
+      <c r="R30" s="14">
         <v>0.62222222222222223</v>
       </c>
-      <c r="R30" s="11" t="s">
+      <c r="S30" s="11" t="s">
         <v>237</v>
       </c>
-      <c r="S30" s="11" t="s">
+      <c r="T30" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="W30" s="2"/>
       <c r="X30" s="2"/>
-    </row>
-    <row r="31" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y30" s="2"/>
+    </row>
+    <row r="31" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
@@ -3163,29 +3205,29 @@
       <c r="J31" t="s">
         <v>31</v>
       </c>
-      <c r="K31" s="4" t="s">
+      <c r="L31" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="L31" t="s">
+      <c r="M31" t="s">
         <v>172</v>
       </c>
-      <c r="M31" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N31" t="s">
+      <c r="N31" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O31" t="s">
         <v>168</v>
       </c>
-      <c r="O31" s="12">
+      <c r="P31" s="12">
         <v>45874</v>
       </c>
-      <c r="P31" s="9"/>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
       <c r="S31" s="9"/>
-      <c r="W31" s="2"/>
+      <c r="T31" s="9"/>
       <c r="X31" s="2"/>
-    </row>
-    <row r="32" spans="1:29" x14ac:dyDescent="0.2">
+      <c r="Y31" s="2"/>
+    </row>
+    <row r="32" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>85</v>
       </c>
@@ -3216,37 +3258,37 @@
       <c r="J32" t="s">
         <v>32</v>
       </c>
-      <c r="K32" s="4" t="s">
+      <c r="L32" s="4" t="s">
         <v>85</v>
       </c>
-      <c r="L32" t="s">
+      <c r="M32" t="s">
         <v>172</v>
       </c>
-      <c r="M32" s="2">
-        <v>45793</v>
-      </c>
-      <c r="N32" t="s">
+      <c r="N32" s="2">
+        <v>45793</v>
+      </c>
+      <c r="O32" t="s">
         <v>168</v>
       </c>
-      <c r="O32" s="12">
+      <c r="P32" s="12">
         <v>45874</v>
       </c>
-      <c r="P32" s="11" t="s">
+      <c r="Q32" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="Q32" s="14">
+      <c r="R32" s="14">
         <v>0.66041666666666665</v>
       </c>
-      <c r="R32" s="11" t="s">
+      <c r="S32" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="S32" s="11" t="s">
+      <c r="T32" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="W32" s="2"/>
       <c r="X32" s="2"/>
-    </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y32" s="2"/>
+    </row>
+    <row r="33" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>86</v>
       </c>
@@ -3277,20 +3319,20 @@
       <c r="J33" t="s">
         <v>33</v>
       </c>
-      <c r="K33" s="4" t="s">
+      <c r="L33" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="L33" t="s">
+      <c r="M33" t="s">
         <v>172</v>
       </c>
-      <c r="M33" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O33" s="2"/>
-      <c r="W33" s="2"/>
+      <c r="N33" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P33" s="2"/>
       <c r="X33" s="2"/>
-    </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y33" s="2"/>
+    </row>
+    <row r="34" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A34" s="4" t="s">
         <v>87</v>
       </c>
@@ -3321,20 +3363,20 @@
       <c r="J34" t="s">
         <v>53</v>
       </c>
-      <c r="K34" s="4" t="s">
+      <c r="L34" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="L34" t="s">
+      <c r="M34" t="s">
         <v>172</v>
       </c>
-      <c r="M34" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O34" s="2"/>
-      <c r="W34" s="2"/>
+      <c r="N34" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P34" s="2"/>
       <c r="X34" s="2"/>
-    </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y34" s="2"/>
+    </row>
+    <row r="35" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>88</v>
       </c>
@@ -3365,20 +3407,20 @@
       <c r="J35" t="s">
         <v>52</v>
       </c>
-      <c r="K35" s="4" t="s">
+      <c r="L35" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="L35" t="s">
+      <c r="M35" t="s">
         <v>172</v>
       </c>
-      <c r="M35" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O35" s="2"/>
-      <c r="W35" s="2"/>
+      <c r="N35" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P35" s="2"/>
       <c r="X35" s="2"/>
-    </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y35" s="2"/>
+    </row>
+    <row r="36" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>89</v>
       </c>
@@ -3409,20 +3451,20 @@
       <c r="J36" t="s">
         <v>34</v>
       </c>
-      <c r="K36" s="4" t="s">
+      <c r="L36" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="L36" t="s">
+      <c r="M36" t="s">
         <v>172</v>
       </c>
-      <c r="M36" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O36" s="2"/>
-      <c r="W36" s="2"/>
+      <c r="N36" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P36" s="2"/>
       <c r="X36" s="2"/>
-    </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y36" s="2"/>
+    </row>
+    <row r="37" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>90</v>
       </c>
@@ -3453,20 +3495,20 @@
       <c r="J37" t="s">
         <v>35</v>
       </c>
-      <c r="K37" s="4" t="s">
+      <c r="L37" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="L37" t="s">
+      <c r="M37" t="s">
         <v>172</v>
       </c>
-      <c r="M37" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O37" s="2"/>
-      <c r="W37" s="2"/>
+      <c r="N37" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P37" s="2"/>
       <c r="X37" s="2"/>
-    </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y37" s="2"/>
+    </row>
+    <row r="38" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>91</v>
       </c>
@@ -3497,23 +3539,23 @@
       <c r="J38" t="s">
         <v>36</v>
       </c>
-      <c r="K38" s="4" t="s">
+      <c r="L38" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="L38" t="s">
+      <c r="M38" t="s">
         <v>172</v>
       </c>
-      <c r="M38" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O38" s="2"/>
-      <c r="U38" t="s">
+      <c r="N38" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P38" s="2"/>
+      <c r="V38" t="s">
         <v>214</v>
       </c>
-      <c r="W38" s="2"/>
       <c r="X38" s="2"/>
-    </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y38" s="2"/>
+    </row>
+    <row r="39" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>92</v>
       </c>
@@ -3542,20 +3584,20 @@
       <c r="J39" t="s">
         <v>37</v>
       </c>
-      <c r="K39" s="4" t="s">
+      <c r="L39" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="L39" t="s">
+      <c r="M39" t="s">
         <v>172</v>
       </c>
-      <c r="M39" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O39" s="2"/>
-      <c r="W39" s="2"/>
+      <c r="N39" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P39" s="2"/>
       <c r="X39" s="2"/>
-    </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y39" s="2"/>
+    </row>
+    <row r="40" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>93</v>
       </c>
@@ -3584,20 +3626,20 @@
       <c r="J40" t="s">
         <v>38</v>
       </c>
-      <c r="K40" s="4" t="s">
+      <c r="L40" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="L40" t="s">
+      <c r="M40" t="s">
         <v>172</v>
       </c>
-      <c r="M40" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O40" s="2"/>
-      <c r="W40" s="2"/>
+      <c r="N40" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P40" s="2"/>
       <c r="X40" s="2"/>
-    </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y40" s="2"/>
+    </row>
+    <row r="41" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A41" s="4" t="s">
         <v>94</v>
       </c>
@@ -3626,23 +3668,23 @@
       <c r="J41" t="s">
         <v>39</v>
       </c>
-      <c r="K41" s="4" t="s">
+      <c r="L41" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="L41" t="s">
+      <c r="M41" t="s">
         <v>172</v>
       </c>
-      <c r="M41" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O41" s="2"/>
-      <c r="U41" t="s">
+      <c r="N41" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P41" s="2"/>
+      <c r="V41" t="s">
         <v>241</v>
       </c>
-      <c r="W41" s="2"/>
       <c r="X41" s="2"/>
-    </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y41" s="2"/>
+    </row>
+    <row r="42" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>95</v>
       </c>
@@ -3671,23 +3713,23 @@
       <c r="J42" t="s">
         <v>40</v>
       </c>
-      <c r="K42" s="4" t="s">
+      <c r="L42" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="L42" t="s">
+      <c r="M42" t="s">
         <v>172</v>
       </c>
-      <c r="M42" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O42" s="2"/>
-      <c r="U42" t="s">
+      <c r="N42" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P42" s="2"/>
+      <c r="V42" t="s">
         <v>242</v>
       </c>
-      <c r="W42" s="2"/>
       <c r="X42" s="2"/>
-    </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y42" s="2"/>
+    </row>
+    <row r="43" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>96</v>
       </c>
@@ -3716,20 +3758,20 @@
       <c r="J43" t="s">
         <v>41</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="L43" s="4" t="s">
         <v>96</v>
       </c>
-      <c r="L43" t="s">
+      <c r="M43" t="s">
         <v>172</v>
       </c>
-      <c r="M43" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O43" s="2"/>
-      <c r="W43" s="2"/>
+      <c r="N43" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P43" s="2"/>
       <c r="X43" s="2"/>
-    </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y43" s="2"/>
+    </row>
+    <row r="44" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>97</v>
       </c>
@@ -3758,20 +3800,20 @@
       <c r="J44" t="s">
         <v>42</v>
       </c>
-      <c r="K44" s="4" t="s">
+      <c r="L44" s="4" t="s">
         <v>97</v>
       </c>
-      <c r="L44" t="s">
+      <c r="M44" t="s">
         <v>172</v>
       </c>
-      <c r="M44" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O44" s="2"/>
-      <c r="W44" s="2"/>
+      <c r="N44" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P44" s="2"/>
       <c r="X44" s="2"/>
-    </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y44" s="2"/>
+    </row>
+    <row r="45" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A45" s="4" t="s">
         <v>98</v>
       </c>
@@ -3800,20 +3842,20 @@
       <c r="J45" t="s">
         <v>43</v>
       </c>
-      <c r="K45" s="4" t="s">
+      <c r="L45" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="L45" t="s">
+      <c r="M45" t="s">
         <v>172</v>
       </c>
-      <c r="M45" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O45" s="2"/>
-      <c r="W45" s="2"/>
+      <c r="N45" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P45" s="2"/>
       <c r="X45" s="2"/>
-    </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y45" s="2"/>
+    </row>
+    <row r="46" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A46" s="4" t="s">
         <v>99</v>
       </c>
@@ -3842,20 +3884,20 @@
       <c r="J46" t="s">
         <v>44</v>
       </c>
-      <c r="K46" s="4" t="s">
+      <c r="L46" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="L46" t="s">
+      <c r="M46" t="s">
         <v>172</v>
       </c>
-      <c r="M46" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O46" s="2"/>
-      <c r="W46" s="2"/>
+      <c r="N46" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P46" s="2"/>
       <c r="X46" s="2"/>
-    </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y46" s="2"/>
+    </row>
+    <row r="47" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A47" s="4" t="s">
         <v>100</v>
       </c>
@@ -3884,20 +3926,20 @@
       <c r="J47" t="s">
         <v>45</v>
       </c>
-      <c r="K47" s="4" t="s">
+      <c r="L47" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="L47" t="s">
+      <c r="M47" t="s">
         <v>172</v>
       </c>
-      <c r="M47" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O47" s="2"/>
-      <c r="W47" s="2"/>
+      <c r="N47" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P47" s="2"/>
       <c r="X47" s="2"/>
-    </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y47" s="2"/>
+    </row>
+    <row r="48" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>101</v>
       </c>
@@ -3926,20 +3968,20 @@
       <c r="J48" t="s">
         <v>46</v>
       </c>
-      <c r="K48" s="4" t="s">
+      <c r="L48" s="4" t="s">
         <v>101</v>
       </c>
-      <c r="L48" t="s">
+      <c r="M48" t="s">
         <v>172</v>
       </c>
-      <c r="M48" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O48" s="2"/>
-      <c r="W48" s="2"/>
+      <c r="N48" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P48" s="2"/>
       <c r="X48" s="2"/>
-    </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y48" s="2"/>
+    </row>
+    <row r="49" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>102</v>
       </c>
@@ -3968,20 +4010,20 @@
       <c r="J49" t="s">
         <v>47</v>
       </c>
-      <c r="K49" s="4" t="s">
+      <c r="L49" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="L49" t="s">
+      <c r="M49" t="s">
         <v>172</v>
       </c>
-      <c r="M49" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O49" s="2"/>
-      <c r="W49" s="2"/>
+      <c r="N49" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P49" s="2"/>
       <c r="X49" s="2"/>
-    </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y49" s="2"/>
+    </row>
+    <row r="50" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>103</v>
       </c>
@@ -4010,20 +4052,20 @@
       <c r="J50" t="s">
         <v>48</v>
       </c>
-      <c r="K50" s="4" t="s">
+      <c r="L50" s="4" t="s">
         <v>103</v>
       </c>
-      <c r="L50" t="s">
+      <c r="M50" t="s">
         <v>172</v>
       </c>
-      <c r="M50" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O50" s="2"/>
-      <c r="W50" s="2"/>
+      <c r="N50" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P50" s="2"/>
       <c r="X50" s="2"/>
-    </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y50" s="2"/>
+    </row>
+    <row r="51" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>104</v>
       </c>
@@ -4052,23 +4094,23 @@
       <c r="J51" t="s">
         <v>49</v>
       </c>
-      <c r="K51" s="4" t="s">
+      <c r="L51" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="L51" t="s">
+      <c r="M51" t="s">
         <v>172</v>
       </c>
-      <c r="M51" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O51" s="2"/>
-      <c r="U51" t="s">
+      <c r="N51" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P51" s="2"/>
+      <c r="V51" t="s">
         <v>241</v>
       </c>
-      <c r="W51" s="2"/>
       <c r="X51" s="2"/>
-    </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y51" s="2"/>
+    </row>
+    <row r="52" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>105</v>
       </c>
@@ -4097,20 +4139,20 @@
       <c r="J52" t="s">
         <v>50</v>
       </c>
-      <c r="K52" s="4" t="s">
+      <c r="L52" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="L52" t="s">
+      <c r="M52" t="s">
         <v>172</v>
       </c>
-      <c r="M52" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O52" s="2"/>
-      <c r="W52" s="2"/>
+      <c r="N52" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P52" s="2"/>
       <c r="X52" s="2"/>
-    </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y52" s="2"/>
+    </row>
+    <row r="53" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>106</v>
       </c>
@@ -4139,20 +4181,20 @@
       <c r="J53" t="s">
         <v>51</v>
       </c>
-      <c r="K53" s="4" t="s">
+      <c r="L53" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="L53" t="s">
+      <c r="M53" t="s">
         <v>172</v>
       </c>
-      <c r="M53" s="2">
-        <v>45793</v>
-      </c>
-      <c r="O53" s="2"/>
-      <c r="W53" s="2"/>
+      <c r="N53" s="2">
+        <v>45793</v>
+      </c>
+      <c r="P53" s="2"/>
       <c r="X53" s="2"/>
-    </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y53" s="2"/>
+    </row>
+    <row r="54" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>107</v>
       </c>
@@ -4178,12 +4220,12 @@
         <v>107</v>
       </c>
       <c r="I54" s="4"/>
-      <c r="M54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="W54" s="2"/>
+      <c r="N54" s="2"/>
+      <c r="P54" s="2"/>
       <c r="X54" s="2"/>
-    </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y54" s="2"/>
+    </row>
+    <row r="55" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>108</v>
       </c>
@@ -4209,12 +4251,12 @@
         <v>108</v>
       </c>
       <c r="I55" s="4"/>
-      <c r="M55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="W55" s="2"/>
+      <c r="N55" s="2"/>
+      <c r="P55" s="2"/>
       <c r="X55" s="2"/>
-    </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="Y55" s="2"/>
+    </row>
+    <row r="56" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>109</v>
       </c>
@@ -4240,10 +4282,10 @@
         <v>109</v>
       </c>
       <c r="I56" s="4"/>
-      <c r="M56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="W56" s="2"/>
+      <c r="N56" s="2"/>
+      <c r="P56" s="2"/>
       <c r="X56" s="2"/>
+      <c r="Y56" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Added Particle module serial number
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F544C5-F917-454A-B283-AEFBBDF29B6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C790E14C-12E0-3A4F-9A47-1C87E0A5EB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="877" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="252">
   <si>
     <t>Box Number</t>
   </si>
@@ -787,6 +787,12 @@
   </si>
   <si>
     <t>P044AD309JYD9NM</t>
+  </si>
+  <si>
+    <t>P044AD348MPK37V</t>
+  </si>
+  <si>
+    <t>e00fce68d3b024424182a0fa</t>
   </si>
 </sst>
 </file>
@@ -4251,6 +4257,12 @@
         <v>108</v>
       </c>
       <c r="I55" s="4"/>
+      <c r="J55" t="s">
+        <v>251</v>
+      </c>
+      <c r="K55" t="s">
+        <v>250</v>
+      </c>
       <c r="N55" s="2"/>
       <c r="P55" s="2"/>
       <c r="X55" s="2"/>

</xml_diff>

<commit_message>
Updated the box deployment tracker sheet
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C790E14C-12E0-3A4F-9A47-1C87E0A5EB49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800B4935-DE88-A943-8EB3-18085BCB21B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="8460" yWindow="1180" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
     <sheet name="BOX Health Checklist" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="275">
   <si>
     <t>Box Number</t>
   </si>
@@ -793,13 +793,85 @@
   </si>
   <si>
     <t>e00fce68d3b024424182a0fa</t>
+  </si>
+  <si>
+    <t>BOX 09 PCB was changed and the box is ready for deployment 08/01/2025</t>
+  </si>
+  <si>
+    <t>08/17/2025</t>
+  </si>
+  <si>
+    <t>08/18/2025</t>
+  </si>
+  <si>
+    <t>08/19/25</t>
+  </si>
+  <si>
+    <t>08/20/25</t>
+  </si>
+  <si>
+    <t>08/21/25</t>
+  </si>
+  <si>
+    <t>08/22/25</t>
+  </si>
+  <si>
+    <t>08/24/25</t>
+  </si>
+  <si>
+    <t>08/25/25</t>
+  </si>
+  <si>
+    <t>08/26/25</t>
+  </si>
+  <si>
+    <t>08/27/25</t>
+  </si>
+  <si>
+    <t>08/28/25</t>
+  </si>
+  <si>
+    <t>08/29/25</t>
+  </si>
+  <si>
+    <t>08/30/25</t>
+  </si>
+  <si>
+    <t>08/31/25</t>
+  </si>
+  <si>
+    <t>09/13/25</t>
+  </si>
+  <si>
+    <t>09/14/25</t>
+  </si>
+  <si>
+    <t>09/15/25</t>
+  </si>
+  <si>
+    <t>09/16/25</t>
+  </si>
+  <si>
+    <t>09/17/25</t>
+  </si>
+  <si>
+    <t>09/18/25</t>
+  </si>
+  <si>
+    <t>09/19/25</t>
+  </si>
+  <si>
+    <t>08/23/25</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -839,8 +911,18 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -865,6 +947,12 @@
         <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -878,7 +966,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -894,6 +982,10 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4308,13 +4400,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33CBFCE6-FDA2-9B4E-A8C1-1998B7362B23}">
-  <dimension ref="A1:AL56"/>
+  <dimension ref="A1:CD56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="11" bestFit="1" customWidth="1"/>
+    <col min="39" max="48" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="64" max="75" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4409,7 +4504,7 @@
         <v>211</v>
       </c>
       <c r="AF1" s="10">
-        <v>45870</v>
+        <v>45665</v>
       </c>
       <c r="AG1" s="10">
         <v>45696</v>
@@ -4429,8 +4524,140 @@
       <c r="AL1" s="10">
         <v>45846</v>
       </c>
-    </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM1" s="15">
+        <v>45876</v>
+      </c>
+      <c r="AN1" s="15">
+        <v>45877</v>
+      </c>
+      <c r="AO1" s="15">
+        <v>45878</v>
+      </c>
+      <c r="AP1" s="15">
+        <v>45879</v>
+      </c>
+      <c r="AQ1" s="15">
+        <v>45880</v>
+      </c>
+      <c r="AR1" s="15">
+        <v>45881</v>
+      </c>
+      <c r="AS1" s="15">
+        <v>45882</v>
+      </c>
+      <c r="AT1" s="15">
+        <v>45883</v>
+      </c>
+      <c r="AU1" s="15">
+        <v>45884</v>
+      </c>
+      <c r="AV1" s="15">
+        <v>45885</v>
+      </c>
+      <c r="AW1" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="AX1" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="AY1" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="AZ1" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="BA1" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="BB1" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="BC1" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="BD1" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="BE1" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="BF1" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="BG1" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="BH1" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="BI1" s="15" t="s">
+        <v>264</v>
+      </c>
+      <c r="BJ1" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="BK1" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="BL1" s="15">
+        <v>45901</v>
+      </c>
+      <c r="BM1" s="15">
+        <v>45902</v>
+      </c>
+      <c r="BN1" s="15">
+        <v>45903</v>
+      </c>
+      <c r="BO1" s="15">
+        <v>45904</v>
+      </c>
+      <c r="BP1" s="15">
+        <v>45905</v>
+      </c>
+      <c r="BQ1" s="15">
+        <v>45906</v>
+      </c>
+      <c r="BR1" s="15">
+        <v>45907</v>
+      </c>
+      <c r="BS1" s="15">
+        <v>45908</v>
+      </c>
+      <c r="BT1" s="15">
+        <v>45909</v>
+      </c>
+      <c r="BU1" s="15">
+        <v>45910</v>
+      </c>
+      <c r="BV1" s="15">
+        <v>45911</v>
+      </c>
+      <c r="BW1" s="15">
+        <v>45912</v>
+      </c>
+      <c r="BX1" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="BY1" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="BZ1" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="CA1" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="CB1" s="15" t="s">
+        <v>271</v>
+      </c>
+      <c r="CC1" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="CD1" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="2" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>55</v>
       </c>
@@ -4471,8 +4698,52 @@
       <c r="AJ2" s="6"/>
       <c r="AK2" s="6"/>
       <c r="AL2" s="6"/>
-    </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM2" s="16"/>
+      <c r="AN2" s="16"/>
+      <c r="AO2" s="16"/>
+      <c r="AP2" s="16"/>
+      <c r="AQ2" s="16"/>
+      <c r="AR2" s="16"/>
+      <c r="AS2" s="16"/>
+      <c r="AT2" s="16"/>
+      <c r="AU2" s="16"/>
+      <c r="AV2" s="16"/>
+      <c r="AW2" s="16"/>
+      <c r="AX2" s="16"/>
+      <c r="AY2" s="16"/>
+      <c r="AZ2" s="16"/>
+      <c r="BA2" s="16"/>
+      <c r="BB2" s="16"/>
+      <c r="BC2" s="16"/>
+      <c r="BD2" s="16"/>
+      <c r="BE2" s="16"/>
+      <c r="BF2" s="16"/>
+      <c r="BG2" s="16"/>
+      <c r="BH2" s="16"/>
+      <c r="BI2" s="16"/>
+      <c r="BJ2" s="16"/>
+      <c r="BK2" s="16"/>
+      <c r="BL2" s="16"/>
+      <c r="BM2" s="16"/>
+      <c r="BN2" s="16"/>
+      <c r="BO2" s="16"/>
+      <c r="BP2" s="16"/>
+      <c r="BQ2" s="16"/>
+      <c r="BR2" s="16"/>
+      <c r="BS2" s="16"/>
+      <c r="BT2" s="16"/>
+      <c r="BU2" s="16"/>
+      <c r="BV2" s="16"/>
+      <c r="BW2" s="16"/>
+      <c r="BX2" s="16"/>
+      <c r="BY2" s="16"/>
+      <c r="BZ2" s="16"/>
+      <c r="CA2" s="16"/>
+      <c r="CB2" s="16"/>
+      <c r="CC2" s="16"/>
+      <c r="CD2" s="16"/>
+    </row>
+    <row r="3" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>56</v>
       </c>
@@ -4513,8 +4784,52 @@
       <c r="AJ3" s="6"/>
       <c r="AK3" s="6"/>
       <c r="AL3" s="6"/>
-    </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM3" s="16"/>
+      <c r="AN3" s="16"/>
+      <c r="AO3" s="16"/>
+      <c r="AP3" s="16"/>
+      <c r="AQ3" s="16"/>
+      <c r="AR3" s="16"/>
+      <c r="AS3" s="16"/>
+      <c r="AT3" s="16"/>
+      <c r="AU3" s="16"/>
+      <c r="AV3" s="16"/>
+      <c r="AW3" s="16"/>
+      <c r="AX3" s="16"/>
+      <c r="AY3" s="16"/>
+      <c r="AZ3" s="16"/>
+      <c r="BA3" s="16"/>
+      <c r="BB3" s="16"/>
+      <c r="BC3" s="16"/>
+      <c r="BD3" s="16"/>
+      <c r="BE3" s="16"/>
+      <c r="BF3" s="16"/>
+      <c r="BG3" s="16"/>
+      <c r="BH3" s="16"/>
+      <c r="BI3" s="16"/>
+      <c r="BJ3" s="16"/>
+      <c r="BK3" s="16"/>
+      <c r="BL3" s="16"/>
+      <c r="BM3" s="16"/>
+      <c r="BN3" s="16"/>
+      <c r="BO3" s="16"/>
+      <c r="BP3" s="16"/>
+      <c r="BQ3" s="16"/>
+      <c r="BR3" s="16"/>
+      <c r="BS3" s="16"/>
+      <c r="BT3" s="16"/>
+      <c r="BU3" s="16"/>
+      <c r="BV3" s="16"/>
+      <c r="BW3" s="16"/>
+      <c r="BX3" s="16"/>
+      <c r="BY3" s="16"/>
+      <c r="BZ3" s="16"/>
+      <c r="CA3" s="16"/>
+      <c r="CB3" s="16"/>
+      <c r="CC3" s="16"/>
+      <c r="CD3" s="16"/>
+    </row>
+    <row r="4" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>57</v>
       </c>
@@ -4555,8 +4870,52 @@
       <c r="AJ4" s="6"/>
       <c r="AK4" s="6"/>
       <c r="AL4" s="6"/>
-    </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM4" s="16"/>
+      <c r="AN4" s="16"/>
+      <c r="AO4" s="16"/>
+      <c r="AP4" s="16"/>
+      <c r="AQ4" s="16"/>
+      <c r="AR4" s="16"/>
+      <c r="AS4" s="16"/>
+      <c r="AT4" s="16"/>
+      <c r="AU4" s="16"/>
+      <c r="AV4" s="16"/>
+      <c r="AW4" s="16"/>
+      <c r="AX4" s="16"/>
+      <c r="AY4" s="16"/>
+      <c r="AZ4" s="16"/>
+      <c r="BA4" s="16"/>
+      <c r="BB4" s="16"/>
+      <c r="BC4" s="16"/>
+      <c r="BD4" s="16"/>
+      <c r="BE4" s="16"/>
+      <c r="BF4" s="16"/>
+      <c r="BG4" s="16"/>
+      <c r="BH4" s="16"/>
+      <c r="BI4" s="16"/>
+      <c r="BJ4" s="16"/>
+      <c r="BK4" s="16"/>
+      <c r="BL4" s="16"/>
+      <c r="BM4" s="16"/>
+      <c r="BN4" s="16"/>
+      <c r="BO4" s="16"/>
+      <c r="BP4" s="16"/>
+      <c r="BQ4" s="16"/>
+      <c r="BR4" s="16"/>
+      <c r="BS4" s="16"/>
+      <c r="BT4" s="16"/>
+      <c r="BU4" s="16"/>
+      <c r="BV4" s="16"/>
+      <c r="BW4" s="16"/>
+      <c r="BX4" s="16"/>
+      <c r="BY4" s="16"/>
+      <c r="BZ4" s="16"/>
+      <c r="CA4" s="16"/>
+      <c r="CB4" s="16"/>
+      <c r="CC4" s="16"/>
+      <c r="CD4" s="16"/>
+    </row>
+    <row r="5" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>58</v>
       </c>
@@ -4597,8 +4956,52 @@
       <c r="AJ5" s="6"/>
       <c r="AK5" s="6"/>
       <c r="AL5" s="6"/>
-    </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM5" s="16"/>
+      <c r="AN5" s="16"/>
+      <c r="AO5" s="16"/>
+      <c r="AP5" s="16"/>
+      <c r="AQ5" s="16"/>
+      <c r="AR5" s="16"/>
+      <c r="AS5" s="16"/>
+      <c r="AT5" s="16"/>
+      <c r="AU5" s="16"/>
+      <c r="AV5" s="16"/>
+      <c r="AW5" s="16"/>
+      <c r="AX5" s="16"/>
+      <c r="AY5" s="16"/>
+      <c r="AZ5" s="16"/>
+      <c r="BA5" s="16"/>
+      <c r="BB5" s="16"/>
+      <c r="BC5" s="16"/>
+      <c r="BD5" s="16"/>
+      <c r="BE5" s="16"/>
+      <c r="BF5" s="16"/>
+      <c r="BG5" s="16"/>
+      <c r="BH5" s="16"/>
+      <c r="BI5" s="16"/>
+      <c r="BJ5" s="16"/>
+      <c r="BK5" s="16"/>
+      <c r="BL5" s="16"/>
+      <c r="BM5" s="16"/>
+      <c r="BN5" s="16"/>
+      <c r="BO5" s="16"/>
+      <c r="BP5" s="16"/>
+      <c r="BQ5" s="16"/>
+      <c r="BR5" s="16"/>
+      <c r="BS5" s="16"/>
+      <c r="BT5" s="16"/>
+      <c r="BU5" s="16"/>
+      <c r="BV5" s="16"/>
+      <c r="BW5" s="16"/>
+      <c r="BX5" s="16"/>
+      <c r="BY5" s="16"/>
+      <c r="BZ5" s="16"/>
+      <c r="CA5" s="16"/>
+      <c r="CB5" s="16"/>
+      <c r="CC5" s="16"/>
+      <c r="CD5" s="16"/>
+    </row>
+    <row r="6" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>59</v>
       </c>
@@ -4639,8 +5042,52 @@
       <c r="AJ6" s="6"/>
       <c r="AK6" s="6"/>
       <c r="AL6" s="6"/>
-    </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM6" s="16"/>
+      <c r="AN6" s="16"/>
+      <c r="AO6" s="16"/>
+      <c r="AP6" s="16"/>
+      <c r="AQ6" s="16"/>
+      <c r="AR6" s="16"/>
+      <c r="AS6" s="16"/>
+      <c r="AT6" s="16"/>
+      <c r="AU6" s="16"/>
+      <c r="AV6" s="16"/>
+      <c r="AW6" s="16"/>
+      <c r="AX6" s="16"/>
+      <c r="AY6" s="16"/>
+      <c r="AZ6" s="16"/>
+      <c r="BA6" s="16"/>
+      <c r="BB6" s="16"/>
+      <c r="BC6" s="16"/>
+      <c r="BD6" s="16"/>
+      <c r="BE6" s="16"/>
+      <c r="BF6" s="16"/>
+      <c r="BG6" s="16"/>
+      <c r="BH6" s="16"/>
+      <c r="BI6" s="16"/>
+      <c r="BJ6" s="16"/>
+      <c r="BK6" s="16"/>
+      <c r="BL6" s="16"/>
+      <c r="BM6" s="16"/>
+      <c r="BN6" s="16"/>
+      <c r="BO6" s="16"/>
+      <c r="BP6" s="16"/>
+      <c r="BQ6" s="16"/>
+      <c r="BR6" s="16"/>
+      <c r="BS6" s="16"/>
+      <c r="BT6" s="16"/>
+      <c r="BU6" s="16"/>
+      <c r="BV6" s="16"/>
+      <c r="BW6" s="16"/>
+      <c r="BX6" s="16"/>
+      <c r="BY6" s="16"/>
+      <c r="BZ6" s="16"/>
+      <c r="CA6" s="16"/>
+      <c r="CB6" s="16"/>
+      <c r="CC6" s="16"/>
+      <c r="CD6" s="16"/>
+    </row>
+    <row r="7" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>60</v>
       </c>
@@ -4681,8 +5128,52 @@
       <c r="AJ7" s="8"/>
       <c r="AK7" s="8"/>
       <c r="AL7" s="8"/>
-    </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM7" s="17"/>
+      <c r="AN7" s="17"/>
+      <c r="AO7" s="17"/>
+      <c r="AP7" s="17"/>
+      <c r="AQ7" s="17"/>
+      <c r="AR7" s="17"/>
+      <c r="AS7" s="17"/>
+      <c r="AT7" s="17"/>
+      <c r="AU7" s="17"/>
+      <c r="AV7" s="17"/>
+      <c r="AW7" s="17"/>
+      <c r="AX7" s="17"/>
+      <c r="AY7" s="17"/>
+      <c r="AZ7" s="17"/>
+      <c r="BA7" s="17"/>
+      <c r="BB7" s="17"/>
+      <c r="BC7" s="17"/>
+      <c r="BD7" s="17"/>
+      <c r="BE7" s="17"/>
+      <c r="BF7" s="17"/>
+      <c r="BG7" s="17"/>
+      <c r="BH7" s="17"/>
+      <c r="BI7" s="17"/>
+      <c r="BJ7" s="17"/>
+      <c r="BK7" s="17"/>
+      <c r="BL7" s="17"/>
+      <c r="BM7" s="17"/>
+      <c r="BN7" s="17"/>
+      <c r="BO7" s="17"/>
+      <c r="BP7" s="17"/>
+      <c r="BQ7" s="17"/>
+      <c r="BR7" s="17"/>
+      <c r="BS7" s="17"/>
+      <c r="BT7" s="17"/>
+      <c r="BU7" s="17"/>
+      <c r="BV7" s="17"/>
+      <c r="BW7" s="17"/>
+      <c r="BX7" s="17"/>
+      <c r="BY7" s="17"/>
+      <c r="BZ7" s="17"/>
+      <c r="CA7" s="17"/>
+      <c r="CB7" s="17"/>
+      <c r="CC7" s="17"/>
+      <c r="CD7" s="17"/>
+    </row>
+    <row r="8" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>61</v>
       </c>
@@ -4723,8 +5214,52 @@
       <c r="AJ8" s="8"/>
       <c r="AK8" s="8"/>
       <c r="AL8" s="8"/>
-    </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM8" s="17"/>
+      <c r="AN8" s="17"/>
+      <c r="AO8" s="17"/>
+      <c r="AP8" s="17"/>
+      <c r="AQ8" s="17"/>
+      <c r="AR8" s="17"/>
+      <c r="AS8" s="17"/>
+      <c r="AT8" s="17"/>
+      <c r="AU8" s="17"/>
+      <c r="AV8" s="17"/>
+      <c r="AW8" s="17"/>
+      <c r="AX8" s="17"/>
+      <c r="AY8" s="17"/>
+      <c r="AZ8" s="17"/>
+      <c r="BA8" s="17"/>
+      <c r="BB8" s="17"/>
+      <c r="BC8" s="17"/>
+      <c r="BD8" s="17"/>
+      <c r="BE8" s="17"/>
+      <c r="BF8" s="17"/>
+      <c r="BG8" s="17"/>
+      <c r="BH8" s="17"/>
+      <c r="BI8" s="17"/>
+      <c r="BJ8" s="17"/>
+      <c r="BK8" s="17"/>
+      <c r="BL8" s="17"/>
+      <c r="BM8" s="17"/>
+      <c r="BN8" s="17"/>
+      <c r="BO8" s="17"/>
+      <c r="BP8" s="17"/>
+      <c r="BQ8" s="17"/>
+      <c r="BR8" s="17"/>
+      <c r="BS8" s="17"/>
+      <c r="BT8" s="17"/>
+      <c r="BU8" s="17"/>
+      <c r="BV8" s="17"/>
+      <c r="BW8" s="17"/>
+      <c r="BX8" s="17"/>
+      <c r="BY8" s="17"/>
+      <c r="BZ8" s="17"/>
+      <c r="CA8" s="17"/>
+      <c r="CB8" s="17"/>
+      <c r="CC8" s="17"/>
+      <c r="CD8" s="17"/>
+    </row>
+    <row r="9" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>62</v>
       </c>
@@ -4765,8 +5300,52 @@
       <c r="AJ9" s="8"/>
       <c r="AK9" s="8"/>
       <c r="AL9" s="8"/>
-    </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM9" s="17"/>
+      <c r="AN9" s="17"/>
+      <c r="AO9" s="17"/>
+      <c r="AP9" s="17"/>
+      <c r="AQ9" s="17"/>
+      <c r="AR9" s="17"/>
+      <c r="AS9" s="17"/>
+      <c r="AT9" s="17"/>
+      <c r="AU9" s="17"/>
+      <c r="AV9" s="17"/>
+      <c r="AW9" s="17"/>
+      <c r="AX9" s="17"/>
+      <c r="AY9" s="17"/>
+      <c r="AZ9" s="17"/>
+      <c r="BA9" s="17"/>
+      <c r="BB9" s="17"/>
+      <c r="BC9" s="17"/>
+      <c r="BD9" s="17"/>
+      <c r="BE9" s="17"/>
+      <c r="BF9" s="17"/>
+      <c r="BG9" s="17"/>
+      <c r="BH9" s="17"/>
+      <c r="BI9" s="17"/>
+      <c r="BJ9" s="17"/>
+      <c r="BK9" s="17"/>
+      <c r="BL9" s="17"/>
+      <c r="BM9" s="17"/>
+      <c r="BN9" s="17"/>
+      <c r="BO9" s="17"/>
+      <c r="BP9" s="17"/>
+      <c r="BQ9" s="17"/>
+      <c r="BR9" s="17"/>
+      <c r="BS9" s="17"/>
+      <c r="BT9" s="17"/>
+      <c r="BU9" s="17"/>
+      <c r="BV9" s="17"/>
+      <c r="BW9" s="17"/>
+      <c r="BX9" s="17"/>
+      <c r="BY9" s="17"/>
+      <c r="BZ9" s="17"/>
+      <c r="CA9" s="17"/>
+      <c r="CB9" s="17"/>
+      <c r="CC9" s="17"/>
+      <c r="CD9" s="17"/>
+    </row>
+    <row r="10" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>63</v>
       </c>
@@ -4780,8 +5359,52 @@
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="7"/>
-    </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM10" s="18"/>
+      <c r="AN10" s="18"/>
+      <c r="AO10" s="18"/>
+      <c r="AP10" s="18"/>
+      <c r="AQ10" s="18"/>
+      <c r="AR10" s="18"/>
+      <c r="AS10" s="18"/>
+      <c r="AT10" s="18"/>
+      <c r="AU10" s="18"/>
+      <c r="AV10" s="18"/>
+      <c r="AW10" s="18"/>
+      <c r="AX10" s="18"/>
+      <c r="AY10" s="18"/>
+      <c r="AZ10" s="18"/>
+      <c r="BA10" s="18"/>
+      <c r="BB10" s="18"/>
+      <c r="BC10" s="18"/>
+      <c r="BD10" s="18"/>
+      <c r="BE10" s="18"/>
+      <c r="BF10" s="18"/>
+      <c r="BG10" s="18"/>
+      <c r="BH10" s="18"/>
+      <c r="BI10" s="18"/>
+      <c r="BJ10" s="18"/>
+      <c r="BK10" s="18"/>
+      <c r="BL10" s="18"/>
+      <c r="BM10" s="18"/>
+      <c r="BN10" s="18"/>
+      <c r="BO10" s="18"/>
+      <c r="BP10" s="18"/>
+      <c r="BQ10" s="18"/>
+      <c r="BR10" s="18"/>
+      <c r="BS10" s="18"/>
+      <c r="BT10" s="18"/>
+      <c r="BU10" s="18"/>
+      <c r="BV10" s="18"/>
+      <c r="BW10" s="18"/>
+      <c r="BX10" s="18"/>
+      <c r="BY10" s="18"/>
+      <c r="BZ10" s="18"/>
+      <c r="CA10" s="18"/>
+      <c r="CB10" s="18"/>
+      <c r="CC10" s="18"/>
+      <c r="CD10" s="18"/>
+    </row>
+    <row r="11" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>64</v>
       </c>
@@ -4822,8 +5445,52 @@
       <c r="AJ11" s="8"/>
       <c r="AK11" s="8"/>
       <c r="AL11" s="8"/>
-    </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM11" s="17"/>
+      <c r="AN11" s="17"/>
+      <c r="AO11" s="17"/>
+      <c r="AP11" s="17"/>
+      <c r="AQ11" s="17"/>
+      <c r="AR11" s="17"/>
+      <c r="AS11" s="17"/>
+      <c r="AT11" s="17"/>
+      <c r="AU11" s="17"/>
+      <c r="AV11" s="17"/>
+      <c r="AW11" s="17"/>
+      <c r="AX11" s="17"/>
+      <c r="AY11" s="17"/>
+      <c r="AZ11" s="17"/>
+      <c r="BA11" s="17"/>
+      <c r="BB11" s="17"/>
+      <c r="BC11" s="17"/>
+      <c r="BD11" s="17"/>
+      <c r="BE11" s="17"/>
+      <c r="BF11" s="17"/>
+      <c r="BG11" s="17"/>
+      <c r="BH11" s="17"/>
+      <c r="BI11" s="17"/>
+      <c r="BJ11" s="17"/>
+      <c r="BK11" s="17"/>
+      <c r="BL11" s="17"/>
+      <c r="BM11" s="17"/>
+      <c r="BN11" s="17"/>
+      <c r="BO11" s="17"/>
+      <c r="BP11" s="17"/>
+      <c r="BQ11" s="17"/>
+      <c r="BR11" s="17"/>
+      <c r="BS11" s="17"/>
+      <c r="BT11" s="17"/>
+      <c r="BU11" s="17"/>
+      <c r="BV11" s="17"/>
+      <c r="BW11" s="17"/>
+      <c r="BX11" s="17"/>
+      <c r="BY11" s="17"/>
+      <c r="BZ11" s="17"/>
+      <c r="CA11" s="17"/>
+      <c r="CB11" s="17"/>
+      <c r="CC11" s="17"/>
+      <c r="CD11" s="17"/>
+    </row>
+    <row r="12" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>65</v>
       </c>
@@ -4864,8 +5531,52 @@
       <c r="AJ12" s="8"/>
       <c r="AK12" s="8"/>
       <c r="AL12" s="8"/>
-    </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM12" s="17"/>
+      <c r="AN12" s="17"/>
+      <c r="AO12" s="17"/>
+      <c r="AP12" s="17"/>
+      <c r="AQ12" s="17"/>
+      <c r="AR12" s="17"/>
+      <c r="AS12" s="17"/>
+      <c r="AT12" s="17"/>
+      <c r="AU12" s="17"/>
+      <c r="AV12" s="17"/>
+      <c r="AW12" s="17"/>
+      <c r="AX12" s="17"/>
+      <c r="AY12" s="17"/>
+      <c r="AZ12" s="17"/>
+      <c r="BA12" s="17"/>
+      <c r="BB12" s="17"/>
+      <c r="BC12" s="17"/>
+      <c r="BD12" s="17"/>
+      <c r="BE12" s="17"/>
+      <c r="BF12" s="17"/>
+      <c r="BG12" s="17"/>
+      <c r="BH12" s="17"/>
+      <c r="BI12" s="17"/>
+      <c r="BJ12" s="17"/>
+      <c r="BK12" s="17"/>
+      <c r="BL12" s="17"/>
+      <c r="BM12" s="17"/>
+      <c r="BN12" s="17"/>
+      <c r="BO12" s="17"/>
+      <c r="BP12" s="17"/>
+      <c r="BQ12" s="17"/>
+      <c r="BR12" s="17"/>
+      <c r="BS12" s="17"/>
+      <c r="BT12" s="17"/>
+      <c r="BU12" s="17"/>
+      <c r="BV12" s="17"/>
+      <c r="BW12" s="17"/>
+      <c r="BX12" s="17"/>
+      <c r="BY12" s="17"/>
+      <c r="BZ12" s="17"/>
+      <c r="CA12" s="17"/>
+      <c r="CB12" s="17"/>
+      <c r="CC12" s="17"/>
+      <c r="CD12" s="17"/>
+    </row>
+    <row r="13" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>66</v>
       </c>
@@ -4906,8 +5617,52 @@
       <c r="AJ13" s="8"/>
       <c r="AK13" s="8"/>
       <c r="AL13" s="8"/>
-    </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM13" s="17"/>
+      <c r="AN13" s="17"/>
+      <c r="AO13" s="17"/>
+      <c r="AP13" s="17"/>
+      <c r="AQ13" s="17"/>
+      <c r="AR13" s="17"/>
+      <c r="AS13" s="17"/>
+      <c r="AT13" s="17"/>
+      <c r="AU13" s="17"/>
+      <c r="AV13" s="17"/>
+      <c r="AW13" s="17"/>
+      <c r="AX13" s="17"/>
+      <c r="AY13" s="17"/>
+      <c r="AZ13" s="17"/>
+      <c r="BA13" s="17"/>
+      <c r="BB13" s="17"/>
+      <c r="BC13" s="17"/>
+      <c r="BD13" s="17"/>
+      <c r="BE13" s="17"/>
+      <c r="BF13" s="17"/>
+      <c r="BG13" s="17"/>
+      <c r="BH13" s="17"/>
+      <c r="BI13" s="17"/>
+      <c r="BJ13" s="17"/>
+      <c r="BK13" s="17"/>
+      <c r="BL13" s="17"/>
+      <c r="BM13" s="17"/>
+      <c r="BN13" s="17"/>
+      <c r="BO13" s="17"/>
+      <c r="BP13" s="17"/>
+      <c r="BQ13" s="17"/>
+      <c r="BR13" s="17"/>
+      <c r="BS13" s="17"/>
+      <c r="BT13" s="17"/>
+      <c r="BU13" s="17"/>
+      <c r="BV13" s="17"/>
+      <c r="BW13" s="17"/>
+      <c r="BX13" s="17"/>
+      <c r="BY13" s="17"/>
+      <c r="BZ13" s="17"/>
+      <c r="CA13" s="17"/>
+      <c r="CB13" s="17"/>
+      <c r="CC13" s="17"/>
+      <c r="CD13" s="17"/>
+    </row>
+    <row r="14" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>67</v>
       </c>
@@ -4948,8 +5703,52 @@
       <c r="AJ14" s="8"/>
       <c r="AK14" s="8"/>
       <c r="AL14" s="8"/>
-    </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM14" s="17"/>
+      <c r="AN14" s="17"/>
+      <c r="AO14" s="17"/>
+      <c r="AP14" s="17"/>
+      <c r="AQ14" s="17"/>
+      <c r="AR14" s="17"/>
+      <c r="AS14" s="17"/>
+      <c r="AT14" s="17"/>
+      <c r="AU14" s="17"/>
+      <c r="AV14" s="17"/>
+      <c r="AW14" s="17"/>
+      <c r="AX14" s="17"/>
+      <c r="AY14" s="17"/>
+      <c r="AZ14" s="17"/>
+      <c r="BA14" s="17"/>
+      <c r="BB14" s="17"/>
+      <c r="BC14" s="17"/>
+      <c r="BD14" s="17"/>
+      <c r="BE14" s="17"/>
+      <c r="BF14" s="17"/>
+      <c r="BG14" s="17"/>
+      <c r="BH14" s="17"/>
+      <c r="BI14" s="17"/>
+      <c r="BJ14" s="17"/>
+      <c r="BK14" s="17"/>
+      <c r="BL14" s="17"/>
+      <c r="BM14" s="17"/>
+      <c r="BN14" s="17"/>
+      <c r="BO14" s="17"/>
+      <c r="BP14" s="17"/>
+      <c r="BQ14" s="17"/>
+      <c r="BR14" s="17"/>
+      <c r="BS14" s="17"/>
+      <c r="BT14" s="17"/>
+      <c r="BU14" s="17"/>
+      <c r="BV14" s="17"/>
+      <c r="BW14" s="17"/>
+      <c r="BX14" s="17"/>
+      <c r="BY14" s="17"/>
+      <c r="BZ14" s="17"/>
+      <c r="CA14" s="17"/>
+      <c r="CB14" s="17"/>
+      <c r="CC14" s="17"/>
+      <c r="CD14" s="17"/>
+    </row>
+    <row r="15" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>68</v>
       </c>
@@ -4958,7 +5757,7 @@
       <c r="G15" s="9"/>
       <c r="H15" s="9"/>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>69</v>
       </c>
@@ -4969,8 +5768,52 @@
       <c r="AJ16" s="8"/>
       <c r="AK16" s="8"/>
       <c r="AL16" s="8"/>
-    </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM16" s="17"/>
+      <c r="AN16" s="17"/>
+      <c r="AO16" s="17"/>
+      <c r="AP16" s="17"/>
+      <c r="AQ16" s="17"/>
+      <c r="AR16" s="17"/>
+      <c r="AS16" s="17"/>
+      <c r="AT16" s="17"/>
+      <c r="AU16" s="17"/>
+      <c r="AV16" s="17"/>
+      <c r="AW16" s="17"/>
+      <c r="AX16" s="17"/>
+      <c r="AY16" s="17"/>
+      <c r="AZ16" s="17"/>
+      <c r="BA16" s="17"/>
+      <c r="BB16" s="17"/>
+      <c r="BC16" s="17"/>
+      <c r="BD16" s="17"/>
+      <c r="BE16" s="17"/>
+      <c r="BF16" s="17"/>
+      <c r="BG16" s="17"/>
+      <c r="BH16" s="17"/>
+      <c r="BI16" s="17"/>
+      <c r="BJ16" s="17"/>
+      <c r="BK16" s="17"/>
+      <c r="BL16" s="17"/>
+      <c r="BM16" s="17"/>
+      <c r="BN16" s="17"/>
+      <c r="BO16" s="17"/>
+      <c r="BP16" s="17"/>
+      <c r="BQ16" s="17"/>
+      <c r="BR16" s="17"/>
+      <c r="BS16" s="17"/>
+      <c r="BT16" s="17"/>
+      <c r="BU16" s="17"/>
+      <c r="BV16" s="17"/>
+      <c r="BW16" s="17"/>
+      <c r="BX16" s="17"/>
+      <c r="BY16" s="17"/>
+      <c r="BZ16" s="17"/>
+      <c r="CA16" s="17"/>
+      <c r="CB16" s="17"/>
+      <c r="CC16" s="17"/>
+      <c r="CD16" s="17"/>
+    </row>
+    <row r="17" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -4981,8 +5824,52 @@
       <c r="AJ17" s="8"/>
       <c r="AK17" s="8"/>
       <c r="AL17" s="8"/>
-    </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM17" s="17"/>
+      <c r="AN17" s="17"/>
+      <c r="AO17" s="17"/>
+      <c r="AP17" s="17"/>
+      <c r="AQ17" s="17"/>
+      <c r="AR17" s="17"/>
+      <c r="AS17" s="17"/>
+      <c r="AT17" s="17"/>
+      <c r="AU17" s="17"/>
+      <c r="AV17" s="17"/>
+      <c r="AW17" s="17"/>
+      <c r="AX17" s="17"/>
+      <c r="AY17" s="17"/>
+      <c r="AZ17" s="17"/>
+      <c r="BA17" s="17"/>
+      <c r="BB17" s="17"/>
+      <c r="BC17" s="17"/>
+      <c r="BD17" s="17"/>
+      <c r="BE17" s="17"/>
+      <c r="BF17" s="17"/>
+      <c r="BG17" s="17"/>
+      <c r="BH17" s="17"/>
+      <c r="BI17" s="17"/>
+      <c r="BJ17" s="17"/>
+      <c r="BK17" s="17"/>
+      <c r="BL17" s="17"/>
+      <c r="BM17" s="17"/>
+      <c r="BN17" s="17"/>
+      <c r="BO17" s="17"/>
+      <c r="BP17" s="17"/>
+      <c r="BQ17" s="17"/>
+      <c r="BR17" s="17"/>
+      <c r="BS17" s="17"/>
+      <c r="BT17" s="17"/>
+      <c r="BU17" s="17"/>
+      <c r="BV17" s="17"/>
+      <c r="BW17" s="17"/>
+      <c r="BX17" s="17"/>
+      <c r="BY17" s="17"/>
+      <c r="BZ17" s="17"/>
+      <c r="CA17" s="17"/>
+      <c r="CB17" s="17"/>
+      <c r="CC17" s="17"/>
+      <c r="CD17" s="17"/>
+    </row>
+    <row r="18" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>71</v>
       </c>
@@ -4993,8 +5880,52 @@
       <c r="AJ18" s="8"/>
       <c r="AK18" s="8"/>
       <c r="AL18" s="8"/>
-    </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM18" s="17"/>
+      <c r="AN18" s="17"/>
+      <c r="AO18" s="17"/>
+      <c r="AP18" s="17"/>
+      <c r="AQ18" s="17"/>
+      <c r="AR18" s="17"/>
+      <c r="AS18" s="17"/>
+      <c r="AT18" s="17"/>
+      <c r="AU18" s="17"/>
+      <c r="AV18" s="17"/>
+      <c r="AW18" s="17"/>
+      <c r="AX18" s="17"/>
+      <c r="AY18" s="17"/>
+      <c r="AZ18" s="17"/>
+      <c r="BA18" s="17"/>
+      <c r="BB18" s="17"/>
+      <c r="BC18" s="17"/>
+      <c r="BD18" s="17"/>
+      <c r="BE18" s="17"/>
+      <c r="BF18" s="17"/>
+      <c r="BG18" s="17"/>
+      <c r="BH18" s="17"/>
+      <c r="BI18" s="17"/>
+      <c r="BJ18" s="17"/>
+      <c r="BK18" s="17"/>
+      <c r="BL18" s="17"/>
+      <c r="BM18" s="17"/>
+      <c r="BN18" s="17"/>
+      <c r="BO18" s="17"/>
+      <c r="BP18" s="17"/>
+      <c r="BQ18" s="17"/>
+      <c r="BR18" s="17"/>
+      <c r="BS18" s="17"/>
+      <c r="BT18" s="17"/>
+      <c r="BU18" s="17"/>
+      <c r="BV18" s="17"/>
+      <c r="BW18" s="17"/>
+      <c r="BX18" s="17"/>
+      <c r="BY18" s="17"/>
+      <c r="BZ18" s="17"/>
+      <c r="CA18" s="17"/>
+      <c r="CB18" s="17"/>
+      <c r="CC18" s="17"/>
+      <c r="CD18" s="17"/>
+    </row>
+    <row r="19" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>72</v>
       </c>
@@ -5035,8 +5966,52 @@
       <c r="AJ19" s="8"/>
       <c r="AK19" s="8"/>
       <c r="AL19" s="8"/>
-    </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM19" s="17"/>
+      <c r="AN19" s="17"/>
+      <c r="AO19" s="17"/>
+      <c r="AP19" s="17"/>
+      <c r="AQ19" s="17"/>
+      <c r="AR19" s="17"/>
+      <c r="AS19" s="17"/>
+      <c r="AT19" s="17"/>
+      <c r="AU19" s="17"/>
+      <c r="AV19" s="17"/>
+      <c r="AW19" s="17"/>
+      <c r="AX19" s="17"/>
+      <c r="AY19" s="17"/>
+      <c r="AZ19" s="17"/>
+      <c r="BA19" s="17"/>
+      <c r="BB19" s="17"/>
+      <c r="BC19" s="17"/>
+      <c r="BD19" s="17"/>
+      <c r="BE19" s="17"/>
+      <c r="BF19" s="17"/>
+      <c r="BG19" s="17"/>
+      <c r="BH19" s="17"/>
+      <c r="BI19" s="17"/>
+      <c r="BJ19" s="17"/>
+      <c r="BK19" s="17"/>
+      <c r="BL19" s="17"/>
+      <c r="BM19" s="17"/>
+      <c r="BN19" s="17"/>
+      <c r="BO19" s="17"/>
+      <c r="BP19" s="17"/>
+      <c r="BQ19" s="17"/>
+      <c r="BR19" s="17"/>
+      <c r="BS19" s="17"/>
+      <c r="BT19" s="17"/>
+      <c r="BU19" s="17"/>
+      <c r="BV19" s="17"/>
+      <c r="BW19" s="17"/>
+      <c r="BX19" s="17"/>
+      <c r="BY19" s="17"/>
+      <c r="BZ19" s="17"/>
+      <c r="CA19" s="17"/>
+      <c r="CB19" s="17"/>
+      <c r="CC19" s="17"/>
+      <c r="CD19" s="17"/>
+    </row>
+    <row r="20" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>73</v>
       </c>
@@ -5077,8 +6052,52 @@
       <c r="AJ20" s="8"/>
       <c r="AK20" s="8"/>
       <c r="AL20" s="8"/>
-    </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM20" s="17"/>
+      <c r="AN20" s="17"/>
+      <c r="AO20" s="17"/>
+      <c r="AP20" s="17"/>
+      <c r="AQ20" s="17"/>
+      <c r="AR20" s="17"/>
+      <c r="AS20" s="17"/>
+      <c r="AT20" s="17"/>
+      <c r="AU20" s="17"/>
+      <c r="AV20" s="17"/>
+      <c r="AW20" s="17"/>
+      <c r="AX20" s="17"/>
+      <c r="AY20" s="17"/>
+      <c r="AZ20" s="17"/>
+      <c r="BA20" s="17"/>
+      <c r="BB20" s="17"/>
+      <c r="BC20" s="17"/>
+      <c r="BD20" s="17"/>
+      <c r="BE20" s="17"/>
+      <c r="BF20" s="17"/>
+      <c r="BG20" s="17"/>
+      <c r="BH20" s="17"/>
+      <c r="BI20" s="17"/>
+      <c r="BJ20" s="17"/>
+      <c r="BK20" s="17"/>
+      <c r="BL20" s="17"/>
+      <c r="BM20" s="17"/>
+      <c r="BN20" s="17"/>
+      <c r="BO20" s="17"/>
+      <c r="BP20" s="17"/>
+      <c r="BQ20" s="17"/>
+      <c r="BR20" s="17"/>
+      <c r="BS20" s="17"/>
+      <c r="BT20" s="17"/>
+      <c r="BU20" s="17"/>
+      <c r="BV20" s="17"/>
+      <c r="BW20" s="17"/>
+      <c r="BX20" s="17"/>
+      <c r="BY20" s="17"/>
+      <c r="BZ20" s="17"/>
+      <c r="CA20" s="17"/>
+      <c r="CB20" s="17"/>
+      <c r="CC20" s="17"/>
+      <c r="CD20" s="17"/>
+    </row>
+    <row r="21" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>74</v>
       </c>
@@ -5119,8 +6138,52 @@
       <c r="AJ21" s="8"/>
       <c r="AK21" s="8"/>
       <c r="AL21" s="8"/>
-    </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM21" s="17"/>
+      <c r="AN21" s="17"/>
+      <c r="AO21" s="17"/>
+      <c r="AP21" s="17"/>
+      <c r="AQ21" s="17"/>
+      <c r="AR21" s="17"/>
+      <c r="AS21" s="17"/>
+      <c r="AT21" s="17"/>
+      <c r="AU21" s="17"/>
+      <c r="AV21" s="17"/>
+      <c r="AW21" s="17"/>
+      <c r="AX21" s="17"/>
+      <c r="AY21" s="17"/>
+      <c r="AZ21" s="17"/>
+      <c r="BA21" s="17"/>
+      <c r="BB21" s="17"/>
+      <c r="BC21" s="17"/>
+      <c r="BD21" s="17"/>
+      <c r="BE21" s="17"/>
+      <c r="BF21" s="17"/>
+      <c r="BG21" s="17"/>
+      <c r="BH21" s="17"/>
+      <c r="BI21" s="17"/>
+      <c r="BJ21" s="17"/>
+      <c r="BK21" s="17"/>
+      <c r="BL21" s="17"/>
+      <c r="BM21" s="17"/>
+      <c r="BN21" s="17"/>
+      <c r="BO21" s="17"/>
+      <c r="BP21" s="17"/>
+      <c r="BQ21" s="17"/>
+      <c r="BR21" s="17"/>
+      <c r="BS21" s="17"/>
+      <c r="BT21" s="17"/>
+      <c r="BU21" s="17"/>
+      <c r="BV21" s="17"/>
+      <c r="BW21" s="17"/>
+      <c r="BX21" s="17"/>
+      <c r="BY21" s="17"/>
+      <c r="BZ21" s="17"/>
+      <c r="CA21" s="17"/>
+      <c r="CB21" s="17"/>
+      <c r="CC21" s="17"/>
+      <c r="CD21" s="17"/>
+    </row>
+    <row r="22" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>75</v>
       </c>
@@ -5161,8 +6224,52 @@
       <c r="AJ22" s="8"/>
       <c r="AK22" s="8"/>
       <c r="AL22" s="8"/>
-    </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM22" s="17"/>
+      <c r="AN22" s="17"/>
+      <c r="AO22" s="17"/>
+      <c r="AP22" s="17"/>
+      <c r="AQ22" s="17"/>
+      <c r="AR22" s="17"/>
+      <c r="AS22" s="17"/>
+      <c r="AT22" s="17"/>
+      <c r="AU22" s="17"/>
+      <c r="AV22" s="17"/>
+      <c r="AW22" s="17"/>
+      <c r="AX22" s="17"/>
+      <c r="AY22" s="17"/>
+      <c r="AZ22" s="17"/>
+      <c r="BA22" s="17"/>
+      <c r="BB22" s="17"/>
+      <c r="BC22" s="17"/>
+      <c r="BD22" s="17"/>
+      <c r="BE22" s="17"/>
+      <c r="BF22" s="17"/>
+      <c r="BG22" s="17"/>
+      <c r="BH22" s="17"/>
+      <c r="BI22" s="17"/>
+      <c r="BJ22" s="17"/>
+      <c r="BK22" s="17"/>
+      <c r="BL22" s="17"/>
+      <c r="BM22" s="17"/>
+      <c r="BN22" s="17"/>
+      <c r="BO22" s="17"/>
+      <c r="BP22" s="17"/>
+      <c r="BQ22" s="17"/>
+      <c r="BR22" s="17"/>
+      <c r="BS22" s="17"/>
+      <c r="BT22" s="17"/>
+      <c r="BU22" s="17"/>
+      <c r="BV22" s="17"/>
+      <c r="BW22" s="17"/>
+      <c r="BX22" s="17"/>
+      <c r="BY22" s="17"/>
+      <c r="BZ22" s="17"/>
+      <c r="CA22" s="17"/>
+      <c r="CB22" s="17"/>
+      <c r="CC22" s="17"/>
+      <c r="CD22" s="17"/>
+    </row>
+    <row r="23" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>76</v>
       </c>
@@ -5203,8 +6310,52 @@
       <c r="AJ23" s="8"/>
       <c r="AK23" s="8"/>
       <c r="AL23" s="8"/>
-    </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM23" s="17"/>
+      <c r="AN23" s="17"/>
+      <c r="AO23" s="17"/>
+      <c r="AP23" s="17"/>
+      <c r="AQ23" s="17"/>
+      <c r="AR23" s="17"/>
+      <c r="AS23" s="17"/>
+      <c r="AT23" s="17"/>
+      <c r="AU23" s="17"/>
+      <c r="AV23" s="17"/>
+      <c r="AW23" s="17"/>
+      <c r="AX23" s="17"/>
+      <c r="AY23" s="17"/>
+      <c r="AZ23" s="17"/>
+      <c r="BA23" s="17"/>
+      <c r="BB23" s="17"/>
+      <c r="BC23" s="17"/>
+      <c r="BD23" s="17"/>
+      <c r="BE23" s="17"/>
+      <c r="BF23" s="17"/>
+      <c r="BG23" s="17"/>
+      <c r="BH23" s="17"/>
+      <c r="BI23" s="17"/>
+      <c r="BJ23" s="17"/>
+      <c r="BK23" s="17"/>
+      <c r="BL23" s="17"/>
+      <c r="BM23" s="17"/>
+      <c r="BN23" s="17"/>
+      <c r="BO23" s="17"/>
+      <c r="BP23" s="17"/>
+      <c r="BQ23" s="17"/>
+      <c r="BR23" s="17"/>
+      <c r="BS23" s="17"/>
+      <c r="BT23" s="17"/>
+      <c r="BU23" s="17"/>
+      <c r="BV23" s="17"/>
+      <c r="BW23" s="17"/>
+      <c r="BX23" s="17"/>
+      <c r="BY23" s="17"/>
+      <c r="BZ23" s="17"/>
+      <c r="CA23" s="17"/>
+      <c r="CB23" s="17"/>
+      <c r="CC23" s="17"/>
+      <c r="CD23" s="17"/>
+    </row>
+    <row r="24" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>77</v>
       </c>
@@ -5245,8 +6396,52 @@
       <c r="AJ24" s="8"/>
       <c r="AK24" s="8"/>
       <c r="AL24" s="8"/>
-    </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM24" s="17"/>
+      <c r="AN24" s="17"/>
+      <c r="AO24" s="17"/>
+      <c r="AP24" s="17"/>
+      <c r="AQ24" s="17"/>
+      <c r="AR24" s="17"/>
+      <c r="AS24" s="17"/>
+      <c r="AT24" s="17"/>
+      <c r="AU24" s="17"/>
+      <c r="AV24" s="17"/>
+      <c r="AW24" s="17"/>
+      <c r="AX24" s="17"/>
+      <c r="AY24" s="17"/>
+      <c r="AZ24" s="17"/>
+      <c r="BA24" s="17"/>
+      <c r="BB24" s="17"/>
+      <c r="BC24" s="17"/>
+      <c r="BD24" s="17"/>
+      <c r="BE24" s="17"/>
+      <c r="BF24" s="17"/>
+      <c r="BG24" s="17"/>
+      <c r="BH24" s="17"/>
+      <c r="BI24" s="17"/>
+      <c r="BJ24" s="17"/>
+      <c r="BK24" s="17"/>
+      <c r="BL24" s="17"/>
+      <c r="BM24" s="17"/>
+      <c r="BN24" s="17"/>
+      <c r="BO24" s="17"/>
+      <c r="BP24" s="17"/>
+      <c r="BQ24" s="17"/>
+      <c r="BR24" s="17"/>
+      <c r="BS24" s="17"/>
+      <c r="BT24" s="17"/>
+      <c r="BU24" s="17"/>
+      <c r="BV24" s="17"/>
+      <c r="BW24" s="17"/>
+      <c r="BX24" s="17"/>
+      <c r="BY24" s="17"/>
+      <c r="BZ24" s="17"/>
+      <c r="CA24" s="17"/>
+      <c r="CB24" s="17"/>
+      <c r="CC24" s="17"/>
+      <c r="CD24" s="17"/>
+    </row>
+    <row r="25" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>78</v>
       </c>
@@ -5278,8 +6473,52 @@
       <c r="AJ25" s="8"/>
       <c r="AK25" s="8"/>
       <c r="AL25" s="8"/>
-    </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM25" s="17"/>
+      <c r="AN25" s="17"/>
+      <c r="AO25" s="17"/>
+      <c r="AP25" s="17"/>
+      <c r="AQ25" s="17"/>
+      <c r="AR25" s="17"/>
+      <c r="AS25" s="17"/>
+      <c r="AT25" s="17"/>
+      <c r="AU25" s="17"/>
+      <c r="AV25" s="17"/>
+      <c r="AW25" s="17"/>
+      <c r="AX25" s="17"/>
+      <c r="AY25" s="17"/>
+      <c r="AZ25" s="17"/>
+      <c r="BA25" s="17"/>
+      <c r="BB25" s="17"/>
+      <c r="BC25" s="17"/>
+      <c r="BD25" s="17"/>
+      <c r="BE25" s="17"/>
+      <c r="BF25" s="17"/>
+      <c r="BG25" s="17"/>
+      <c r="BH25" s="17"/>
+      <c r="BI25" s="17"/>
+      <c r="BJ25" s="17"/>
+      <c r="BK25" s="17"/>
+      <c r="BL25" s="17"/>
+      <c r="BM25" s="17"/>
+      <c r="BN25" s="17"/>
+      <c r="BO25" s="17"/>
+      <c r="BP25" s="17"/>
+      <c r="BQ25" s="17"/>
+      <c r="BR25" s="17"/>
+      <c r="BS25" s="17"/>
+      <c r="BT25" s="17"/>
+      <c r="BU25" s="17"/>
+      <c r="BV25" s="17"/>
+      <c r="BW25" s="17"/>
+      <c r="BX25" s="17"/>
+      <c r="BY25" s="17"/>
+      <c r="BZ25" s="17"/>
+      <c r="CA25" s="17"/>
+      <c r="CB25" s="17"/>
+      <c r="CC25" s="17"/>
+      <c r="CD25" s="17"/>
+    </row>
+    <row r="26" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>79</v>
       </c>
@@ -5320,39 +6559,216 @@
       <c r="AJ26" s="8"/>
       <c r="AK26" s="8"/>
       <c r="AL26" s="8"/>
-    </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM26" s="17"/>
+      <c r="AN26" s="17"/>
+      <c r="AO26" s="17"/>
+      <c r="AP26" s="17"/>
+      <c r="AQ26" s="17"/>
+      <c r="AR26" s="17"/>
+      <c r="AS26" s="17"/>
+      <c r="AT26" s="17"/>
+      <c r="AU26" s="17"/>
+      <c r="AV26" s="17"/>
+      <c r="AW26" s="17"/>
+      <c r="AX26" s="17"/>
+      <c r="AY26" s="17"/>
+      <c r="AZ26" s="17"/>
+      <c r="BA26" s="17"/>
+      <c r="BB26" s="17"/>
+      <c r="BC26" s="17"/>
+      <c r="BD26" s="17"/>
+      <c r="BE26" s="17"/>
+      <c r="BF26" s="17"/>
+      <c r="BG26" s="17"/>
+      <c r="BH26" s="17"/>
+      <c r="BI26" s="17"/>
+      <c r="BJ26" s="17"/>
+      <c r="BK26" s="17"/>
+      <c r="BL26" s="17"/>
+      <c r="BM26" s="17"/>
+      <c r="BN26" s="17"/>
+      <c r="BO26" s="17"/>
+      <c r="BP26" s="17"/>
+      <c r="BQ26" s="17"/>
+      <c r="BR26" s="17"/>
+      <c r="BS26" s="17"/>
+      <c r="BT26" s="17"/>
+      <c r="BU26" s="17"/>
+      <c r="BV26" s="17"/>
+      <c r="BW26" s="17"/>
+      <c r="BX26" s="17"/>
+      <c r="BY26" s="17"/>
+      <c r="BZ26" s="17"/>
+      <c r="CA26" s="17"/>
+      <c r="CB26" s="17"/>
+      <c r="CC26" s="17"/>
+      <c r="CD26" s="17"/>
+    </row>
+    <row r="27" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AT27" s="17"/>
+      <c r="AU27" s="17"/>
+      <c r="AV27" s="17"/>
+      <c r="AW27" s="17"/>
+      <c r="AX27" s="17"/>
+      <c r="AY27" s="17"/>
+      <c r="AZ27" s="17"/>
+      <c r="BA27" s="17"/>
+      <c r="BB27" s="17"/>
+      <c r="BC27" s="17"/>
+      <c r="BD27" s="17"/>
+      <c r="BE27" s="17"/>
+      <c r="BF27" s="17"/>
+      <c r="BG27" s="17"/>
+      <c r="BH27" s="17"/>
+      <c r="BI27" s="17"/>
+      <c r="BJ27" s="17"/>
+      <c r="BK27" s="17"/>
+      <c r="BL27" s="17"/>
+      <c r="BM27" s="17"/>
+      <c r="BN27" s="17"/>
+      <c r="BO27" s="17"/>
+      <c r="BP27" s="17"/>
+      <c r="BQ27" s="17"/>
+      <c r="BR27" s="17"/>
+      <c r="BS27" s="17"/>
+      <c r="BT27" s="17"/>
+      <c r="BU27" s="17"/>
+      <c r="BV27" s="17"/>
+      <c r="BW27" s="17"/>
+      <c r="BX27" s="17"/>
+      <c r="BY27" s="17"/>
+      <c r="BZ27" s="17"/>
+      <c r="CA27" s="17"/>
+      <c r="CB27" s="17"/>
+      <c r="CC27" s="17"/>
+      <c r="CD27" s="17"/>
+    </row>
+    <row r="28" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="BG28" s="17"/>
+      <c r="BH28" s="17"/>
+      <c r="BI28" s="17"/>
+      <c r="BJ28" s="17"/>
+      <c r="BK28" s="17"/>
+      <c r="BL28" s="17"/>
+      <c r="BM28" s="17"/>
+      <c r="BN28" s="17"/>
+      <c r="BO28" s="17"/>
+      <c r="BP28" s="17"/>
+      <c r="BQ28" s="17"/>
+      <c r="BR28" s="17"/>
+      <c r="BS28" s="17"/>
+      <c r="BT28" s="17"/>
+      <c r="BU28" s="17"/>
+      <c r="BV28" s="17"/>
+      <c r="BW28" s="17"/>
+      <c r="BX28" s="17"/>
+      <c r="BY28" s="17"/>
+      <c r="BZ28" s="17"/>
+      <c r="CA28" s="17"/>
+      <c r="CB28" s="17"/>
+      <c r="CC28" s="17"/>
+      <c r="CD28" s="17"/>
+    </row>
+    <row r="29" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="BG29" s="17"/>
+      <c r="BH29" s="17"/>
+      <c r="BI29" s="17"/>
+      <c r="BJ29" s="17"/>
+      <c r="BK29" s="17"/>
+      <c r="BL29" s="17"/>
+      <c r="BM29" s="17"/>
+      <c r="BN29" s="17"/>
+      <c r="BO29" s="17"/>
+      <c r="BP29" s="17"/>
+      <c r="BQ29" s="17"/>
+      <c r="BR29" s="17"/>
+      <c r="BS29" s="17"/>
+      <c r="BT29" s="17"/>
+      <c r="BU29" s="17"/>
+      <c r="BV29" s="17"/>
+      <c r="BW29" s="17"/>
+      <c r="BX29" s="17"/>
+      <c r="BY29" s="17"/>
+      <c r="BZ29" s="17"/>
+      <c r="CA29" s="17"/>
+      <c r="CB29" s="17"/>
+      <c r="CC29" s="17"/>
+      <c r="CD29" s="17"/>
+    </row>
+    <row r="30" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="BG30" s="17"/>
+      <c r="BH30" s="17"/>
+      <c r="BI30" s="17"/>
+      <c r="BJ30" s="17"/>
+      <c r="BK30" s="17"/>
+      <c r="BL30" s="17"/>
+      <c r="BM30" s="17"/>
+      <c r="BN30" s="17"/>
+      <c r="BO30" s="17"/>
+      <c r="BP30" s="17"/>
+      <c r="BQ30" s="17"/>
+      <c r="BR30" s="17"/>
+      <c r="BS30" s="17"/>
+      <c r="BT30" s="17"/>
+      <c r="BU30" s="17"/>
+      <c r="BV30" s="17"/>
+      <c r="BW30" s="17"/>
+      <c r="BX30" s="17"/>
+      <c r="BY30" s="17"/>
+      <c r="BZ30" s="17"/>
+      <c r="CA30" s="17"/>
+      <c r="CB30" s="17"/>
+      <c r="CC30" s="17"/>
+      <c r="CD30" s="17"/>
+    </row>
+    <row r="31" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:82" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>85</v>
       </c>
       <c r="F32" t="s">
         <v>159</v>
       </c>
+      <c r="BG32" s="17"/>
+      <c r="BH32" s="17"/>
+      <c r="BI32" s="17"/>
+      <c r="BJ32" s="17"/>
+      <c r="BK32" s="17"/>
+      <c r="BL32" s="17"/>
+      <c r="BM32" s="17"/>
+      <c r="BN32" s="17"/>
+      <c r="BO32" s="17"/>
+      <c r="BP32" s="17"/>
+      <c r="BQ32" s="17"/>
+      <c r="BR32" s="17"/>
+      <c r="BS32" s="17"/>
+      <c r="BT32" s="17"/>
+      <c r="BU32" s="17"/>
+      <c r="BV32" s="17"/>
+      <c r="BW32" s="17"/>
+      <c r="BX32" s="17"/>
+      <c r="BY32" s="17"/>
+      <c r="BZ32" s="17"/>
+      <c r="CA32" s="17"/>
+      <c r="CB32" s="17"/>
+      <c r="CC32" s="17"/>
+      <c r="CD32" s="17"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
@@ -5381,6 +6797,9 @@
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>88</v>
+      </c>
+      <c r="I35" s="11" t="s">
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Register cell module to new account
Register cell module to new account
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{005D967E-CB2C-DE41-BEE0-1C2937F8BFB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C469DB8-724D-3740-AF3D-C15EEEA04E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="328">
   <si>
     <t>Box Number</t>
   </si>
@@ -1015,6 +1015,12 @@
   </si>
   <si>
     <t>COMMONSENSES2@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>COMMONSENSES3@LISTSERV.NEU.EDU </t>
+  </si>
+  <si>
+    <t>COMMONSENSES4@LISTSERV.NEU.EDU</t>
   </si>
 </sst>
 </file>
@@ -4253,7 +4259,9 @@
       <c r="N43" s="2">
         <v>45793</v>
       </c>
-      <c r="O43" s="2"/>
+      <c r="O43" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="Q43" s="2"/>
       <c r="Y43" s="2"/>
       <c r="Z43" s="2"/>
@@ -4299,7 +4307,9 @@
       <c r="N44" s="2">
         <v>45793</v>
       </c>
-      <c r="O44" s="2"/>
+      <c r="O44" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="Q44" s="2"/>
       <c r="Y44" s="2"/>
       <c r="Z44" s="2"/>
@@ -4345,7 +4355,9 @@
       <c r="N45" s="2">
         <v>45793</v>
       </c>
-      <c r="O45" s="2"/>
+      <c r="O45" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="Q45" s="2"/>
       <c r="Y45" s="2"/>
       <c r="Z45" s="2"/>
@@ -4391,7 +4403,9 @@
       <c r="N46" s="2">
         <v>45793</v>
       </c>
-      <c r="O46" s="2"/>
+      <c r="O46" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="Q46" s="2"/>
       <c r="Y46" s="2"/>
       <c r="Z46" s="2"/>
@@ -4437,7 +4451,9 @@
       <c r="N47" s="2">
         <v>45793</v>
       </c>
-      <c r="O47" s="2"/>
+      <c r="O47" s="2" t="s">
+        <v>326</v>
+      </c>
       <c r="Q47" s="2"/>
       <c r="Y47" s="2"/>
       <c r="Z47" s="2"/>
@@ -4483,7 +4499,9 @@
       <c r="N48" s="2">
         <v>45793</v>
       </c>
-      <c r="O48" s="2"/>
+      <c r="O48" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="Q48" s="2"/>
       <c r="Y48" s="2"/>
       <c r="Z48" s="2"/>
@@ -4529,7 +4547,9 @@
       <c r="N49" s="2">
         <v>45793</v>
       </c>
-      <c r="O49" s="2"/>
+      <c r="O49" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="Q49" s="2"/>
       <c r="Y49" s="2"/>
       <c r="Z49" s="2"/>
@@ -4575,7 +4595,9 @@
       <c r="N50" s="2">
         <v>45793</v>
       </c>
-      <c r="O50" s="2"/>
+      <c r="O50" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="Q50" s="2"/>
       <c r="Y50" s="2"/>
       <c r="Z50" s="2"/>
@@ -4621,7 +4643,9 @@
       <c r="N51" s="2">
         <v>45793</v>
       </c>
-      <c r="O51" s="2"/>
+      <c r="O51" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="Q51" s="2"/>
       <c r="W51" t="s">
         <v>241</v>
@@ -4670,7 +4694,9 @@
       <c r="N52" s="2">
         <v>45793</v>
       </c>
-      <c r="O52" s="2"/>
+      <c r="O52" s="2" t="s">
+        <v>327</v>
+      </c>
       <c r="Q52" s="2"/>
       <c r="Y52" s="2"/>
       <c r="Z52" s="2"/>

</xml_diff>

<commit_message>
Register cell modules to new accounts
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C469DB8-724D-3740-AF3D-C15EEEA04E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB92964-ECE1-4A44-8DA8-6D6E5817A7C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1010" uniqueCount="333">
   <si>
     <t>Box Number</t>
   </si>
@@ -1021,6 +1021,21 @@
   </si>
   <si>
     <t>COMMONSENSES4@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>P044AD3487D35K8</t>
+  </si>
+  <si>
+    <t>BlueHill2_7</t>
+  </si>
+  <si>
+    <t>BlueHill2_8</t>
+  </si>
+  <si>
+    <t>BlueHill2_9</t>
+  </si>
+  <si>
+    <t>Changed the RTC battery on 10/09/2025</t>
   </si>
 </sst>
 </file>
@@ -4599,6 +4614,9 @@
         <v>327</v>
       </c>
       <c r="Q50" s="2"/>
+      <c r="W50" t="s">
+        <v>332</v>
+      </c>
       <c r="Y50" s="2"/>
       <c r="Z50" s="2"/>
     </row>
@@ -4781,6 +4799,9 @@
       </c>
       <c r="L54" s="4" t="s">
         <v>107</v>
+      </c>
+      <c r="M54" t="s">
+        <v>329</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -4820,6 +4841,12 @@
       <c r="K55" t="s">
         <v>250</v>
       </c>
+      <c r="L55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="M55" t="s">
+        <v>330</v>
+      </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="Q55" s="2"/>
@@ -4852,6 +4879,15 @@
         <v>109</v>
       </c>
       <c r="I56" s="4"/>
+      <c r="K56" s="4" t="s">
+        <v>328</v>
+      </c>
+      <c r="L56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="M56" t="s">
+        <v>331</v>
+      </c>
       <c r="N56" s="2"/>
       <c r="O56" s="2"/>
       <c r="Q56" s="2"/>

</xml_diff>

<commit_message>
Updated the deployment tracker sheet with dates and log in information
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{800B4935-DE88-A943-8EB3-18085BCB21B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{437AE354-6AE3-CA4A-BEF0-56AD356B62C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8460" yWindow="1180" windowWidth="30240" windowHeight="18880" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20520" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="902" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="294">
   <si>
     <t>Box Number</t>
   </si>
@@ -862,6 +862,63 @@
   </si>
   <si>
     <t>08/23/25</t>
+  </si>
+  <si>
+    <t>Account name</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>data volume/month</t>
+  </si>
+  <si>
+    <t>Box Numbers</t>
+  </si>
+  <si>
+    <t>envsensorslab@gmail.com</t>
+  </si>
+  <si>
+    <t>Envlab257</t>
+  </si>
+  <si>
+    <t>500 MB</t>
+  </si>
+  <si>
+    <t>COMMONSENSES1@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>Envsensorslab257</t>
+  </si>
+  <si>
+    <t>100 MB</t>
+  </si>
+  <si>
+    <t>32 to 36</t>
+  </si>
+  <si>
+    <t>COMMONSENSES2@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>37 to 41</t>
+  </si>
+  <si>
+    <t>COMMONSENSES3@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>42 to 46</t>
+  </si>
+  <si>
+    <t>COMMONSENSES4@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>47 to 51</t>
+  </si>
+  <si>
+    <t>COMMONSENSES5@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>52 to 55</t>
   </si>
 </sst>
 </file>
@@ -869,7 +926,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -982,7 +1039,7 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="20" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1320,7 +1377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAF163E4-59DB-9747-B16B-025799580D26}">
-  <dimension ref="A1:AD56"/>
+  <dimension ref="A1:AF56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.1640625" bestFit="1" customWidth="1"/>
@@ -2396,7 +2453,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="17" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>70</v>
       </c>
@@ -2461,7 +2518,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="18" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>71</v>
       </c>
@@ -2529,7 +2586,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="19" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>72</v>
       </c>
@@ -2594,7 +2651,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="20" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>73</v>
       </c>
@@ -2659,7 +2716,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="21" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>74</v>
       </c>
@@ -2724,7 +2781,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="22" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>75</v>
       </c>
@@ -2789,7 +2846,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="23" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>76</v>
       </c>
@@ -2848,7 +2905,7 @@
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
     </row>
-    <row r="24" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>77</v>
       </c>
@@ -2907,7 +2964,7 @@
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
     </row>
-    <row r="25" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>78</v>
       </c>
@@ -2965,8 +3022,20 @@
       </c>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
-    </row>
-    <row r="26" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC25" t="s">
+        <v>275</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>276</v>
+      </c>
+      <c r="AE25" t="s">
+        <v>277</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="26" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>79</v>
       </c>
@@ -3024,8 +3093,17 @@
       </c>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
-    </row>
-    <row r="27" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC26" t="s">
+        <v>279</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>280</v>
+      </c>
+      <c r="AE26" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="27" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A27" s="4" t="s">
         <v>80</v>
       </c>
@@ -3085,8 +3163,20 @@
       </c>
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
-    </row>
-    <row r="28" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC27" t="s">
+        <v>282</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>283</v>
+      </c>
+      <c r="AE27" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF27" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="28" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A28" s="4" t="s">
         <v>81</v>
       </c>
@@ -3149,8 +3239,20 @@
       </c>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
-    </row>
-    <row r="29" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC28" t="s">
+        <v>286</v>
+      </c>
+      <c r="AD28" t="s">
+        <v>283</v>
+      </c>
+      <c r="AE28" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF28" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="29" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>82</v>
       </c>
@@ -3210,8 +3312,20 @@
       </c>
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
-    </row>
-    <row r="30" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC29" t="s">
+        <v>288</v>
+      </c>
+      <c r="AD29" t="s">
+        <v>283</v>
+      </c>
+      <c r="AE29" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF29" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="30" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>83</v>
       </c>
@@ -3271,8 +3385,20 @@
       </c>
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
-    </row>
-    <row r="31" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC30" t="s">
+        <v>290</v>
+      </c>
+      <c r="AD30" t="s">
+        <v>283</v>
+      </c>
+      <c r="AE30" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF30" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="31" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>84</v>
       </c>
@@ -3324,8 +3450,20 @@
       <c r="T31" s="9"/>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
-    </row>
-    <row r="32" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="AC31" t="s">
+        <v>292</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>283</v>
+      </c>
+      <c r="AE31" t="s">
+        <v>284</v>
+      </c>
+      <c r="AF31" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="32" spans="1:32" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>85</v>
       </c>
@@ -3426,7 +3564,12 @@
       <c r="N33" s="2">
         <v>45793</v>
       </c>
-      <c r="P33" s="2"/>
+      <c r="O33" t="s">
+        <v>168</v>
+      </c>
+      <c r="P33" s="12">
+        <v>45874</v>
+      </c>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
     </row>
@@ -3470,7 +3613,12 @@
       <c r="N34" s="2">
         <v>45793</v>
       </c>
-      <c r="P34" s="2"/>
+      <c r="O34" t="s">
+        <v>168</v>
+      </c>
+      <c r="P34" s="12">
+        <v>45874</v>
+      </c>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
     </row>
@@ -3514,7 +3662,12 @@
       <c r="N35" s="2">
         <v>45793</v>
       </c>
-      <c r="P35" s="2"/>
+      <c r="O35" t="s">
+        <v>168</v>
+      </c>
+      <c r="P35" s="12">
+        <v>45874</v>
+      </c>
       <c r="X35" s="2"/>
       <c r="Y35" s="2"/>
     </row>
@@ -3558,7 +3711,12 @@
       <c r="N36" s="2">
         <v>45793</v>
       </c>
-      <c r="P36" s="2"/>
+      <c r="O36" t="s">
+        <v>168</v>
+      </c>
+      <c r="P36" s="12">
+        <v>45874</v>
+      </c>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
     </row>
@@ -3602,7 +3760,12 @@
       <c r="N37" s="2">
         <v>45793</v>
       </c>
-      <c r="P37" s="2"/>
+      <c r="O37" t="s">
+        <v>168</v>
+      </c>
+      <c r="P37" s="12">
+        <v>45874</v>
+      </c>
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
     </row>
@@ -3646,7 +3809,12 @@
       <c r="N38" s="2">
         <v>45793</v>
       </c>
-      <c r="P38" s="2"/>
+      <c r="O38" t="s">
+        <v>168</v>
+      </c>
+      <c r="P38" s="12">
+        <v>45874</v>
+      </c>
       <c r="V38" t="s">
         <v>214</v>
       </c>
@@ -3691,7 +3859,12 @@
       <c r="N39" s="2">
         <v>45793</v>
       </c>
-      <c r="P39" s="2"/>
+      <c r="O39" t="s">
+        <v>168</v>
+      </c>
+      <c r="P39" s="12">
+        <v>45874</v>
+      </c>
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
     </row>
@@ -3733,7 +3906,12 @@
       <c r="N40" s="2">
         <v>45793</v>
       </c>
-      <c r="P40" s="2"/>
+      <c r="O40" t="s">
+        <v>168</v>
+      </c>
+      <c r="P40" s="12">
+        <v>45874</v>
+      </c>
       <c r="X40" s="2"/>
       <c r="Y40" s="2"/>
     </row>
@@ -3775,7 +3953,12 @@
       <c r="N41" s="2">
         <v>45793</v>
       </c>
-      <c r="P41" s="2"/>
+      <c r="O41" t="s">
+        <v>168</v>
+      </c>
+      <c r="P41" s="12">
+        <v>45874</v>
+      </c>
       <c r="V41" t="s">
         <v>241</v>
       </c>
@@ -3820,7 +4003,12 @@
       <c r="N42" s="2">
         <v>45793</v>
       </c>
-      <c r="P42" s="2"/>
+      <c r="O42" t="s">
+        <v>168</v>
+      </c>
+      <c r="P42" s="12">
+        <v>45874</v>
+      </c>
       <c r="V42" t="s">
         <v>242</v>
       </c>
@@ -3865,7 +4053,12 @@
       <c r="N43" s="2">
         <v>45793</v>
       </c>
-      <c r="P43" s="2"/>
+      <c r="O43" t="s">
+        <v>168</v>
+      </c>
+      <c r="P43" s="12">
+        <v>45874</v>
+      </c>
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
     </row>
@@ -3907,7 +4100,12 @@
       <c r="N44" s="2">
         <v>45793</v>
       </c>
-      <c r="P44" s="2"/>
+      <c r="O44" t="s">
+        <v>168</v>
+      </c>
+      <c r="P44" s="12">
+        <v>45874</v>
+      </c>
       <c r="X44" s="2"/>
       <c r="Y44" s="2"/>
     </row>
@@ -3949,7 +4147,12 @@
       <c r="N45" s="2">
         <v>45793</v>
       </c>
-      <c r="P45" s="2"/>
+      <c r="O45" t="s">
+        <v>168</v>
+      </c>
+      <c r="P45" s="12">
+        <v>45874</v>
+      </c>
       <c r="X45" s="2"/>
       <c r="Y45" s="2"/>
     </row>
@@ -3991,7 +4194,12 @@
       <c r="N46" s="2">
         <v>45793</v>
       </c>
-      <c r="P46" s="2"/>
+      <c r="O46" t="s">
+        <v>168</v>
+      </c>
+      <c r="P46" s="12">
+        <v>45874</v>
+      </c>
       <c r="X46" s="2"/>
       <c r="Y46" s="2"/>
     </row>
@@ -4033,7 +4241,12 @@
       <c r="N47" s="2">
         <v>45793</v>
       </c>
-      <c r="P47" s="2"/>
+      <c r="O47" t="s">
+        <v>168</v>
+      </c>
+      <c r="P47" s="12">
+        <v>45874</v>
+      </c>
       <c r="X47" s="2"/>
       <c r="Y47" s="2"/>
     </row>
@@ -4075,7 +4288,12 @@
       <c r="N48" s="2">
         <v>45793</v>
       </c>
-      <c r="P48" s="2"/>
+      <c r="O48" t="s">
+        <v>168</v>
+      </c>
+      <c r="P48" s="12">
+        <v>45874</v>
+      </c>
       <c r="X48" s="2"/>
       <c r="Y48" s="2"/>
     </row>
@@ -4117,7 +4335,12 @@
       <c r="N49" s="2">
         <v>45793</v>
       </c>
-      <c r="P49" s="2"/>
+      <c r="O49" t="s">
+        <v>168</v>
+      </c>
+      <c r="P49" s="12">
+        <v>45874</v>
+      </c>
       <c r="X49" s="2"/>
       <c r="Y49" s="2"/>
     </row>
@@ -4159,7 +4382,12 @@
       <c r="N50" s="2">
         <v>45793</v>
       </c>
-      <c r="P50" s="2"/>
+      <c r="O50" t="s">
+        <v>168</v>
+      </c>
+      <c r="P50" s="12">
+        <v>45874</v>
+      </c>
       <c r="X50" s="2"/>
       <c r="Y50" s="2"/>
     </row>
@@ -4201,7 +4429,12 @@
       <c r="N51" s="2">
         <v>45793</v>
       </c>
-      <c r="P51" s="2"/>
+      <c r="O51" t="s">
+        <v>168</v>
+      </c>
+      <c r="P51" s="12">
+        <v>45874</v>
+      </c>
       <c r="V51" t="s">
         <v>241</v>
       </c>
@@ -4246,7 +4479,12 @@
       <c r="N52" s="2">
         <v>45793</v>
       </c>
-      <c r="P52" s="2"/>
+      <c r="O52" t="s">
+        <v>168</v>
+      </c>
+      <c r="P52" s="12">
+        <v>45874</v>
+      </c>
       <c r="X52" s="2"/>
       <c r="Y52" s="2"/>
     </row>
@@ -4288,7 +4526,12 @@
       <c r="N53" s="2">
         <v>45793</v>
       </c>
-      <c r="P53" s="2"/>
+      <c r="O53" t="s">
+        <v>168</v>
+      </c>
+      <c r="P53" s="12">
+        <v>45874</v>
+      </c>
       <c r="X53" s="2"/>
       <c r="Y53" s="2"/>
     </row>

</xml_diff>

<commit_message>
Updated the states of box 37, 42, and 43
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30D0F393-C86F-C44B-BC3D-2BE4CA266D45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB3845B-270C-F64A-875F-119BADCF104B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20520" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="301">
   <si>
     <t>Box Number</t>
   </si>
@@ -919,6 +919,27 @@
   </si>
   <si>
     <t>52 to 55</t>
+  </si>
+  <si>
+    <t>Changed the RTC battery on 8/01/2025, after the failure of the deployment on 10/13/2025, followed the final pre-deployment checlist and recerified the box on 10/17/2025</t>
+  </si>
+  <si>
+    <t>The noise sensor light is broken but the sensor works well. Checked on 10/17/2025, after the failure of the deployment on 10/13/2025, followed the final pre-deployment checlist and recerified the box on 10/17/2025</t>
+  </si>
+  <si>
+    <t>after the failure of the deployment on 10/13/2025, followed the final pre-deployment checlist and recerified the box on 10/17/2025</t>
+  </si>
+  <si>
+    <t>e00fce686f304c6ebe0392cf</t>
+  </si>
+  <si>
+    <t>P044AD3488NMAWG</t>
+  </si>
+  <si>
+    <t>e00fce68be63790f452e32f2</t>
+  </si>
+  <si>
+    <t>P044AD3487D35K8</t>
   </si>
 </sst>
 </file>
@@ -3816,7 +3837,7 @@
         <v>45874</v>
       </c>
       <c r="V38" t="s">
-        <v>214</v>
+        <v>294</v>
       </c>
       <c r="X38" s="2"/>
       <c r="Y38" s="2"/>
@@ -4059,6 +4080,9 @@
       <c r="P43" s="12">
         <v>45874</v>
       </c>
+      <c r="V43" t="s">
+        <v>295</v>
+      </c>
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
     </row>
@@ -4106,6 +4130,9 @@
       <c r="P44" s="12">
         <v>45874</v>
       </c>
+      <c r="V44" t="s">
+        <v>296</v>
+      </c>
       <c r="X44" s="2"/>
       <c r="Y44" s="2"/>
     </row>
@@ -4561,6 +4588,12 @@
         <v>107</v>
       </c>
       <c r="I54" s="4"/>
+      <c r="J54" t="s">
+        <v>297</v>
+      </c>
+      <c r="K54" t="s">
+        <v>298</v>
+      </c>
       <c r="N54" s="2"/>
       <c r="P54" s="2"/>
       <c r="X54" s="2"/>
@@ -4629,6 +4662,12 @@
         <v>109</v>
       </c>
       <c r="I56" s="4"/>
+      <c r="J56" t="s">
+        <v>299</v>
+      </c>
+      <c r="K56" t="s">
+        <v>300</v>
+      </c>
       <c r="N56" s="2"/>
       <c r="P56" s="2"/>
       <c r="X56" s="2"/>

</xml_diff>

<commit_message>
updated the ID and serial number of cell module 52, 53, 54, and 55
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FB3845B-270C-F64A-875F-119BADCF104B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD9C6B3-971C-4E4F-B80B-19457D015764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="956" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="307">
   <si>
     <t>Box Number</t>
   </si>
@@ -940,6 +940,24 @@
   </si>
   <si>
     <t>P044AD3487D35K8</t>
+  </si>
+  <si>
+    <t>BlueHill2_7</t>
+  </si>
+  <si>
+    <t>BlueHill2_8</t>
+  </si>
+  <si>
+    <t>BlueHill2_9</t>
+  </si>
+  <si>
+    <t>CS20250614</t>
+  </si>
+  <si>
+    <t>CS20250615</t>
+  </si>
+  <si>
+    <t>CS20250616</t>
   </si>
 </sst>
 </file>
@@ -4594,8 +4612,21 @@
       <c r="K54" t="s">
         <v>298</v>
       </c>
-      <c r="N54" s="2"/>
-      <c r="P54" s="2"/>
+      <c r="L54" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="M54" t="s">
+        <v>301</v>
+      </c>
+      <c r="N54" s="2">
+        <v>45794</v>
+      </c>
+      <c r="O54" t="s">
+        <v>304</v>
+      </c>
+      <c r="P54" s="12">
+        <v>45875</v>
+      </c>
       <c r="X54" s="2"/>
       <c r="Y54" s="2"/>
     </row>
@@ -4631,8 +4662,21 @@
       <c r="K55" t="s">
         <v>250</v>
       </c>
-      <c r="N55" s="2"/>
-      <c r="P55" s="2"/>
+      <c r="L55" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="M55" t="s">
+        <v>302</v>
+      </c>
+      <c r="N55" s="2">
+        <v>45795</v>
+      </c>
+      <c r="O55" t="s">
+        <v>305</v>
+      </c>
+      <c r="P55" s="12">
+        <v>45876</v>
+      </c>
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
     </row>
@@ -4668,8 +4712,21 @@
       <c r="K56" t="s">
         <v>300</v>
       </c>
-      <c r="N56" s="2"/>
-      <c r="P56" s="2"/>
+      <c r="L56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="M56" t="s">
+        <v>303</v>
+      </c>
+      <c r="N56" s="2">
+        <v>45796</v>
+      </c>
+      <c r="O56" t="s">
+        <v>306</v>
+      </c>
+      <c r="P56" s="12">
+        <v>45877</v>
+      </c>
       <c r="X56" s="2"/>
       <c r="Y56" s="2"/>
     </row>

</xml_diff>

<commit_message>
Correct the Arduino code version
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCD9C6B3-971C-4E4F-B80B-19457D015764}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7367F312-525C-FD42-9CAE-F6FD0E4EC9EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="965" uniqueCount="304">
   <si>
     <t>Box Number</t>
   </si>
@@ -949,15 +949,6 @@
   </si>
   <si>
     <t>BlueHill2_9</t>
-  </si>
-  <si>
-    <t>CS20250614</t>
-  </si>
-  <si>
-    <t>CS20250615</t>
-  </si>
-  <si>
-    <t>CS20250616</t>
   </si>
 </sst>
 </file>
@@ -4622,7 +4613,7 @@
         <v>45794</v>
       </c>
       <c r="O54" t="s">
-        <v>304</v>
+        <v>168</v>
       </c>
       <c r="P54" s="12">
         <v>45875</v>
@@ -4672,7 +4663,7 @@
         <v>45795</v>
       </c>
       <c r="O55" t="s">
-        <v>305</v>
+        <v>168</v>
       </c>
       <c r="P55" s="12">
         <v>45876</v>
@@ -4722,7 +4713,7 @@
         <v>45796</v>
       </c>
       <c r="O56" t="s">
-        <v>306</v>
+        <v>168</v>
       </c>
       <c r="P56" s="12">
         <v>45877</v>

</xml_diff>

<commit_message>
Updated the deployment tracker sheet
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1545D221-8841-F245-AEA3-355F0B318141}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6000B0F9-191C-3942-B8C0-F80B695CAAFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="307">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1036" uniqueCount="356">
   <si>
     <t>Box Number</t>
   </si>
@@ -453,9 +453,6 @@
     <t>Blue Hill @ Dacia</t>
   </si>
   <si>
-    <t xml:space="preserve">Quincy @ Dacia </t>
-  </si>
-  <si>
     <t>42.3142633, -71.0780641</t>
   </si>
   <si>
@@ -465,9 +462,6 @@
     <t>42.3157997, -71.0887256</t>
   </si>
   <si>
-    <t>Freedom  House Warren St</t>
-  </si>
-  <si>
     <t>42.3108226, -71.0832951</t>
   </si>
   <si>
@@ -498,9 +492,6 @@
     <t>42.308337, -71.0870204</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue Hill @ Columbia Road </t>
-  </si>
-  <si>
     <t>42.3039870, -71.0849420</t>
   </si>
   <si>
@@ -510,9 +501,6 @@
     <t>Blue Hill @ Seaver St</t>
   </si>
   <si>
-    <t xml:space="preserve">Elm Hill Ave </t>
-  </si>
-  <si>
     <t>42.3082767, -71.0886139</t>
   </si>
   <si>
@@ -723,9 +711,6 @@
     <t>42.3255823, -71.0817659</t>
   </si>
   <si>
-    <t>Warren @ Quincy</t>
-  </si>
-  <si>
     <t>42.3164061, -71.0826839</t>
   </si>
   <si>
@@ -738,9 +723,6 @@
     <t>08/27/2025</t>
   </si>
   <si>
-    <t>Daureath St</t>
-  </si>
-  <si>
     <t>42.3232051, -71.0805673</t>
   </si>
   <si>
@@ -750,9 +732,6 @@
     <t>42.3267352, -71.0755563</t>
   </si>
   <si>
-    <t>Lauydon St Farm</t>
-  </si>
-  <si>
     <t>42.3243402, -71.0723826</t>
   </si>
   <si>
@@ -958,6 +937,174 @@
   </si>
   <si>
     <t>COMMONSENSES7@LISTSERV.NEU.EDU</t>
+  </si>
+  <si>
+    <t>Warren @ Townsend/Quincy</t>
+  </si>
+  <si>
+    <t>Elm Hill Ave</t>
+  </si>
+  <si>
+    <t>Quincy @ Dacia</t>
+  </si>
+  <si>
+    <t>Blue Hill @ Columbia Road</t>
+  </si>
+  <si>
+    <t>Freedom House Warren St</t>
+  </si>
+  <si>
+    <t>Dunreath St</t>
+  </si>
+  <si>
+    <t>Langdon St Farm</t>
+  </si>
+  <si>
+    <t>10/31/2025</t>
+  </si>
+  <si>
+    <t>E. Cottage &amp; Batchelder St</t>
+  </si>
+  <si>
+    <t>42.32156. -71.06928</t>
+  </si>
+  <si>
+    <t>Normandy and Stanwood</t>
+  </si>
+  <si>
+    <t>42.30926, -71.08027</t>
+  </si>
+  <si>
+    <t>10/21/2025</t>
+  </si>
+  <si>
+    <t>Weldon St and Gannet St</t>
+  </si>
+  <si>
+    <t>42.31487, -71.08192</t>
+  </si>
+  <si>
+    <t>Homestead and Harold</t>
+  </si>
+  <si>
+    <t>42.31285, -71.09263</t>
+  </si>
+  <si>
+    <t>Ruthven and Humboldt</t>
+  </si>
+  <si>
+    <t>42.31267, -71.09006</t>
+  </si>
+  <si>
+    <t>Waumbeck and Warren</t>
+  </si>
+  <si>
+    <t>42.3133, -71.0837</t>
+  </si>
+  <si>
+    <t>Crawford (behind Crispus Attucks Children Center)</t>
+  </si>
+  <si>
+    <t>42.31387, -71.09082</t>
+  </si>
+  <si>
+    <t>10/17/2025</t>
+  </si>
+  <si>
+    <t>Elm Hill and Crawford</t>
+  </si>
+  <si>
+    <t>42.311667, -71.085833</t>
+  </si>
+  <si>
+    <t>Batchelder and Marshfield</t>
+  </si>
+  <si>
+    <t>42.322778, -71.069167</t>
+  </si>
+  <si>
+    <t>Hampden and Eustis</t>
+  </si>
+  <si>
+    <t>42.326944, -71.075278</t>
+  </si>
+  <si>
+    <t>Forest St and Vine St</t>
+  </si>
+  <si>
+    <t>42.32667, -71.0775</t>
+  </si>
+  <si>
+    <t>W.Cottage and Brook</t>
+  </si>
+  <si>
+    <t>42.32069, -71.07425</t>
+  </si>
+  <si>
+    <t>Washington St and Bishop Joe L. Smith</t>
+  </si>
+  <si>
+    <t>42.30620, -71.08143</t>
+  </si>
+  <si>
+    <t>10/24/2025</t>
+  </si>
+  <si>
+    <t>Children's Park (Intervale and Normandy)</t>
+  </si>
+  <si>
+    <t>42.31067, -71.07822</t>
+  </si>
+  <si>
+    <t>Bynoe Park</t>
+  </si>
+  <si>
+    <t>42.329, -71.076</t>
+  </si>
+  <si>
+    <t>Elm Hill and Cheney</t>
+  </si>
+  <si>
+    <t>42.31047,-71.08691</t>
+  </si>
+  <si>
+    <t>Quincy and Magnolia</t>
+  </si>
+  <si>
+    <t>42.31227, -71.07349</t>
+  </si>
+  <si>
+    <t>42.32404, -71.07928</t>
+  </si>
+  <si>
+    <t>Warren Pl</t>
+  </si>
+  <si>
+    <t>42.32787, -71.0820</t>
+  </si>
+  <si>
+    <t>Normandy and Seaver</t>
+  </si>
+  <si>
+    <t>42.30499, -71.08363</t>
+  </si>
+  <si>
+    <t>Winthrop Playground</t>
+  </si>
+  <si>
+    <t>42.31742, -71.07608</t>
+  </si>
+  <si>
+    <t>Dennis St Park</t>
+  </si>
+  <si>
+    <t>42.32258, -71.07489</t>
+  </si>
+  <si>
+    <t>Fayston and Perth</t>
+  </si>
+  <si>
+    <t>42.31298, -71.07653</t>
   </si>
 </sst>
 </file>
@@ -1447,34 +1594,34 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>177</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>181</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>185</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>1</v>
@@ -1483,13 +1630,13 @@
         <v>2</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>113</v>
@@ -1504,10 +1651,10 @@
         <v>112</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
@@ -1544,19 +1691,19 @@
         <v>4</v>
       </c>
       <c r="K2" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="L2" s="4" t="s">
         <v>55</v>
       </c>
       <c r="M2" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N2" s="2">
         <v>45793</v>
       </c>
       <c r="O2" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P2" s="2">
         <v>45793</v>
@@ -1606,34 +1753,34 @@
         <v>5</v>
       </c>
       <c r="K3" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="L3" s="4" t="s">
         <v>56</v>
       </c>
       <c r="M3" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N3" s="2">
         <v>45793</v>
       </c>
       <c r="O3" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P3" s="2">
         <v>45793</v>
       </c>
       <c r="Q3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="R3" s="5">
         <v>0.47499999999999998</v>
       </c>
       <c r="S3" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="T3" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="X3" s="2"/>
       <c r="Y3" s="2"/>
@@ -1668,19 +1815,19 @@
         <v>6</v>
       </c>
       <c r="K4" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>57</v>
       </c>
       <c r="M4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N4" s="2">
         <v>45793</v>
       </c>
       <c r="O4" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P4" s="2">
         <v>45793</v>
@@ -1703,7 +1850,7 @@
         <v>0</v>
       </c>
       <c r="AD4" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
@@ -1736,19 +1883,19 @@
         <v>7</v>
       </c>
       <c r="K5" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="L5" s="4" t="s">
         <v>58</v>
       </c>
       <c r="M5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N5" s="2">
         <v>45793</v>
       </c>
       <c r="O5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P5" s="2">
         <v>45793</v>
@@ -1768,10 +1915,10 @@
       <c r="X5" s="2"/>
       <c r="Y5" s="2"/>
       <c r="AC5" s="1" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="AD5" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.2">
@@ -1804,19 +1951,19 @@
         <v>8</v>
       </c>
       <c r="K6" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="L6" s="4" t="s">
         <v>59</v>
       </c>
       <c r="M6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N6" s="2">
         <v>45793</v>
       </c>
       <c r="O6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P6" s="2">
         <v>45793</v>
@@ -1836,10 +1983,10 @@
       <c r="X6" s="2"/>
       <c r="Y6" s="2"/>
       <c r="AC6" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="AD6" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="7" spans="1:30" x14ac:dyDescent="0.2">
@@ -1872,19 +2019,19 @@
         <v>9</v>
       </c>
       <c r="K7" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="L7" s="4" t="s">
         <v>60</v>
       </c>
       <c r="M7" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N7" s="2">
         <v>45793</v>
       </c>
       <c r="O7" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P7" s="2">
         <v>45793</v>
@@ -1904,10 +2051,10 @@
       <c r="X7" s="2"/>
       <c r="Y7" s="2"/>
       <c r="AC7" s="1" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="AD7" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
     </row>
     <row r="8" spans="1:30" x14ac:dyDescent="0.2">
@@ -1943,13 +2090,13 @@
         <v>61</v>
       </c>
       <c r="M8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N8" s="2">
         <v>45793</v>
       </c>
       <c r="O8" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P8" s="2">
         <v>45793</v>
@@ -1969,10 +2116,10 @@
       <c r="X8" s="2"/>
       <c r="Y8" s="2"/>
       <c r="AC8" s="1" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="AD8" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.2">
@@ -2008,13 +2155,13 @@
         <v>62</v>
       </c>
       <c r="M9" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N9" s="2">
         <v>45793</v>
       </c>
       <c r="O9" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P9" s="2">
         <v>45793</v>
@@ -2034,10 +2181,10 @@
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>
       <c r="AC9" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="AD9" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.2">
@@ -2073,42 +2220,42 @@
         <v>63</v>
       </c>
       <c r="M10" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N10" s="2">
         <v>45793</v>
       </c>
       <c r="O10" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P10" s="2">
         <v>45793</v>
       </c>
       <c r="Q10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="R10" s="5">
         <v>0.44444444444444442</v>
       </c>
       <c r="S10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="T10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="U10" s="10">
         <v>45968</v>
       </c>
       <c r="V10" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="X10" s="2"/>
       <c r="Y10" s="2"/>
       <c r="AC10" s="1" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="AD10" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.2">
@@ -2144,13 +2291,13 @@
         <v>64</v>
       </c>
       <c r="M11" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N11" s="2">
         <v>45793</v>
       </c>
       <c r="O11" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P11" s="2">
         <v>45793</v>
@@ -2170,10 +2317,10 @@
       <c r="X11" s="2"/>
       <c r="Y11" s="2"/>
       <c r="AC11" s="1" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="AD11" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.2">
@@ -2209,13 +2356,13 @@
         <v>65</v>
       </c>
       <c r="M12" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N12" s="2">
         <v>45793</v>
       </c>
       <c r="O12" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P12" s="2">
         <v>45793</v>
@@ -2227,18 +2374,18 @@
         <v>0.55347222222222225</v>
       </c>
       <c r="S12" t="s">
+        <v>139</v>
+      </c>
+      <c r="T12" t="s">
         <v>140</v>
-      </c>
-      <c r="T12" t="s">
-        <v>141</v>
       </c>
       <c r="X12" s="2"/>
       <c r="Y12" s="2"/>
       <c r="AC12" s="1" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="AD12" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="13" spans="1:30" x14ac:dyDescent="0.2">
@@ -2274,13 +2421,13 @@
         <v>66</v>
       </c>
       <c r="M13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N13" s="2">
         <v>45793</v>
       </c>
       <c r="O13" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P13" s="2">
         <v>45793</v>
@@ -2303,7 +2450,7 @@
         <v>3</v>
       </c>
       <c r="AD13" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="14" spans="1:30" x14ac:dyDescent="0.2">
@@ -2339,13 +2486,13 @@
         <v>67</v>
       </c>
       <c r="M14" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N14" s="2">
         <v>45826</v>
       </c>
       <c r="O14" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P14" s="2">
         <v>45826</v>
@@ -2368,7 +2515,7 @@
         <v>1</v>
       </c>
       <c r="AD14" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:30" x14ac:dyDescent="0.2">
@@ -2404,19 +2551,19 @@
         <v>68</v>
       </c>
       <c r="M15" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N15" s="2">
         <v>45793</v>
       </c>
       <c r="O15" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P15" s="2">
         <v>45793</v>
       </c>
       <c r="V15" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="X15" s="2"/>
       <c r="Y15" s="2"/>
@@ -2424,7 +2571,7 @@
         <v>2</v>
       </c>
       <c r="AD15" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:30" x14ac:dyDescent="0.2">
@@ -2460,36 +2607,36 @@
         <v>69</v>
       </c>
       <c r="M16" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N16" s="2">
         <v>45793</v>
       </c>
       <c r="O16" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P16" s="2">
         <v>45793</v>
       </c>
-      <c r="Q16" s="2">
+      <c r="Q16" s="10">
         <v>45785</v>
       </c>
-      <c r="R16" s="5">
+      <c r="R16" s="13">
         <v>0.48055555555555557</v>
       </c>
-      <c r="S16" t="s">
-        <v>226</v>
-      </c>
-      <c r="T16" t="s">
-        <v>227</v>
+      <c r="S16" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="T16" s="9" t="s">
+        <v>223</v>
       </c>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
       <c r="AC16" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="AD16" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:32" x14ac:dyDescent="0.2">
@@ -2525,36 +2672,36 @@
         <v>70</v>
       </c>
       <c r="M17" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N17" s="2">
         <v>45793</v>
       </c>
       <c r="O17" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P17" s="2">
         <v>45793</v>
       </c>
-      <c r="Q17" s="2">
+      <c r="Q17" s="10">
         <v>45785</v>
       </c>
-      <c r="R17" s="5">
+      <c r="R17" s="13">
         <v>0.49722222222222223</v>
       </c>
-      <c r="S17" t="s">
-        <v>228</v>
-      </c>
-      <c r="T17" t="s">
-        <v>229</v>
+      <c r="S17" s="11" t="s">
+        <v>300</v>
+      </c>
+      <c r="T17" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="X17" s="2"/>
       <c r="Y17" s="2"/>
       <c r="AC17" s="1" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="AD17" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="1:32" x14ac:dyDescent="0.2">
@@ -2590,39 +2737,39 @@
         <v>71</v>
       </c>
       <c r="M18" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N18" s="2">
         <v>45793</v>
       </c>
       <c r="O18" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P18" s="2">
         <v>45793</v>
       </c>
-      <c r="Q18" s="2">
+      <c r="Q18" s="10">
         <v>45785</v>
       </c>
-      <c r="R18" s="5">
+      <c r="R18" s="13">
         <v>0.51736111111111116</v>
       </c>
-      <c r="S18" t="s">
-        <v>224</v>
-      </c>
-      <c r="T18" t="s">
-        <v>225</v>
+      <c r="S18" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="T18" s="9" t="s">
+        <v>221</v>
       </c>
       <c r="V18" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
       <c r="AC18" s="1" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="AD18" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:32" x14ac:dyDescent="0.2">
@@ -2658,28 +2805,28 @@
         <v>72</v>
       </c>
       <c r="M19" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N19" s="2">
         <v>45793</v>
       </c>
       <c r="O19" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P19" s="2">
         <v>45793</v>
       </c>
-      <c r="Q19" t="s">
-        <v>150</v>
-      </c>
-      <c r="R19" s="5">
+      <c r="Q19" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="R19" s="13">
         <v>0.40625</v>
       </c>
-      <c r="S19" t="s">
-        <v>157</v>
-      </c>
-      <c r="T19" t="s">
-        <v>158</v>
+      <c r="S19" s="9" t="s">
+        <v>301</v>
+      </c>
+      <c r="T19" s="9" t="s">
+        <v>154</v>
       </c>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
@@ -2687,7 +2834,7 @@
         <v>113</v>
       </c>
       <c r="AD19" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:32" x14ac:dyDescent="0.2">
@@ -2723,28 +2870,28 @@
         <v>73</v>
       </c>
       <c r="M20" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N20" s="2">
         <v>45793</v>
       </c>
       <c r="O20" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P20" s="2">
         <v>45793</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="Q20" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="R20" s="5">
+      <c r="R20" s="13">
         <v>0.51597222222222228</v>
       </c>
-      <c r="S20" t="s">
+      <c r="S20" s="9" t="s">
+        <v>302</v>
+      </c>
+      <c r="T20" s="9" t="s">
         <v>138</v>
-      </c>
-      <c r="T20" t="s">
-        <v>139</v>
       </c>
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
@@ -2752,7 +2899,7 @@
         <v>131</v>
       </c>
       <c r="AD20" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:32" x14ac:dyDescent="0.2">
@@ -2788,28 +2935,28 @@
         <v>74</v>
       </c>
       <c r="M21" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N21" s="2">
         <v>45793</v>
       </c>
       <c r="O21" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P21" s="2">
         <v>45793</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="Q21" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="R21" s="5">
+      <c r="R21" s="13">
         <v>0.60972222222222228</v>
       </c>
-      <c r="S21" t="s">
-        <v>146</v>
-      </c>
-      <c r="T21" t="s">
-        <v>147</v>
+      <c r="S21" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="T21" s="9" t="s">
+        <v>145</v>
       </c>
       <c r="X21" s="2"/>
       <c r="Y21" s="2"/>
@@ -2817,7 +2964,7 @@
         <v>111</v>
       </c>
       <c r="AD21" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="22" spans="1:32" x14ac:dyDescent="0.2">
@@ -2853,28 +3000,28 @@
         <v>75</v>
       </c>
       <c r="M22" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N22" s="2">
         <v>45793</v>
       </c>
       <c r="O22" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P22" s="2">
         <v>45793</v>
       </c>
-      <c r="Q22" t="s">
-        <v>150</v>
-      </c>
-      <c r="R22" s="5">
+      <c r="Q22" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="R22" s="13">
         <v>0.45763888888888887</v>
       </c>
-      <c r="S22" t="s">
-        <v>153</v>
-      </c>
-      <c r="T22" t="s">
-        <v>154</v>
+      <c r="S22" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="T22" s="9" t="s">
+        <v>151</v>
       </c>
       <c r="X22" s="2"/>
       <c r="Y22" s="2"/>
@@ -2882,7 +3029,7 @@
         <v>112</v>
       </c>
       <c r="AD22" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" spans="1:32" x14ac:dyDescent="0.2">
@@ -2918,28 +3065,28 @@
         <v>76</v>
       </c>
       <c r="M23" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N23" s="2">
         <v>45793</v>
       </c>
       <c r="O23" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P23" s="2">
         <v>45793</v>
       </c>
-      <c r="Q23" t="s">
+      <c r="Q23" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="R23" s="13">
+        <v>0.42499999999999999</v>
+      </c>
+      <c r="S23" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="T23" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="R23" s="5">
-        <v>0.42499999999999999</v>
-      </c>
-      <c r="S23" t="s">
-        <v>151</v>
-      </c>
-      <c r="T23" t="s">
-        <v>152</v>
       </c>
       <c r="X23" s="2"/>
       <c r="Y23" s="2"/>
@@ -2977,28 +3124,28 @@
         <v>77</v>
       </c>
       <c r="M24" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N24" s="2">
         <v>45793</v>
       </c>
       <c r="O24" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P24" s="2">
         <v>45793</v>
       </c>
-      <c r="Q24" t="s">
+      <c r="Q24" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="R24" s="5">
+      <c r="R24" s="13">
         <v>0.56458333333333333</v>
       </c>
-      <c r="S24" t="s">
-        <v>142</v>
-      </c>
-      <c r="T24" t="s">
-        <v>143</v>
+      <c r="S24" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="T24" s="9" t="s">
+        <v>141</v>
       </c>
       <c r="X24" s="2"/>
       <c r="Y24" s="2"/>
@@ -3036,42 +3183,42 @@
         <v>78</v>
       </c>
       <c r="M25" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N25" s="2">
         <v>45793</v>
       </c>
       <c r="O25" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P25" s="2">
         <v>45793</v>
       </c>
-      <c r="Q25" t="s">
-        <v>187</v>
-      </c>
-      <c r="R25" s="5">
+      <c r="Q25" s="9" t="s">
+        <v>183</v>
+      </c>
+      <c r="R25" s="13">
         <v>0.66736111111111107</v>
       </c>
-      <c r="S25" t="s">
-        <v>188</v>
-      </c>
-      <c r="T25" t="s">
-        <v>189</v>
+      <c r="S25" s="9" t="s">
+        <v>184</v>
+      </c>
+      <c r="T25" s="11" t="s">
+        <v>185</v>
       </c>
       <c r="X25" s="2"/>
       <c r="Y25" s="2"/>
       <c r="AC25" t="s">
-        <v>275</v>
+        <v>268</v>
       </c>
       <c r="AD25" t="s">
-        <v>276</v>
+        <v>269</v>
       </c>
       <c r="AE25" t="s">
-        <v>277</v>
+        <v>270</v>
       </c>
       <c r="AF25" t="s">
-        <v>278</v>
+        <v>271</v>
       </c>
     </row>
     <row r="26" spans="1:32" x14ac:dyDescent="0.2">
@@ -3107,36 +3254,36 @@
         <v>79</v>
       </c>
       <c r="M26" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N26" s="2">
         <v>45793</v>
       </c>
       <c r="O26" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P26" s="2">
         <v>45793</v>
       </c>
-      <c r="Q26" t="s">
+      <c r="Q26" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="R26" s="5">
+      <c r="R26" s="13">
         <v>0.58750000000000002</v>
       </c>
-      <c r="S26" t="s">
-        <v>145</v>
-      </c>
-      <c r="T26" t="s">
-        <v>144</v>
+      <c r="S26" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="T26" s="9" t="s">
+        <v>142</v>
       </c>
       <c r="X26" s="2"/>
       <c r="Y26" s="2"/>
       <c r="AC26" t="s">
-        <v>279</v>
+        <v>272</v>
       </c>
       <c r="AD26" t="s">
-        <v>280</v>
+        <v>273</v>
       </c>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.2">
@@ -3165,7 +3312,7 @@
         <v>80</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J27" t="s">
         <v>28</v>
@@ -3174,42 +3321,42 @@
         <v>80</v>
       </c>
       <c r="M27" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N27" s="2">
         <v>45793</v>
       </c>
       <c r="O27" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P27" s="12">
         <v>45874</v>
       </c>
       <c r="Q27" s="11" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="R27" s="13">
         <v>0.4909722222222222</v>
       </c>
-      <c r="S27" s="9" t="s">
-        <v>148</v>
+      <c r="S27" s="11" t="s">
+        <v>146</v>
       </c>
       <c r="T27" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
       <c r="AC27" t="s">
-        <v>282</v>
+        <v>275</v>
       </c>
       <c r="AD27" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE27" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="AF27" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.2">
@@ -3238,7 +3385,7 @@
         <v>81</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J28" t="s">
         <v>54</v>
@@ -3247,45 +3394,45 @@
         <v>81</v>
       </c>
       <c r="M28" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N28" s="2">
         <v>45793</v>
       </c>
       <c r="O28" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P28" s="12">
         <v>45874</v>
       </c>
       <c r="Q28" s="11" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="R28" s="14">
         <v>0.68472222222222223</v>
       </c>
       <c r="S28" s="11" t="s">
-        <v>233</v>
+        <v>305</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="V28" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
       <c r="AC28" t="s">
-        <v>286</v>
+        <v>279</v>
       </c>
       <c r="AD28" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE28" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="AF28" t="s">
-        <v>287</v>
+        <v>280</v>
       </c>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.2">
@@ -3314,7 +3461,7 @@
         <v>82</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="J29" t="s">
         <v>29</v>
@@ -3323,42 +3470,42 @@
         <v>82</v>
       </c>
       <c r="M29" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N29" s="2">
         <v>45793</v>
       </c>
       <c r="O29" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P29" s="12">
         <v>45874</v>
       </c>
       <c r="Q29" s="11" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="R29" s="14">
         <v>0.63749999999999996</v>
       </c>
       <c r="S29" s="11" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="T29" s="11" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
       <c r="AC29" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
       <c r="AD29" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE29" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="AF29" t="s">
-        <v>289</v>
+        <v>282</v>
       </c>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.2">
@@ -3387,7 +3534,7 @@
         <v>83</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J30" t="s">
         <v>30</v>
@@ -3396,42 +3543,42 @@
         <v>83</v>
       </c>
       <c r="M30" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N30" s="2">
         <v>45793</v>
       </c>
       <c r="O30" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P30" s="12">
         <v>45874</v>
       </c>
       <c r="Q30" s="11" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="R30" s="14">
         <v>0.62222222222222223</v>
       </c>
       <c r="S30" s="11" t="s">
-        <v>237</v>
+        <v>306</v>
       </c>
       <c r="T30" s="11" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
       <c r="AC30" t="s">
-        <v>290</v>
+        <v>283</v>
       </c>
       <c r="AD30" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE30" t="s">
+        <v>277</v>
+      </c>
+      <c r="AF30" t="s">
         <v>284</v>
-      </c>
-      <c r="AF30" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.2">
@@ -3460,7 +3607,7 @@
         <v>84</v>
       </c>
       <c r="I31" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J31" t="s">
         <v>31</v>
@@ -3469,34 +3616,42 @@
         <v>84</v>
       </c>
       <c r="M31" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N31" s="2">
         <v>45793</v>
       </c>
       <c r="O31" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P31" s="12">
         <v>45874</v>
       </c>
-      <c r="Q31" s="9"/>
-      <c r="R31" s="9"/>
-      <c r="S31" s="9"/>
-      <c r="T31" s="9"/>
+      <c r="Q31" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="R31" s="14">
+        <v>0.56458333333333333</v>
+      </c>
+      <c r="S31" s="11" t="s">
+        <v>308</v>
+      </c>
+      <c r="T31" s="11" t="s">
+        <v>309</v>
+      </c>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
       <c r="AC31" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="AD31" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE31" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="AF31" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.2">
@@ -3525,7 +3680,7 @@
         <v>85</v>
       </c>
       <c r="I32" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J32" t="s">
         <v>32</v>
@@ -3534,42 +3689,42 @@
         <v>85</v>
       </c>
       <c r="M32" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N32" s="2">
         <v>45793</v>
       </c>
       <c r="O32" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P32" s="12">
         <v>45874</v>
       </c>
       <c r="Q32" s="11" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="R32" s="14">
         <v>0.66041666666666665</v>
       </c>
       <c r="S32" s="11" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="T32" s="11" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
       <c r="AC32" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="AD32" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE32" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="AF32" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.2">
@@ -3598,7 +3753,7 @@
         <v>86</v>
       </c>
       <c r="I33" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J33" t="s">
         <v>33</v>
@@ -3607,27 +3762,39 @@
         <v>86</v>
       </c>
       <c r="M33" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N33" s="2">
         <v>45793</v>
       </c>
       <c r="O33" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P33" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q33" s="10">
+        <v>45940</v>
+      </c>
+      <c r="R33" s="14">
+        <v>0.56597222222222221</v>
+      </c>
+      <c r="S33" s="11" t="s">
+        <v>310</v>
+      </c>
+      <c r="T33" s="11" t="s">
+        <v>311</v>
       </c>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
       <c r="AC33" t="s">
-        <v>306</v>
+        <v>299</v>
       </c>
       <c r="AD33" t="s">
-        <v>283</v>
+        <v>276</v>
       </c>
       <c r="AE33" t="s">
-        <v>281</v>
+        <v>274</v>
       </c>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.2">
@@ -3656,7 +3823,7 @@
         <v>87</v>
       </c>
       <c r="I34" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J34" t="s">
         <v>53</v>
@@ -3665,16 +3832,28 @@
         <v>87</v>
       </c>
       <c r="M34" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N34" s="2">
         <v>45793</v>
       </c>
       <c r="O34" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P34" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q34" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R34" s="14">
+        <v>0.4861111111111111</v>
+      </c>
+      <c r="S34" s="11" t="s">
+        <v>313</v>
+      </c>
+      <c r="T34" s="11" t="s">
+        <v>314</v>
       </c>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
@@ -3705,7 +3884,7 @@
         <v>88</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J35" t="s">
         <v>52</v>
@@ -3714,16 +3893,28 @@
         <v>88</v>
       </c>
       <c r="M35" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N35" s="2">
         <v>45793</v>
       </c>
       <c r="O35" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P35" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q35" s="10">
+        <v>45940</v>
+      </c>
+      <c r="R35" s="14">
+        <v>0.51458333333333328</v>
+      </c>
+      <c r="S35" s="11" t="s">
+        <v>315</v>
+      </c>
+      <c r="T35" s="11" t="s">
+        <v>316</v>
       </c>
       <c r="X35" s="2"/>
       <c r="Y35" s="2"/>
@@ -3754,7 +3945,7 @@
         <v>89</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J36" t="s">
         <v>34</v>
@@ -3763,16 +3954,28 @@
         <v>89</v>
       </c>
       <c r="M36" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N36" s="2">
         <v>45793</v>
       </c>
       <c r="O36" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P36" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q36" s="10">
+        <v>45940</v>
+      </c>
+      <c r="R36" s="14">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="S36" s="11" t="s">
+        <v>317</v>
+      </c>
+      <c r="T36" s="11" t="s">
+        <v>318</v>
       </c>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
@@ -3803,7 +4006,7 @@
         <v>90</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J37" t="s">
         <v>35</v>
@@ -3812,16 +4015,28 @@
         <v>90</v>
       </c>
       <c r="M37" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N37" s="2">
         <v>45793</v>
       </c>
       <c r="O37" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P37" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q37" s="10">
+        <v>45940</v>
+      </c>
+      <c r="R37" s="14">
+        <v>0.46805555555555556</v>
+      </c>
+      <c r="S37" s="11" t="s">
+        <v>319</v>
+      </c>
+      <c r="T37" s="11" t="s">
+        <v>320</v>
       </c>
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
@@ -3852,7 +4067,7 @@
         <v>91</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="J38" t="s">
         <v>36</v>
@@ -3861,19 +4076,31 @@
         <v>91</v>
       </c>
       <c r="M38" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N38" s="2">
         <v>45793</v>
       </c>
       <c r="O38" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P38" s="12">
         <v>45874</v>
       </c>
+      <c r="Q38" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="R38" s="14">
+        <v>0.47708333333333336</v>
+      </c>
+      <c r="S38" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="T38" s="11" t="s">
+        <v>322</v>
+      </c>
       <c r="V38" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="X38" s="2"/>
       <c r="Y38" s="2"/>
@@ -3911,16 +4138,28 @@
         <v>92</v>
       </c>
       <c r="M39" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N39" s="2">
         <v>45793</v>
       </c>
       <c r="O39" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P39" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q39" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="R39" s="14">
+        <v>0.69652777777777775</v>
+      </c>
+      <c r="S39" s="11" t="s">
+        <v>324</v>
+      </c>
+      <c r="T39" s="11" t="s">
+        <v>325</v>
       </c>
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
@@ -3958,16 +4197,28 @@
         <v>93</v>
       </c>
       <c r="M40" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N40" s="2">
         <v>45793</v>
       </c>
       <c r="O40" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P40" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q40" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="R40" s="14">
+        <v>0.65486111111111112</v>
+      </c>
+      <c r="S40" s="11" t="s">
+        <v>326</v>
+      </c>
+      <c r="T40" s="11" t="s">
+        <v>327</v>
       </c>
       <c r="X40" s="2"/>
       <c r="Y40" s="2"/>
@@ -4005,19 +4256,31 @@
         <v>94</v>
       </c>
       <c r="M41" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N41" s="2">
         <v>45793</v>
       </c>
       <c r="O41" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P41" s="12">
         <v>45874</v>
       </c>
+      <c r="Q41" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="R41" s="14">
+        <v>0.64097222222222228</v>
+      </c>
+      <c r="S41" s="11" t="s">
+        <v>328</v>
+      </c>
+      <c r="T41" s="11" t="s">
+        <v>329</v>
+      </c>
       <c r="V41" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="X41" s="2"/>
       <c r="Y41" s="2"/>
@@ -4055,19 +4318,31 @@
         <v>95</v>
       </c>
       <c r="M42" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N42" s="2">
         <v>45793</v>
       </c>
       <c r="O42" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P42" s="12">
         <v>45874</v>
       </c>
+      <c r="Q42" s="10">
+        <v>45910</v>
+      </c>
+      <c r="R42" s="14">
+        <v>0.46111111111111114</v>
+      </c>
+      <c r="S42" s="11" t="s">
+        <v>330</v>
+      </c>
+      <c r="T42" s="11" t="s">
+        <v>331</v>
+      </c>
       <c r="V42" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="X42" s="2"/>
       <c r="Y42" s="2"/>
@@ -4105,19 +4380,23 @@
         <v>96</v>
       </c>
       <c r="M43" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N43" s="2">
         <v>45793</v>
       </c>
       <c r="O43" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P43" s="12">
         <v>45874</v>
       </c>
+      <c r="Q43" s="9"/>
+      <c r="R43" s="9"/>
+      <c r="S43" s="9"/>
+      <c r="T43" s="9"/>
       <c r="V43" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
@@ -4155,19 +4434,31 @@
         <v>97</v>
       </c>
       <c r="M44" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N44" s="2">
         <v>45793</v>
       </c>
       <c r="O44" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P44" s="12">
         <v>45874</v>
       </c>
+      <c r="Q44" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R44" s="14">
+        <v>0.50555555555555554</v>
+      </c>
+      <c r="S44" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="T44" s="11" t="s">
+        <v>333</v>
+      </c>
       <c r="V44" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="X44" s="2"/>
       <c r="Y44" s="2"/>
@@ -4205,16 +4496,28 @@
         <v>98</v>
       </c>
       <c r="M45" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N45" s="2">
         <v>45793</v>
       </c>
       <c r="O45" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P45" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q45" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R45" s="14">
+        <v>0.53888888888888886</v>
+      </c>
+      <c r="S45" s="11" t="s">
+        <v>334</v>
+      </c>
+      <c r="T45" s="11" t="s">
+        <v>335</v>
       </c>
       <c r="X45" s="2"/>
       <c r="Y45" s="2"/>
@@ -4252,16 +4555,28 @@
         <v>99</v>
       </c>
       <c r="M46" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N46" s="2">
         <v>45793</v>
       </c>
       <c r="O46" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P46" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q46" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="R46" s="14">
+        <v>0.5131944444444444</v>
+      </c>
+      <c r="S46" s="11" t="s">
+        <v>337</v>
+      </c>
+      <c r="T46" s="11" t="s">
+        <v>338</v>
       </c>
       <c r="X46" s="2"/>
       <c r="Y46" s="2"/>
@@ -4299,16 +4614,28 @@
         <v>100</v>
       </c>
       <c r="M47" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N47" s="2">
         <v>45793</v>
       </c>
       <c r="O47" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P47" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q47" s="11" t="s">
+        <v>323</v>
+      </c>
+      <c r="R47" s="14">
+        <v>0.625</v>
+      </c>
+      <c r="S47" s="11" t="s">
+        <v>339</v>
+      </c>
+      <c r="T47" s="11" t="s">
+        <v>340</v>
       </c>
       <c r="X47" s="2"/>
       <c r="Y47" s="2"/>
@@ -4346,16 +4673,28 @@
         <v>101</v>
       </c>
       <c r="M48" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N48" s="2">
         <v>45793</v>
       </c>
       <c r="O48" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P48" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q48" s="10">
+        <v>45940</v>
+      </c>
+      <c r="R48" s="14">
+        <v>0.53819444444444442</v>
+      </c>
+      <c r="S48" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="T48" s="11" t="s">
+        <v>342</v>
       </c>
       <c r="X48" s="2"/>
       <c r="Y48" s="2"/>
@@ -4393,16 +4732,28 @@
         <v>102</v>
       </c>
       <c r="M49" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N49" s="2">
         <v>45793</v>
       </c>
       <c r="O49" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P49" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q49" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R49" s="14">
+        <v>0.47222222222222221</v>
+      </c>
+      <c r="S49" s="11" t="s">
+        <v>343</v>
+      </c>
+      <c r="T49" s="11" t="s">
+        <v>344</v>
       </c>
       <c r="X49" s="2"/>
       <c r="Y49" s="2"/>
@@ -4440,16 +4791,28 @@
         <v>103</v>
       </c>
       <c r="M50" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N50" s="2">
         <v>45793</v>
       </c>
       <c r="O50" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P50" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q50" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R50" s="14">
+        <v>0.52430555555555558</v>
+      </c>
+      <c r="S50" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="T50" s="11" t="s">
+        <v>345</v>
       </c>
       <c r="X50" s="2"/>
       <c r="Y50" s="2"/>
@@ -4487,19 +4850,31 @@
         <v>104</v>
       </c>
       <c r="M51" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N51" s="2">
         <v>45793</v>
       </c>
       <c r="O51" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P51" s="12">
         <v>45874</v>
       </c>
+      <c r="Q51" s="11" t="s">
+        <v>307</v>
+      </c>
+      <c r="R51" s="14">
+        <v>0.625</v>
+      </c>
+      <c r="S51" s="11" t="s">
+        <v>346</v>
+      </c>
+      <c r="T51" s="11" t="s">
+        <v>347</v>
+      </c>
       <c r="V51" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="X51" s="2"/>
       <c r="Y51" s="2"/>
@@ -4537,16 +4912,28 @@
         <v>105</v>
       </c>
       <c r="M52" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N52" s="2">
         <v>45793</v>
       </c>
       <c r="O52" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P52" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q52" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R52" s="14">
+        <v>0.44305555555555554</v>
+      </c>
+      <c r="S52" s="11" t="s">
+        <v>348</v>
+      </c>
+      <c r="T52" s="11" t="s">
+        <v>349</v>
       </c>
       <c r="X52" s="2"/>
       <c r="Y52" s="2"/>
@@ -4584,16 +4971,28 @@
         <v>106</v>
       </c>
       <c r="M53" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="N53" s="2">
         <v>45793</v>
       </c>
       <c r="O53" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P53" s="12">
         <v>45874</v>
+      </c>
+      <c r="Q53" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="R53" s="14">
+        <v>0.48958333333333331</v>
+      </c>
+      <c r="S53" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="T53" s="11" t="s">
+        <v>351</v>
       </c>
       <c r="X53" s="2"/>
       <c r="Y53" s="2"/>
@@ -4625,25 +5024,37 @@
       </c>
       <c r="I54" s="4"/>
       <c r="J54" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="K54" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="L54" s="4" t="s">
         <v>107</v>
       </c>
       <c r="M54" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="N54" s="2">
         <v>45794</v>
       </c>
       <c r="O54" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P54" s="12">
         <v>45875</v>
+      </c>
+      <c r="Q54" s="11" t="s">
+        <v>336</v>
+      </c>
+      <c r="R54" s="14">
+        <v>0.46666666666666667</v>
+      </c>
+      <c r="S54" s="11" t="s">
+        <v>352</v>
+      </c>
+      <c r="T54" s="11" t="s">
+        <v>353</v>
       </c>
       <c r="X54" s="2"/>
       <c r="Y54" s="2"/>
@@ -4675,25 +5086,37 @@
       </c>
       <c r="I55" s="4"/>
       <c r="J55" t="s">
-        <v>251</v>
+        <v>244</v>
       </c>
       <c r="K55" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="L55" s="4" t="s">
         <v>108</v>
       </c>
       <c r="M55" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="N55" s="2">
         <v>45795</v>
       </c>
       <c r="O55" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P55" s="12">
         <v>45876</v>
+      </c>
+      <c r="Q55" s="10">
+        <v>45849</v>
+      </c>
+      <c r="R55" s="14">
+        <v>0.53194444444444444</v>
+      </c>
+      <c r="S55" s="9" t="s">
+        <v>304</v>
+      </c>
+      <c r="T55" s="9" t="s">
+        <v>141</v>
       </c>
       <c r="X55" s="2"/>
       <c r="Y55" s="2"/>
@@ -4725,25 +5148,37 @@
       </c>
       <c r="I56" s="4"/>
       <c r="J56" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="K56" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="L56" s="4" t="s">
         <v>109</v>
       </c>
       <c r="M56" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="N56" s="2">
         <v>45796</v>
       </c>
       <c r="O56" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="P56" s="12">
         <v>45877</v>
+      </c>
+      <c r="Q56" s="11" t="s">
+        <v>312</v>
+      </c>
+      <c r="R56" s="14">
+        <v>0.46180555555555558</v>
+      </c>
+      <c r="S56" s="11" t="s">
+        <v>354</v>
+      </c>
+      <c r="T56" s="11" t="s">
+        <v>355</v>
       </c>
       <c r="X56" s="2"/>
       <c r="Y56" s="2"/>
@@ -4804,61 +5239,61 @@
         <v>45998</v>
       </c>
       <c r="M1" s="11" t="s">
+        <v>189</v>
+      </c>
+      <c r="N1" s="11" t="s">
+        <v>190</v>
+      </c>
+      <c r="O1" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="P1" s="11" t="s">
+        <v>192</v>
+      </c>
+      <c r="Q1" s="11" t="s">
         <v>193</v>
       </c>
-      <c r="N1" s="11" t="s">
+      <c r="R1" s="11" t="s">
         <v>194</v>
       </c>
-      <c r="O1" s="11" t="s">
+      <c r="S1" s="11" t="s">
         <v>195</v>
       </c>
-      <c r="P1" s="11" t="s">
+      <c r="T1" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="Q1" s="11" t="s">
+      <c r="U1" s="11" t="s">
         <v>197</v>
       </c>
-      <c r="R1" s="11" t="s">
+      <c r="V1" s="11" t="s">
         <v>198</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="W1" s="11" t="s">
         <v>199</v>
       </c>
-      <c r="T1" s="11" t="s">
+      <c r="X1" s="11" t="s">
         <v>200</v>
       </c>
-      <c r="U1" s="11" t="s">
+      <c r="Y1" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="V1" s="11" t="s">
+      <c r="Z1" s="11" t="s">
         <v>202</v>
       </c>
-      <c r="W1" s="11" t="s">
+      <c r="AA1" s="11" t="s">
         <v>203</v>
       </c>
-      <c r="X1" s="11" t="s">
+      <c r="AB1" s="11" t="s">
         <v>204</v>
       </c>
-      <c r="Y1" s="11" t="s">
+      <c r="AC1" s="11" t="s">
         <v>205</v>
       </c>
-      <c r="Z1" s="11" t="s">
+      <c r="AD1" s="11" t="s">
         <v>206</v>
       </c>
-      <c r="AA1" s="11" t="s">
+      <c r="AE1" s="11" t="s">
         <v>207</v>
-      </c>
-      <c r="AB1" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="AC1" s="11" t="s">
-        <v>209</v>
-      </c>
-      <c r="AD1" s="11" t="s">
-        <v>210</v>
-      </c>
-      <c r="AE1" s="11" t="s">
-        <v>211</v>
       </c>
       <c r="AF1" s="10">
         <v>45665</v>
@@ -4912,49 +5347,49 @@
         <v>45885</v>
       </c>
       <c r="AW1" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="AX1" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="AY1" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="AZ1" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="BA1" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="BB1" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="BC1" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="BD1" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="BE1" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="AX1" s="15" t="s">
+      <c r="BF1" s="15" t="s">
         <v>254</v>
       </c>
-      <c r="AY1" s="15" t="s">
+      <c r="BG1" s="15" t="s">
         <v>255</v>
       </c>
-      <c r="AZ1" s="15" t="s">
+      <c r="BH1" s="15" t="s">
         <v>256</v>
       </c>
-      <c r="BA1" s="15" t="s">
+      <c r="BI1" s="15" t="s">
         <v>257</v>
       </c>
-      <c r="BB1" s="15" t="s">
+      <c r="BJ1" s="15" t="s">
         <v>258</v>
       </c>
-      <c r="BC1" s="15" t="s">
-        <v>274</v>
-      </c>
-      <c r="BD1" s="15" t="s">
+      <c r="BK1" s="15" t="s">
         <v>259</v>
-      </c>
-      <c r="BE1" s="15" t="s">
-        <v>260</v>
-      </c>
-      <c r="BF1" s="15" t="s">
-        <v>261</v>
-      </c>
-      <c r="BG1" s="15" t="s">
-        <v>262</v>
-      </c>
-      <c r="BH1" s="15" t="s">
-        <v>263</v>
-      </c>
-      <c r="BI1" s="15" t="s">
-        <v>264</v>
-      </c>
-      <c r="BJ1" s="15" t="s">
-        <v>265</v>
-      </c>
-      <c r="BK1" s="15" t="s">
-        <v>266</v>
       </c>
       <c r="BL1" s="15">
         <v>45901</v>
@@ -4993,25 +5428,25 @@
         <v>45912</v>
       </c>
       <c r="BX1" s="15" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="BY1" s="15" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="BZ1" s="15" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="CA1" s="15" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="CB1" s="15" t="s">
-        <v>271</v>
+        <v>264</v>
       </c>
       <c r="CC1" s="15" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="CD1" s="15" t="s">
-        <v>273</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" spans="1:82" x14ac:dyDescent="0.2">
@@ -7100,7 +7535,7 @@
         <v>85</v>
       </c>
       <c r="F32" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="BG32" s="17"/>
       <c r="BH32" s="17"/>
@@ -7133,10 +7568,10 @@
       </c>
       <c r="F33" s="6"/>
       <c r="G33" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="I33" s="11" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
@@ -7145,10 +7580,10 @@
       </c>
       <c r="F34" s="7"/>
       <c r="G34" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="I34" s="11" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
@@ -7156,7 +7591,7 @@
         <v>88</v>
       </c>
       <c r="I35" s="11" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Updated the particle account passwords on the sensor box component tracker sheet
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kriishhate/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81460AC7-1BD6-1448-B004-356C414A2C2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAE80837-BA4F-8149-97DF-1CE399A1BAF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
   <sheets>
     <sheet name="Deployment Tracker " sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="355">
   <si>
     <t>Box Number</t>
   </si>
@@ -858,18 +858,12 @@
     <t>envsensorslab@gmail.com</t>
   </si>
   <si>
-    <t>Envlab257</t>
-  </si>
-  <si>
     <t>500 MB</t>
   </si>
   <si>
     <t>COMMONSENSES1@LISTSERV.NEU.EDU</t>
   </si>
   <si>
-    <t>Envsensorslab257</t>
-  </si>
-  <si>
     <t>100 MB</t>
   </si>
   <si>
@@ -1105,6 +1099,9 @@
   </si>
   <si>
     <t>42.31298, -71.07653</t>
+  </si>
+  <si>
+    <t>EnvsensorsLab257</t>
   </si>
 </sst>
 </file>
@@ -2695,7 +2692,7 @@
         <v>0.49722222222222223</v>
       </c>
       <c r="S17" s="11" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="T17" s="9" t="s">
         <v>224</v>
@@ -2828,7 +2825,7 @@
         <v>0.40625</v>
       </c>
       <c r="S19" s="9" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="T19" s="9" t="s">
         <v>154</v>
@@ -2893,7 +2890,7 @@
         <v>0.51597222222222228</v>
       </c>
       <c r="S20" s="9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="T20" s="9" t="s">
         <v>138</v>
@@ -3023,7 +3020,7 @@
         <v>0.45763888888888887</v>
       </c>
       <c r="S22" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="T22" s="9" t="s">
         <v>151</v>
@@ -3149,7 +3146,7 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="S24" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="T24" s="9" t="s">
         <v>141</v>
@@ -3290,7 +3287,7 @@
         <v>272</v>
       </c>
       <c r="AD26" t="s">
-        <v>273</v>
+        <v>354</v>
       </c>
     </row>
     <row r="27" spans="1:32" x14ac:dyDescent="0.2">
@@ -3354,16 +3351,16 @@
       <c r="X27" s="2"/>
       <c r="Y27" s="2"/>
       <c r="AC27" t="s">
+        <v>274</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>354</v>
+      </c>
+      <c r="AE27" t="s">
         <v>275</v>
       </c>
-      <c r="AD27" t="s">
+      <c r="AF27" t="s">
         <v>276</v>
-      </c>
-      <c r="AE27" t="s">
-        <v>277</v>
-      </c>
-      <c r="AF27" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="28" spans="1:32" x14ac:dyDescent="0.2">
@@ -3419,7 +3416,7 @@
         <v>0.68472222222222223</v>
       </c>
       <c r="S28" s="11" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="T28" s="11" t="s">
         <v>228</v>
@@ -3430,16 +3427,16 @@
       <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
       <c r="AC28" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="AD28" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE28" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AF28" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" spans="1:32" x14ac:dyDescent="0.2">
@@ -3503,16 +3500,16 @@
       <c r="X29" s="2"/>
       <c r="Y29" s="2"/>
       <c r="AC29" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="AD29" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE29" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AF29" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" spans="1:32" x14ac:dyDescent="0.2">
@@ -3568,7 +3565,7 @@
         <v>0.62222222222222223</v>
       </c>
       <c r="S30" s="11" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="T30" s="11" t="s">
         <v>231</v>
@@ -3576,16 +3573,16 @@
       <c r="X30" s="2"/>
       <c r="Y30" s="2"/>
       <c r="AC30" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="AD30" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE30" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AF30" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="31" spans="1:32" x14ac:dyDescent="0.2">
@@ -3639,24 +3636,24 @@
         <v>0.56458333333333333</v>
       </c>
       <c r="S31" s="11" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="T31" s="11" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="X31" s="2"/>
       <c r="Y31" s="2"/>
       <c r="AC31" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="AD31" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE31" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AF31" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
     </row>
     <row r="32" spans="1:32" x14ac:dyDescent="0.2">
@@ -3720,16 +3717,16 @@
       <c r="X32" s="2"/>
       <c r="Y32" s="2"/>
       <c r="AC32" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="AD32" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE32" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="AF32" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
     </row>
     <row r="33" spans="1:31" x14ac:dyDescent="0.2">
@@ -3782,21 +3779,21 @@
         <v>0.56597222222222221</v>
       </c>
       <c r="S33" s="11" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="T33" s="11" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="X33" s="2"/>
       <c r="Y33" s="2"/>
       <c r="AC33" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="AD33" t="s">
-        <v>276</v>
+        <v>354</v>
       </c>
       <c r="AE33" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="34" spans="1:31" x14ac:dyDescent="0.2">
@@ -3849,10 +3846,10 @@
         <v>0.4861111111111111</v>
       </c>
       <c r="S34" s="11" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="T34" s="11" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="X34" s="2"/>
       <c r="Y34" s="2"/>
@@ -3907,10 +3904,10 @@
         <v>0.51458333333333328</v>
       </c>
       <c r="S35" s="11" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="T35" s="11" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="X35" s="2"/>
       <c r="Y35" s="2"/>
@@ -3965,10 +3962,10 @@
         <v>0.49652777777777779</v>
       </c>
       <c r="S36" s="11" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="T36" s="11" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="X36" s="2"/>
       <c r="Y36" s="2"/>
@@ -4023,10 +4020,10 @@
         <v>0.46805555555555556</v>
       </c>
       <c r="S37" s="11" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="T37" s="11" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="X37" s="2"/>
       <c r="Y37" s="2"/>
@@ -4081,13 +4078,13 @@
         <v>0.47708333333333336</v>
       </c>
       <c r="S38" s="11" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="V38" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="X38" s="2"/>
       <c r="Y38" s="2"/>
@@ -4140,10 +4137,10 @@
         <v>0.69652777777777775</v>
       </c>
       <c r="S39" s="11" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="T39" s="11" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="X39" s="2"/>
       <c r="Y39" s="2"/>
@@ -4196,10 +4193,10 @@
         <v>0.65486111111111112</v>
       </c>
       <c r="S40" s="11" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="T40" s="11" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="X40" s="2"/>
       <c r="Y40" s="2"/>
@@ -4252,10 +4249,10 @@
         <v>0.64097222222222228</v>
       </c>
       <c r="S41" s="11" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="V41" t="s">
         <v>234</v>
@@ -4311,10 +4308,10 @@
         <v>0.46111111111111114</v>
       </c>
       <c r="S42" s="11" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="T42" s="11" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="V42" t="s">
         <v>235</v>
@@ -4375,7 +4372,7 @@
       <c r="S43" s="9"/>
       <c r="T43" s="9"/>
       <c r="V43" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="X43" s="2"/>
       <c r="Y43" s="2"/>
@@ -4425,19 +4422,19 @@
         <v>45874</v>
       </c>
       <c r="Q44" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R44" s="14">
         <v>0.50555555555555554</v>
       </c>
       <c r="S44" s="11" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="V44" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="X44" s="2"/>
       <c r="Y44" s="2"/>
@@ -4487,16 +4484,16 @@
         <v>45874</v>
       </c>
       <c r="Q45" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R45" s="14">
         <v>0.53888888888888886</v>
       </c>
       <c r="S45" s="11" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="T45" s="11" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="X45" s="2"/>
       <c r="Y45" s="2"/>
@@ -4546,16 +4543,16 @@
         <v>45874</v>
       </c>
       <c r="Q46" s="11" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="R46" s="14">
         <v>0.5131944444444444</v>
       </c>
       <c r="S46" s="11" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="T46" s="11" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="X46" s="2"/>
       <c r="Y46" s="2"/>
@@ -4605,16 +4602,16 @@
         <v>45874</v>
       </c>
       <c r="Q47" s="11" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="R47" s="14">
         <v>0.625</v>
       </c>
       <c r="S47" s="11" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="T47" s="11" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="X47" s="2"/>
       <c r="Y47" s="2"/>
@@ -4670,10 +4667,10 @@
         <v>0.53819444444444442</v>
       </c>
       <c r="S48" s="11" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="T48" s="11" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="X48" s="2"/>
       <c r="Y48" s="2"/>
@@ -4723,16 +4720,16 @@
         <v>45874</v>
       </c>
       <c r="Q49" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R49" s="14">
         <v>0.47222222222222221</v>
       </c>
       <c r="S49" s="11" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="T49" s="11" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="X49" s="2"/>
       <c r="Y49" s="2"/>
@@ -4782,7 +4779,7 @@
         <v>45874</v>
       </c>
       <c r="Q50" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R50" s="14">
         <v>0.52430555555555558</v>
@@ -4791,7 +4788,7 @@
         <v>232</v>
       </c>
       <c r="T50" s="11" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="X50" s="2"/>
       <c r="Y50" s="2"/>
@@ -4841,16 +4838,16 @@
         <v>45874</v>
       </c>
       <c r="Q51" s="11" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="R51" s="14">
         <v>0.625</v>
       </c>
       <c r="S51" s="11" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="T51" s="11" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="V51" t="s">
         <v>234</v>
@@ -4903,16 +4900,16 @@
         <v>45874</v>
       </c>
       <c r="Q52" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R52" s="14">
         <v>0.44305555555555554</v>
       </c>
       <c r="S52" s="11" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="T52" s="11" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="X52" s="2"/>
       <c r="Y52" s="2"/>
@@ -4962,16 +4959,16 @@
         <v>45874</v>
       </c>
       <c r="Q53" s="11" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="R53" s="14">
         <v>0.48958333333333331</v>
       </c>
       <c r="S53" s="11" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="T53" s="11" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="X53" s="2"/>
       <c r="Y53" s="2"/>
@@ -5003,16 +5000,16 @@
       </c>
       <c r="I54" s="4"/>
       <c r="J54" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="K54" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="L54" s="4" t="s">
         <v>107</v>
       </c>
       <c r="M54" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="N54" s="2">
         <v>45794</v>
@@ -5024,16 +5021,16 @@
         <v>45875</v>
       </c>
       <c r="Q54" s="11" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="R54" s="14">
         <v>0.46666666666666667</v>
       </c>
       <c r="S54" s="11" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="T54" s="11" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="X54" s="2"/>
       <c r="Y54" s="2"/>
@@ -5074,7 +5071,7 @@
         <v>108</v>
       </c>
       <c r="M55" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="N55" s="2">
         <v>45795</v>
@@ -5092,7 +5089,7 @@
         <v>0.53194444444444444</v>
       </c>
       <c r="S55" s="9" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="T55" s="9" t="s">
         <v>141</v>
@@ -5127,16 +5124,16 @@
       </c>
       <c r="I56" s="4"/>
       <c r="J56" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="K56" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="L56" s="4" t="s">
         <v>109</v>
       </c>
       <c r="M56" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="N56" s="2">
         <v>45796</v>
@@ -5148,16 +5145,16 @@
         <v>45877</v>
       </c>
       <c r="Q56" s="11" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="R56" s="14">
         <v>0.46180555555555558</v>
       </c>
       <c r="S56" s="11" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="T56" s="11" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="X56" s="2"/>
       <c r="Y56" s="2"/>

</xml_diff>

<commit_message>
updated on maintenance of box 08,39,40
</commit_message>
<xml_diff>
--- a/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
+++ b/Sensor Box Deployment Inventory /Deployment Invetory Excel File/SensorBox_Component_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/allensong/Documents/GitHub/CommonSENSES/Sensor Box Deployment Inventory /Deployment Invetory Excel File/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBBDA35D-B916-7D46-9D55-D3B354656203}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1836600-1D66-ED4B-8773-D2D29A3DAC9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="18960" xr2:uid="{9F8D9832-C5EF-1142-B4F9-7517213DD771}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1029" uniqueCount="357">
   <si>
     <t>Box Number</t>
   </si>
@@ -1105,6 +1105,9 @@
   </si>
   <si>
     <t>RTC OK 2026-03-27</t>
+  </si>
+  <si>
+    <t>RTC OK 2026-03-27. Files:08250613.txt corrupted, `pdj also corrupted seen on 20260327.</t>
   </si>
 </sst>
 </file>
@@ -2179,7 +2182,7 @@
         <v>130</v>
       </c>
       <c r="V9" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="X9" s="2"/>
       <c r="Y9" s="2"/>

</xml_diff>